<commit_message>
Atualização automática: 2026-09-14 13:29
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7928" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7930" uniqueCount="381">
   <si>
     <t>CodCliente</t>
   </si>
@@ -30410,6 +30410,9 @@
       <c r="O434">
         <v>18273589</v>
       </c>
+      <c r="P434" t="s">
+        <v>205</v>
+      </c>
       <c r="Q434" t="s">
         <v>223</v>
       </c>
@@ -30424,6 +30427,9 @@
       </c>
       <c r="AF434" t="s">
         <v>372</v>
+      </c>
+      <c r="AG434" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="435" spans="1:33">

</xml_diff>

<commit_message>
Atualização automática: 2026-09-15 13:19
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8411" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8415" uniqueCount="420">
   <si>
     <t>CodCliente</t>
   </si>
@@ -40873,6 +40873,9 @@
       <c r="O589">
         <v>18274360</v>
       </c>
+      <c r="P589" t="s">
+        <v>234</v>
+      </c>
       <c r="Q589" t="s">
         <v>242</v>
       </c>
@@ -40926,6 +40929,9 @@
       <c r="O590">
         <v>18274348</v>
       </c>
+      <c r="P590" t="s">
+        <v>234</v>
+      </c>
       <c r="Q590" t="s">
         <v>242</v>
       </c>
@@ -41351,6 +41357,9 @@
       <c r="O597">
         <v>18274368</v>
       </c>
+      <c r="P597" t="s">
+        <v>235</v>
+      </c>
       <c r="Q597" t="s">
         <v>242</v>
       </c>
@@ -41403,6 +41412,9 @@
       </c>
       <c r="O598">
         <v>18274352</v>
+      </c>
+      <c r="P598" t="s">
+        <v>235</v>
       </c>
       <c r="Q598" t="s">
         <v>242</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-17 17:58
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1293,8 +1293,7 @@
 Falha na emissão do arquivo para baixa - Data Comentário: 17/09/2026 16:45</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 17/09/2026 
-Fechamento em andamento - Data Comentário: 15/09/2026 17:34</t>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 18/09/2026 - Data Comentário: 17/09/2026 17:50</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 17/09/2026 - Data Comentário: 16/09/2026 18:49</t>
@@ -41728,7 +41727,7 @@
         <v>46280</v>
       </c>
       <c r="M582" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="N582" t="s">
         <v>214</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-21 14:00
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1174,7 +1174,9 @@
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 22/09/2026 - Data Comentário: 18/09/2026 15:24</t>
   </si>
   <si>
-    <t>Reaberto via API integração MGC x Sistema de Analise Fiscal em 21/09/2026 12:44:23. - Data Comentário: 21/09/2026 12:41</t>
+    <t>Integração com Sistema de Análise 
+Nenhum comentário informado pelo GC 
+Data Simulação: 21/09/2026 12:44:24 - Data Comentário: 21/09/2026 13:15</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 24/09/2026 - Data Comentário: 18/09/2026 15:24</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-22 13:49
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8980" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8981" uniqueCount="480">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1142,7 +1142,7 @@
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 28/09/2026 - Data Comentário: 18/09/2026 15:27</t>
   </si>
   <si>
-    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1807] sendo a ultima baixa feita [1807]-22/09/2026 10:05:26.. - Data Comentário: 22/09/2026 10:00</t>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1807] sendo a ultima baixa feita [1807]-22/09/2026 10:05:26.. - Data Comentário: 22/09/2026 12:56</t>
   </si>
   <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1882] sendo a ultima baixa feita [1882]-18/09/2026 18:05:29.. - Data Comentário: 21/09/2026 09:20</t>
@@ -26634,6 +26634,9 @@
       <c r="L355" s="1">
         <v>46290</v>
       </c>
+      <c r="M355" t="s">
+        <v>210</v>
+      </c>
       <c r="N355" t="s">
         <v>218</v>
       </c>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-22 15:50
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8980" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8977" uniqueCount="480">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1136,7 +1136,7 @@
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 22/09/2026 - Data Comentário: 18/09/2026 15:24</t>
   </si>
   <si>
-    <t>Reaberto via API integração MGC x Sistema de Analise Fiscal em 22/09/2026 14:36:22. - Data Comentário: 22/09/2026 14:35</t>
+    <t>Reaberto via API integração MGC x Sistema de Analise Fiscal em 22/09/2026 15:19:22. - Data Comentário: 22/09/2026 15:16</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 24/09/2026 - Data Comentário: 18/09/2026 15:24</t>
@@ -33287,9 +33287,6 @@
       <c r="O449">
         <v>18274307</v>
       </c>
-      <c r="P449" t="s">
-        <v>232</v>
-      </c>
       <c r="Q449" t="s">
         <v>251</v>
       </c>
@@ -42169,9 +42166,6 @@
       <c r="O573">
         <v>18275526</v>
       </c>
-      <c r="P573" t="s">
-        <v>247</v>
-      </c>
       <c r="Q573" t="s">
         <v>251</v>
       </c>
@@ -42240,9 +42234,6 @@
       <c r="O574">
         <v>18274091</v>
       </c>
-      <c r="P574" t="s">
-        <v>247</v>
-      </c>
       <c r="Q574" t="s">
         <v>251</v>
       </c>
@@ -42578,7 +42569,7 @@
         <v>18216396</v>
       </c>
       <c r="P579" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="Q579" t="s">
         <v>252</v>
@@ -42643,7 +42634,7 @@
         <v>18216401</v>
       </c>
       <c r="P580" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="Q580" t="s">
         <v>252</v>
@@ -42708,7 +42699,7 @@
         <v>18216376</v>
       </c>
       <c r="P581" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="Q581" t="s">
         <v>252</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-23 10:00
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8740" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8782" uniqueCount="466">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1444,9 +1444,6 @@
     <t>Isabella Nascimento</t>
   </si>
   <si>
-    <t>Karina Santos</t>
-  </si>
-  <si>
     <t>Fernanda Araujo</t>
   </si>
   <si>
@@ -1456,7 +1453,7 @@
     <t>Leandro Matos</t>
   </si>
   <si>
-    <t>Ricardo Fischer</t>
+    <t>Larice Souza</t>
   </si>
 </sst>
 </file>
@@ -2449,7 +2446,7 @@
         <v>457</v>
       </c>
       <c r="AH9" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="10" spans="1:34">
@@ -2520,7 +2517,7 @@
         <v>457</v>
       </c>
       <c r="AH10" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="11" spans="1:34">
@@ -2588,7 +2585,7 @@
         <v>457</v>
       </c>
       <c r="AH11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="12" spans="1:34">
@@ -2659,7 +2656,7 @@
         <v>457</v>
       </c>
       <c r="AH12" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="13" spans="1:34">
@@ -2736,7 +2733,7 @@
         <v>458</v>
       </c>
       <c r="AH13" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="14" spans="1:34">
@@ -2804,7 +2801,7 @@
         <v>458</v>
       </c>
       <c r="AH14" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="15" spans="1:34">
@@ -2878,7 +2875,7 @@
         <v>458</v>
       </c>
       <c r="AH15" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="16" spans="1:34">
@@ -2951,6 +2948,9 @@
       <c r="AG16" t="s">
         <v>459</v>
       </c>
+      <c r="AH16" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="17" spans="1:34">
       <c r="A17">
@@ -3020,7 +3020,7 @@
         <v>459</v>
       </c>
       <c r="AH17" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="18" spans="1:34">
@@ -3097,7 +3097,7 @@
         <v>459</v>
       </c>
       <c r="AH18" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="19" spans="1:34">
@@ -3171,7 +3171,7 @@
         <v>459</v>
       </c>
       <c r="AH19" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="20" spans="1:34">
@@ -3239,7 +3239,7 @@
         <v>459</v>
       </c>
       <c r="AH20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="21" spans="1:34">
@@ -3312,6 +3312,9 @@
       <c r="AG21" t="s">
         <v>457</v>
       </c>
+      <c r="AH21" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="22" spans="1:34">
       <c r="A22">
@@ -3461,7 +3464,7 @@
         <v>457</v>
       </c>
       <c r="AH23" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="24" spans="1:34">
@@ -3538,7 +3541,7 @@
         <v>457</v>
       </c>
       <c r="AH24" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="25" spans="1:34">
@@ -3615,7 +3618,7 @@
         <v>457</v>
       </c>
       <c r="AH25" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="26" spans="1:34">
@@ -3692,7 +3695,7 @@
         <v>457</v>
       </c>
       <c r="AH26" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="27" spans="1:34">
@@ -3766,7 +3769,7 @@
         <v>457</v>
       </c>
       <c r="AH27" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="28" spans="1:34">
@@ -3917,7 +3920,7 @@
         <v>457</v>
       </c>
       <c r="AH29" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="30" spans="1:34">
@@ -3985,7 +3988,7 @@
         <v>457</v>
       </c>
       <c r="AH30" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="31" spans="1:34">
@@ -4058,6 +4061,9 @@
       <c r="AG31" t="s">
         <v>459</v>
       </c>
+      <c r="AH31" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="32" spans="1:34">
       <c r="A32">
@@ -4133,7 +4139,7 @@
         <v>459</v>
       </c>
       <c r="AH32" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="33" spans="1:34">
@@ -4210,7 +4216,7 @@
         <v>459</v>
       </c>
       <c r="AH33" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="34" spans="1:34">
@@ -4287,7 +4293,7 @@
         <v>459</v>
       </c>
       <c r="AH34" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="35" spans="1:34">
@@ -4361,7 +4367,7 @@
         <v>459</v>
       </c>
       <c r="AH35" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="36" spans="1:34">
@@ -4512,7 +4518,7 @@
         <v>459</v>
       </c>
       <c r="AH37" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="38" spans="1:34">
@@ -4586,7 +4592,7 @@
         <v>459</v>
       </c>
       <c r="AH38" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="39" spans="1:34">
@@ -4653,6 +4659,9 @@
       <c r="AG39" t="s">
         <v>457</v>
       </c>
+      <c r="AH39" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="40" spans="1:34">
       <c r="A40">
@@ -4722,7 +4731,7 @@
         <v>457</v>
       </c>
       <c r="AH40" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="41" spans="1:34">
@@ -4793,7 +4802,7 @@
         <v>457</v>
       </c>
       <c r="AH41" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="42" spans="1:34">
@@ -4864,7 +4873,7 @@
         <v>457</v>
       </c>
       <c r="AH42" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="43" spans="1:34">
@@ -4932,7 +4941,7 @@
         <v>457</v>
       </c>
       <c r="AH43" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="44" spans="1:34">
@@ -5077,7 +5086,7 @@
         <v>457</v>
       </c>
       <c r="AH45" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="46" spans="1:34">
@@ -5145,7 +5154,7 @@
         <v>457</v>
       </c>
       <c r="AH46" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="47" spans="1:34">
@@ -5215,6 +5224,9 @@
       <c r="AG47" t="s">
         <v>458</v>
       </c>
+      <c r="AH47" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="48" spans="1:34">
       <c r="A48">
@@ -5290,7 +5302,7 @@
         <v>458</v>
       </c>
       <c r="AH48" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="49" spans="1:34">
@@ -5364,7 +5376,7 @@
         <v>458</v>
       </c>
       <c r="AH49" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="50" spans="1:34">
@@ -5441,7 +5453,7 @@
         <v>458</v>
       </c>
       <c r="AH50" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="51" spans="1:34">
@@ -5518,7 +5530,7 @@
         <v>458</v>
       </c>
       <c r="AH51" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="52" spans="1:34">
@@ -5589,7 +5601,7 @@
         <v>458</v>
       </c>
       <c r="AH52" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="53" spans="1:34">
@@ -5734,7 +5746,7 @@
         <v>458</v>
       </c>
       <c r="AH54" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="55" spans="1:34">
@@ -5805,7 +5817,7 @@
         <v>458</v>
       </c>
       <c r="AH55" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="56" spans="1:34">
@@ -5872,6 +5884,9 @@
       <c r="AG56" t="s">
         <v>459</v>
       </c>
+      <c r="AH56" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="57" spans="1:34">
       <c r="A57">
@@ -5941,7 +5956,7 @@
         <v>459</v>
       </c>
       <c r="AH57" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="58" spans="1:34">
@@ -6018,7 +6033,7 @@
         <v>459</v>
       </c>
       <c r="AH58" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="59" spans="1:34">
@@ -6092,7 +6107,7 @@
         <v>459</v>
       </c>
       <c r="AH59" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="60" spans="1:34">
@@ -6160,7 +6175,7 @@
         <v>459</v>
       </c>
       <c r="AH60" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="61" spans="1:34">
@@ -6227,6 +6242,9 @@
       <c r="AG61" t="s">
         <v>457</v>
       </c>
+      <c r="AH61" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="62" spans="1:34">
       <c r="A62">
@@ -6296,7 +6314,7 @@
         <v>457</v>
       </c>
       <c r="AH62" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="63" spans="1:34">
@@ -6367,7 +6385,7 @@
         <v>457</v>
       </c>
       <c r="AH63" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="64" spans="1:34">
@@ -6438,7 +6456,7 @@
         <v>457</v>
       </c>
       <c r="AH64" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="65" spans="1:34">
@@ -6509,7 +6527,7 @@
         <v>457</v>
       </c>
       <c r="AH65" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="66" spans="1:34">
@@ -6648,7 +6666,7 @@
         <v>457</v>
       </c>
       <c r="AH67" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="68" spans="1:34">
@@ -6716,7 +6734,7 @@
         <v>457</v>
       </c>
       <c r="AH68" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="69" spans="1:34">
@@ -6793,7 +6811,7 @@
         <v>457</v>
       </c>
       <c r="AH69" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="70" spans="1:34">
@@ -6870,7 +6888,7 @@
         <v>457</v>
       </c>
       <c r="AH70" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="71" spans="1:34">
@@ -6947,7 +6965,7 @@
         <v>457</v>
       </c>
       <c r="AH71" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="72" spans="1:34">
@@ -7021,7 +7039,7 @@
         <v>457</v>
       </c>
       <c r="AH72" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="73" spans="1:34">
@@ -7092,7 +7110,7 @@
         <v>457</v>
       </c>
       <c r="AH73" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="74" spans="1:34">
@@ -7165,6 +7183,9 @@
       <c r="AG74" t="s">
         <v>459</v>
       </c>
+      <c r="AH74" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="75" spans="1:34">
       <c r="A75">
@@ -7314,7 +7335,7 @@
         <v>459</v>
       </c>
       <c r="AH76" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="77" spans="1:34">
@@ -7391,7 +7412,7 @@
         <v>459</v>
       </c>
       <c r="AH77" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="78" spans="1:34">
@@ -7468,7 +7489,7 @@
         <v>459</v>
       </c>
       <c r="AH78" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="79" spans="1:34">
@@ -7542,7 +7563,7 @@
         <v>459</v>
       </c>
       <c r="AH79" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="80" spans="1:34">
@@ -7693,7 +7714,7 @@
         <v>459</v>
       </c>
       <c r="AH81" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="82" spans="1:34">
@@ -7767,7 +7788,7 @@
         <v>459</v>
       </c>
       <c r="AH82" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="83" spans="1:34">
@@ -7844,7 +7865,7 @@
         <v>457</v>
       </c>
       <c r="AH83" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="84" spans="1:34">
@@ -7911,6 +7932,9 @@
       <c r="AG84" t="s">
         <v>457</v>
       </c>
+      <c r="AH84" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="85" spans="1:34">
       <c r="A85">
@@ -8048,7 +8072,7 @@
         <v>457</v>
       </c>
       <c r="AH86" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="87" spans="1:34">
@@ -8119,7 +8143,7 @@
         <v>457</v>
       </c>
       <c r="AH87" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="88" spans="1:34">
@@ -8190,7 +8214,7 @@
         <v>457</v>
       </c>
       <c r="AH88" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="89" spans="1:34">
@@ -8258,7 +8282,7 @@
         <v>457</v>
       </c>
       <c r="AH89" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="90" spans="1:34">
@@ -8397,7 +8421,7 @@
         <v>457</v>
       </c>
       <c r="AH91" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="92" spans="1:34">
@@ -8465,7 +8489,7 @@
         <v>457</v>
       </c>
       <c r="AH92" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="93" spans="1:34">
@@ -8952,6 +8976,9 @@
       <c r="AG99" t="s">
         <v>457</v>
       </c>
+      <c r="AH99" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="100" spans="1:34">
       <c r="A100">
@@ -9221,6 +9248,9 @@
       <c r="AG103" t="s">
         <v>457</v>
       </c>
+      <c r="AH103" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="104" spans="1:34">
       <c r="A104">
@@ -9555,6 +9585,9 @@
       <c r="AG108" t="s">
         <v>457</v>
       </c>
+      <c r="AH108" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="109" spans="1:34">
       <c r="A109">
@@ -9889,6 +9922,9 @@
       <c r="AG113" t="s">
         <v>457</v>
       </c>
+      <c r="AH113" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="114" spans="1:34">
       <c r="A114">
@@ -10096,6 +10132,9 @@
       <c r="AG116" t="s">
         <v>457</v>
       </c>
+      <c r="AH116" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="117" spans="1:34">
       <c r="A117">
@@ -10235,6 +10274,9 @@
       <c r="AG118" t="s">
         <v>457</v>
       </c>
+      <c r="AH118" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="119" spans="1:34">
       <c r="A119">
@@ -10634,6 +10676,9 @@
       <c r="AG124" t="s">
         <v>457</v>
       </c>
+      <c r="AH124" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="125" spans="1:34">
       <c r="A125">
@@ -10767,6 +10812,9 @@
       <c r="AG126" t="s">
         <v>457</v>
       </c>
+      <c r="AH126" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="127" spans="1:34">
       <c r="A127">
@@ -10971,6 +11019,9 @@
       <c r="AG129" t="s">
         <v>457</v>
       </c>
+      <c r="AH129" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="130" spans="1:34">
       <c r="A130">
@@ -11178,6 +11229,9 @@
       <c r="AG132" t="s">
         <v>457</v>
       </c>
+      <c r="AH132" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="133" spans="1:34">
       <c r="A133">
@@ -11512,6 +11566,9 @@
       <c r="AG137" t="s">
         <v>457</v>
       </c>
+      <c r="AH137" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="138" spans="1:34">
       <c r="A138">
@@ -11929,6 +11986,9 @@
       <c r="AG143" t="s">
         <v>459</v>
       </c>
+      <c r="AH143" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="144" spans="1:34">
       <c r="A144">
@@ -12077,6 +12137,9 @@
       <c r="AG145" t="s">
         <v>459</v>
       </c>
+      <c r="AH145" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="146" spans="1:34">
       <c r="A146">
@@ -12367,6 +12430,9 @@
       <c r="AG149" t="s">
         <v>458</v>
       </c>
+      <c r="AH149" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="150" spans="1:34">
       <c r="A150">
@@ -12728,6 +12794,9 @@
       <c r="AG154" t="s">
         <v>458</v>
       </c>
+      <c r="AH154" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="155" spans="1:34">
       <c r="A155">
@@ -12799,6 +12868,9 @@
       <c r="AG155" t="s">
         <v>458</v>
       </c>
+      <c r="AH155" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="156" spans="1:34">
       <c r="A156">
@@ -13151,6 +13223,9 @@
       <c r="AG160" t="s">
         <v>457</v>
       </c>
+      <c r="AH160" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="161" spans="1:34">
       <c r="A161">
@@ -13222,6 +13297,9 @@
       <c r="AG161" t="s">
         <v>457</v>
       </c>
+      <c r="AH161" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="162" spans="1:34">
       <c r="A162">
@@ -13362,7 +13440,7 @@
         <v>457</v>
       </c>
       <c r="AH163" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="164" spans="1:34">
@@ -13430,7 +13508,7 @@
         <v>457</v>
       </c>
       <c r="AH164" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="165" spans="1:34">
@@ -13507,7 +13585,7 @@
         <v>457</v>
       </c>
       <c r="AH165" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="166" spans="1:34">
@@ -13578,7 +13656,7 @@
         <v>457</v>
       </c>
       <c r="AH166" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="167" spans="1:34">
@@ -13646,7 +13724,7 @@
         <v>457</v>
       </c>
       <c r="AH167" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="168" spans="1:34">
@@ -13714,7 +13792,7 @@
         <v>457</v>
       </c>
       <c r="AH168" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="169" spans="1:34">
@@ -13782,7 +13860,7 @@
         <v>457</v>
       </c>
       <c r="AH169" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="170" spans="1:34">
@@ -13859,7 +13937,7 @@
         <v>457</v>
       </c>
       <c r="AH170" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="171" spans="1:34">
@@ -13930,7 +14008,7 @@
         <v>457</v>
       </c>
       <c r="AH171" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="172" spans="1:34">
@@ -13998,7 +14076,7 @@
         <v>457</v>
       </c>
       <c r="AH172" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="173" spans="1:34">
@@ -14066,7 +14144,7 @@
         <v>457</v>
       </c>
       <c r="AH173" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="174" spans="1:34">
@@ -14143,7 +14221,7 @@
         <v>457</v>
       </c>
       <c r="AH174" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="175" spans="1:34">
@@ -14211,7 +14289,7 @@
         <v>457</v>
       </c>
       <c r="AH175" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="176" spans="1:34">
@@ -14282,7 +14360,7 @@
         <v>457</v>
       </c>
       <c r="AH176" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="177" spans="1:34">
@@ -14350,7 +14428,7 @@
         <v>457</v>
       </c>
       <c r="AH177" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="178" spans="1:34">
@@ -14427,7 +14505,7 @@
         <v>457</v>
       </c>
       <c r="AH178" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="179" spans="1:34">
@@ -14498,7 +14576,7 @@
         <v>457</v>
       </c>
       <c r="AH179" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="180" spans="1:34">
@@ -14566,7 +14644,7 @@
         <v>457</v>
       </c>
       <c r="AH180" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="181" spans="1:34">
@@ -14634,7 +14712,7 @@
         <v>457</v>
       </c>
       <c r="AH181" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="182" spans="1:34">
@@ -14705,7 +14783,7 @@
         <v>457</v>
       </c>
       <c r="AH182" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="183" spans="1:34">
@@ -14773,7 +14851,7 @@
         <v>457</v>
       </c>
       <c r="AH183" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="184" spans="1:34">
@@ -14844,7 +14922,7 @@
         <v>457</v>
       </c>
       <c r="AH184" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="185" spans="1:34">
@@ -14912,7 +14990,7 @@
         <v>457</v>
       </c>
       <c r="AH185" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="186" spans="1:34">
@@ -14986,7 +15064,7 @@
         <v>459</v>
       </c>
       <c r="AH186" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="187" spans="1:34">
@@ -15054,7 +15132,7 @@
         <v>459</v>
       </c>
       <c r="AH187" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="188" spans="1:34">
@@ -15122,7 +15200,7 @@
         <v>459</v>
       </c>
       <c r="AH188" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="189" spans="1:34">
@@ -15193,7 +15271,7 @@
         <v>459</v>
       </c>
       <c r="AH189" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="190" spans="1:34">
@@ -15261,7 +15339,7 @@
         <v>459</v>
       </c>
       <c r="AH190" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="191" spans="1:34">
@@ -15332,7 +15410,7 @@
         <v>459</v>
       </c>
       <c r="AH191" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="192" spans="1:34">
@@ -15406,7 +15484,7 @@
         <v>459</v>
       </c>
       <c r="AH192" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="193" spans="1:34">
@@ -15477,7 +15555,7 @@
         <v>459</v>
       </c>
       <c r="AH193" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="194" spans="1:34">
@@ -15551,7 +15629,7 @@
         <v>457</v>
       </c>
       <c r="AH194" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="195" spans="1:34">
@@ -15619,7 +15697,7 @@
         <v>458</v>
       </c>
       <c r="AH195" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="196" spans="1:34">
@@ -15687,7 +15765,7 @@
         <v>458</v>
       </c>
       <c r="AH196" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="197" spans="1:34">
@@ -15758,7 +15836,7 @@
         <v>458</v>
       </c>
       <c r="AH197" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="198" spans="1:34">
@@ -15826,7 +15904,7 @@
         <v>458</v>
       </c>
       <c r="AH198" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="199" spans="1:34">
@@ -15897,7 +15975,7 @@
         <v>458</v>
       </c>
       <c r="AH199" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="200" spans="1:34">
@@ -15965,7 +16043,7 @@
         <v>458</v>
       </c>
       <c r="AH200" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="201" spans="1:34">
@@ -16036,7 +16114,7 @@
         <v>458</v>
       </c>
       <c r="AH201" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="202" spans="1:34">
@@ -16104,7 +16182,7 @@
         <v>458</v>
       </c>
       <c r="AH202" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="203" spans="1:34">
@@ -16175,7 +16253,7 @@
         <v>458</v>
       </c>
       <c r="AH203" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="204" spans="1:34">
@@ -16249,7 +16327,7 @@
         <v>457</v>
       </c>
       <c r="AH204" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="205" spans="1:34">
@@ -16326,7 +16404,7 @@
         <v>457</v>
       </c>
       <c r="AH205" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="206" spans="1:34">
@@ -16397,7 +16475,7 @@
         <v>457</v>
       </c>
       <c r="AH206" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="207" spans="1:34">
@@ -16465,7 +16543,7 @@
         <v>457</v>
       </c>
       <c r="AH207" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="208" spans="1:34">
@@ -16539,7 +16617,7 @@
         <v>457</v>
       </c>
       <c r="AH208" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="209" spans="1:34">
@@ -16610,7 +16688,7 @@
         <v>457</v>
       </c>
       <c r="AH209" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="210" spans="1:34">
@@ -16684,7 +16762,7 @@
         <v>457</v>
       </c>
       <c r="AH210" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="211" spans="1:34">
@@ -16752,7 +16830,7 @@
         <v>457</v>
       </c>
       <c r="AH211" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="212" spans="1:34">
@@ -22408,7 +22486,7 @@
         <v>457</v>
       </c>
       <c r="AH294" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="295" spans="1:34">
@@ -22476,7 +22554,7 @@
         <v>457</v>
       </c>
       <c r="AH295" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="296" spans="1:34">
@@ -22612,7 +22690,7 @@
         <v>458</v>
       </c>
       <c r="AH297" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="298" spans="1:34">
@@ -22683,7 +22761,7 @@
         <v>458</v>
       </c>
       <c r="AH298" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="299" spans="1:34">
@@ -24413,7 +24491,7 @@
         <v>457</v>
       </c>
       <c r="AH323" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="324" spans="1:34">
@@ -24484,7 +24562,7 @@
         <v>457</v>
       </c>
       <c r="AH324" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="325" spans="1:34">
@@ -24552,7 +24630,7 @@
         <v>459</v>
       </c>
       <c r="AH325" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="326" spans="1:34">
@@ -24623,7 +24701,7 @@
         <v>459</v>
       </c>
       <c r="AH326" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="327" spans="1:34">
@@ -24691,7 +24769,7 @@
         <v>459</v>
       </c>
       <c r="AH327" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="328" spans="1:34">
@@ -24762,7 +24840,7 @@
         <v>459</v>
       </c>
       <c r="AH328" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="329" spans="1:34">
@@ -24830,7 +24908,7 @@
         <v>459</v>
       </c>
       <c r="AH329" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="330" spans="1:34">
@@ -24901,7 +24979,7 @@
         <v>459</v>
       </c>
       <c r="AH330" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="331" spans="1:34">
@@ -24969,7 +25047,7 @@
         <v>459</v>
       </c>
       <c r="AH331" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="332" spans="1:34">
@@ -25040,7 +25118,7 @@
         <v>459</v>
       </c>
       <c r="AH332" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="333" spans="1:34">
@@ -25108,7 +25186,7 @@
         <v>459</v>
       </c>
       <c r="AH333" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="334" spans="1:34">
@@ -25179,7 +25257,7 @@
         <v>459</v>
       </c>
       <c r="AH334" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="335" spans="1:34">
@@ -25247,7 +25325,7 @@
         <v>457</v>
       </c>
       <c r="AH335" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="336" spans="1:34">
@@ -25315,7 +25393,7 @@
         <v>457</v>
       </c>
       <c r="AH336" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="337" spans="1:34">
@@ -25386,7 +25464,7 @@
         <v>457</v>
       </c>
       <c r="AH337" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="338" spans="1:34">
@@ -25457,7 +25535,7 @@
         <v>457</v>
       </c>
       <c r="AH338" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="339" spans="1:34">
@@ -25525,7 +25603,7 @@
         <v>457</v>
       </c>
       <c r="AH339" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="340" spans="1:34">
@@ -25596,7 +25674,7 @@
         <v>457</v>
       </c>
       <c r="AH340" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="341" spans="1:34">
@@ -25667,7 +25745,7 @@
         <v>458</v>
       </c>
       <c r="AH341" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="342" spans="1:34">
@@ -25738,7 +25816,7 @@
         <v>459</v>
       </c>
       <c r="AH342" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="343" spans="1:34">
@@ -25809,7 +25887,7 @@
         <v>457</v>
       </c>
       <c r="AH343" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="344" spans="1:34">
@@ -25876,6 +25954,9 @@
       <c r="AG344" t="s">
         <v>457</v>
       </c>
+      <c r="AH344" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="345" spans="1:34">
       <c r="A345">
@@ -26016,7 +26097,7 @@
         <v>459</v>
       </c>
       <c r="AH346" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="347" spans="1:34">
@@ -26087,7 +26168,7 @@
         <v>457</v>
       </c>
       <c r="AH347" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="348" spans="1:34">
@@ -26154,6 +26235,9 @@
       <c r="AG348" t="s">
         <v>459</v>
       </c>
+      <c r="AH348" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="349" spans="1:34">
       <c r="A349">
@@ -26219,6 +26303,9 @@
       <c r="AG349" t="s">
         <v>458</v>
       </c>
+      <c r="AH349" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="350" spans="1:34">
       <c r="A350">
@@ -26288,7 +26375,7 @@
         <v>457</v>
       </c>
       <c r="AH350" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="351" spans="1:34">
@@ -26356,7 +26443,7 @@
         <v>457</v>
       </c>
       <c r="AH351" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="352" spans="1:34">
@@ -26424,7 +26511,7 @@
         <v>458</v>
       </c>
       <c r="AH352" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="353" spans="1:34">
@@ -27982,7 +28069,7 @@
         <v>457</v>
       </c>
       <c r="AH375" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="376" spans="1:34">
@@ -28056,7 +28143,7 @@
         <v>459</v>
       </c>
       <c r="AH376" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="377" spans="1:34">
@@ -28124,7 +28211,7 @@
         <v>457</v>
       </c>
       <c r="AH377" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="378" spans="1:34">
@@ -28195,7 +28282,7 @@
         <v>457</v>
       </c>
       <c r="AH378" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="379" spans="1:34">
@@ -28263,7 +28350,7 @@
         <v>458</v>
       </c>
       <c r="AH379" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="380" spans="1:34">
@@ -28529,7 +28616,7 @@
         <v>458</v>
       </c>
       <c r="AH383" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="384" spans="1:34">
@@ -28600,7 +28687,7 @@
         <v>458</v>
       </c>
       <c r="AH384" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="385" spans="1:34">
@@ -28674,7 +28761,7 @@
         <v>459</v>
       </c>
       <c r="AH385" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="386" spans="1:34">
@@ -28745,7 +28832,7 @@
         <v>457</v>
       </c>
       <c r="AH386" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="387" spans="1:34">
@@ -28813,7 +28900,7 @@
         <v>457</v>
       </c>
       <c r="AH387" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="388" spans="1:34">
@@ -28881,7 +28968,7 @@
         <v>457</v>
       </c>
       <c r="AH388" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="389" spans="1:34">
@@ -28949,7 +29036,7 @@
         <v>457</v>
       </c>
       <c r="AH389" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="390" spans="1:34">
@@ -29020,7 +29107,7 @@
         <v>457</v>
       </c>
       <c r="AH390" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="391" spans="1:34">
@@ -29088,7 +29175,7 @@
         <v>457</v>
       </c>
       <c r="AH391" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="392" spans="1:34">
@@ -29159,7 +29246,7 @@
         <v>457</v>
       </c>
       <c r="AH392" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="393" spans="1:34">
@@ -29236,7 +29323,7 @@
         <v>458</v>
       </c>
       <c r="AH393" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="394" spans="1:34">
@@ -29313,7 +29400,7 @@
         <v>458</v>
       </c>
       <c r="AH394" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="395" spans="1:34">
@@ -29387,7 +29474,7 @@
         <v>458</v>
       </c>
       <c r="AH395" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="396" spans="1:34">
@@ -29455,7 +29542,7 @@
         <v>457</v>
       </c>
       <c r="AH396" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="397" spans="1:34">
@@ -29599,6 +29686,9 @@
       <c r="AG398" t="s">
         <v>457</v>
       </c>
+      <c r="AH398" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="399" spans="1:34">
       <c r="A399">
@@ -29674,7 +29764,7 @@
         <v>457</v>
       </c>
       <c r="AH399" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="400" spans="1:34">
@@ -29751,7 +29841,7 @@
         <v>457</v>
       </c>
       <c r="AH400" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="401" spans="1:34">
@@ -29828,7 +29918,7 @@
         <v>457</v>
       </c>
       <c r="AH401" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="402" spans="1:34">
@@ -29905,7 +29995,7 @@
         <v>457</v>
       </c>
       <c r="AH402" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="403" spans="1:34">
@@ -29973,7 +30063,7 @@
         <v>457</v>
       </c>
       <c r="AH403" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="404" spans="1:34">
@@ -30118,7 +30208,7 @@
         <v>457</v>
       </c>
       <c r="AH405" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="406" spans="1:34">
@@ -30185,6 +30275,9 @@
       <c r="AG406" t="s">
         <v>457</v>
       </c>
+      <c r="AH406" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="407" spans="1:34">
       <c r="A407">
@@ -30260,7 +30353,7 @@
         <v>457</v>
       </c>
       <c r="AH407" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="408" spans="1:34">
@@ -30337,7 +30430,7 @@
         <v>457</v>
       </c>
       <c r="AH408" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="409" spans="1:34">
@@ -30414,7 +30507,7 @@
         <v>457</v>
       </c>
       <c r="AH409" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="410" spans="1:34">
@@ -30491,7 +30584,7 @@
         <v>457</v>
       </c>
       <c r="AH410" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="411" spans="1:34">
@@ -30559,7 +30652,7 @@
         <v>457</v>
       </c>
       <c r="AH411" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="412" spans="1:34">
@@ -30704,7 +30797,7 @@
         <v>457</v>
       </c>
       <c r="AH413" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="414" spans="1:34">
@@ -30774,6 +30867,9 @@
       <c r="AG414" t="s">
         <v>457</v>
       </c>
+      <c r="AH414" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="415" spans="1:34">
       <c r="A415">
@@ -30917,7 +31013,7 @@
         <v>457</v>
       </c>
       <c r="AH416" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="417" spans="1:34">
@@ -30991,7 +31087,7 @@
         <v>457</v>
       </c>
       <c r="AH417" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="418" spans="1:34">
@@ -31065,7 +31161,7 @@
         <v>457</v>
       </c>
       <c r="AH418" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="419" spans="1:34">
@@ -31139,7 +31235,7 @@
         <v>457</v>
       </c>
       <c r="AH419" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="420" spans="1:34">
@@ -31213,7 +31309,7 @@
         <v>457</v>
       </c>
       <c r="AH420" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="421" spans="1:34">
@@ -31358,7 +31454,7 @@
         <v>457</v>
       </c>
       <c r="AH422" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="423" spans="1:34">
@@ -31429,7 +31525,7 @@
         <v>457</v>
       </c>
       <c r="AH423" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="424" spans="1:34">
@@ -31502,6 +31598,9 @@
       <c r="AG424" t="s">
         <v>457</v>
       </c>
+      <c r="AH424" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="425" spans="1:34">
       <c r="A425">
@@ -31577,7 +31676,7 @@
         <v>457</v>
       </c>
       <c r="AH425" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="426" spans="1:34">
@@ -31654,7 +31753,7 @@
         <v>457</v>
       </c>
       <c r="AH426" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="427" spans="1:34">
@@ -31731,7 +31830,7 @@
         <v>457</v>
       </c>
       <c r="AH427" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="428" spans="1:34">
@@ -31808,7 +31907,7 @@
         <v>457</v>
       </c>
       <c r="AH428" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="429" spans="1:34">
@@ -31882,7 +31981,7 @@
         <v>457</v>
       </c>
       <c r="AH429" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="430" spans="1:34">
@@ -32033,7 +32132,7 @@
         <v>457</v>
       </c>
       <c r="AH431" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="432" spans="1:34">
@@ -32242,6 +32341,9 @@
       <c r="AG434" t="s">
         <v>458</v>
       </c>
+      <c r="AH434" t="s">
+        <v>449</v>
+      </c>
     </row>
     <row r="435" spans="1:34">
       <c r="A435">
@@ -32379,7 +32481,7 @@
         <v>458</v>
       </c>
       <c r="AH436" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="437" spans="1:34">
@@ -32450,7 +32552,7 @@
         <v>458</v>
       </c>
       <c r="AH437" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="438" spans="1:34">
@@ -32521,7 +32623,7 @@
         <v>458</v>
       </c>
       <c r="AH438" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="439" spans="1:34">
@@ -32592,7 +32694,7 @@
         <v>458</v>
       </c>
       <c r="AH439" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="440" spans="1:34">
@@ -32731,7 +32833,7 @@
         <v>458</v>
       </c>
       <c r="AH441" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="442" spans="1:34">
@@ -32799,7 +32901,7 @@
         <v>458</v>
       </c>
       <c r="AH442" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="443" spans="1:34">
@@ -33352,7 +33454,7 @@
         <v>458</v>
       </c>
       <c r="AH450" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="451" spans="1:34">
@@ -33493,6 +33595,9 @@
       <c r="AG452" t="s">
         <v>457</v>
       </c>
+      <c r="AH452" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="453" spans="1:34">
       <c r="A453">
@@ -33706,6 +33811,9 @@
       <c r="AG455" t="s">
         <v>457</v>
       </c>
+      <c r="AH455" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="456" spans="1:34">
       <c r="A456">
@@ -34073,6 +34181,9 @@
       <c r="AG460" t="s">
         <v>458</v>
       </c>
+      <c r="AH460" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="461" spans="1:34">
       <c r="A461">
@@ -34280,6 +34391,9 @@
       <c r="AG463" t="s">
         <v>457</v>
       </c>
+      <c r="AH463" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="464" spans="1:34">
       <c r="A464">
@@ -34422,6 +34536,9 @@
       <c r="AG465" t="s">
         <v>458</v>
       </c>
+      <c r="AH465" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="466" spans="1:34">
       <c r="A466">
@@ -34712,6 +34829,9 @@
       <c r="AG469" t="s">
         <v>458</v>
       </c>
+      <c r="AH469" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="470" spans="1:34">
       <c r="A470">
@@ -34860,6 +34980,9 @@
       <c r="AG471" t="s">
         <v>457</v>
       </c>
+      <c r="AH471" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="472" spans="1:34">
       <c r="A472">
@@ -35151,7 +35274,7 @@
         <v>457</v>
       </c>
       <c r="AH475" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="476" spans="1:34">
@@ -35225,7 +35348,7 @@
         <v>457</v>
       </c>
       <c r="AH476" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="477" spans="1:34">
@@ -35299,7 +35422,7 @@
         <v>457</v>
       </c>
       <c r="AH477" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="478" spans="1:34">
@@ -35376,7 +35499,7 @@
         <v>457</v>
       </c>
       <c r="AH478" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="479" spans="1:34">
@@ -35453,7 +35576,7 @@
         <v>458</v>
       </c>
       <c r="AH479" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="480" spans="1:34">
@@ -35527,7 +35650,7 @@
         <v>458</v>
       </c>
       <c r="AH480" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="481" spans="1:34">
@@ -35598,7 +35721,7 @@
         <v>458</v>
       </c>
       <c r="AH481" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="482" spans="1:34">
@@ -35675,7 +35798,7 @@
         <v>458</v>
       </c>
       <c r="AH482" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="483" spans="1:34">
@@ -35749,7 +35872,7 @@
         <v>458</v>
       </c>
       <c r="AH483" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="484" spans="1:34">
@@ -35823,7 +35946,7 @@
         <v>458</v>
       </c>
       <c r="AH484" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="485" spans="1:34">
@@ -35897,7 +36020,7 @@
         <v>458</v>
       </c>
       <c r="AH485" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="486" spans="1:34">
@@ -35968,7 +36091,7 @@
         <v>457</v>
       </c>
       <c r="AH486" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="487" spans="1:34">
@@ -36039,7 +36162,7 @@
         <v>458</v>
       </c>
       <c r="AH487" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="488" spans="1:34">
@@ -36113,7 +36236,7 @@
         <v>458</v>
       </c>
       <c r="AH488" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="489" spans="1:34">
@@ -36181,7 +36304,7 @@
         <v>458</v>
       </c>
       <c r="AH489" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="490" spans="1:34">
@@ -36255,7 +36378,7 @@
         <v>458</v>
       </c>
       <c r="AH490" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="491" spans="1:34">
@@ -36329,7 +36452,7 @@
         <v>458</v>
       </c>
       <c r="AH491" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="492" spans="1:34">
@@ -36403,7 +36526,7 @@
         <v>458</v>
       </c>
       <c r="AH492" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="493" spans="1:34">
@@ -36474,7 +36597,7 @@
         <v>457</v>
       </c>
       <c r="AH493" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="494" spans="1:34">
@@ -36545,7 +36668,7 @@
         <v>457</v>
       </c>
       <c r="AH494" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="495" spans="1:34">
@@ -36619,7 +36742,7 @@
         <v>458</v>
       </c>
       <c r="AH495" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="496" spans="1:34">
@@ -42568,7 +42691,7 @@
         <v>457</v>
       </c>
       <c r="AH579" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="580" spans="1:34">
@@ -42633,7 +42756,7 @@
         <v>457</v>
       </c>
       <c r="AH580" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="581" spans="1:34">
@@ -42698,7 +42821,7 @@
         <v>457</v>
       </c>
       <c r="AH581" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="582" spans="1:34">
@@ -42763,7 +42886,7 @@
         <v>458</v>
       </c>
       <c r="AH582" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="583" spans="1:34">
@@ -42828,7 +42951,7 @@
         <v>457</v>
       </c>
       <c r="AH583" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="584" spans="1:34">

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 16:53
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1045,8 +1045,8 @@
 Reunião confirmada pelo cliente - Data Comentário: 04/09/2026 11:03</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 23/09/2026 
-Em atendimento - Data Comentário: 23/09/2026 18:28</t>
+    <t>Aguardando a Liberação da Gerência de Contas   Previsão para conclusão dia 24/09/2026 
+SALDO CREDOR - Data Comentário: 24/09/2026 16:23</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 25/09/2026 - Data Comentário: 18/09/2026 15:25</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 19:23
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1393,8 +1393,8 @@
 Reunião confirmada pelo cliente - Data Comentário: 22/09/2026 11:45</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/09/2026 
-Sem informações que permite identificar e aplicar modelo - Data Comentário: 23/09/2026 18:28</t>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 25/09/2026 
+Sem informações que permite identificar e aplicar modelo - Data Comentário: 24/09/2026 18:27</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/09/2026 
@@ -42756,7 +42756,7 @@
         <v>46269</v>
       </c>
       <c r="M579" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="N579" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-28 09:54
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8828" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8841" uniqueCount="498">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1445,46 +1445,47 @@
 Aguardando assinatura do contrato, link enviado ao cliente! - Data Comentário: 23/09/2026 08:19</t>
   </si>
   <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11617; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: pvolpe - Data Comentário: 18/09/2026 15:28</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11686; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11687; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11688; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11689; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11070; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11870; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11871; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11868; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11684; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11681; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11680; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11683; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
-  </si>
-  <si>
-    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11682; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 14/09/2026 15:08</t>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 29/09/2026 
+Priscila - em atendimento - Data Comentário: 28/09/2026 08:50</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11686; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11687; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11688; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11689; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11070; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11870; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11871; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11868; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11684; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11681; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11680; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11683; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
+  </si>
+  <si>
+    <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 7095; Tarefa Incluida: 11682; Vencimento: 14/09/2026 00:00:00; UsuarioResponsavel: sfernandes - Data Comentário: 28/09/2026 09:11</t>
   </si>
   <si>
     <t>Juan Rodrigues</t>
@@ -42789,7 +42790,7 @@
         <v>46293</v>
       </c>
       <c r="M581" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N581" t="s">
         <v>217</v>
@@ -42850,6 +42851,9 @@
       <c r="L582" s="1">
         <v>46293</v>
       </c>
+      <c r="M582" t="s">
+        <v>204</v>
+      </c>
       <c r="N582" t="s">
         <v>217</v>
       </c>
@@ -42909,6 +42913,9 @@
       <c r="L583" s="1">
         <v>46293</v>
       </c>
+      <c r="M583" t="s">
+        <v>204</v>
+      </c>
       <c r="N583" t="s">
         <v>217</v>
       </c>
@@ -42968,6 +42975,9 @@
       <c r="L584" s="1">
         <v>46293</v>
       </c>
+      <c r="M584" t="s">
+        <v>204</v>
+      </c>
       <c r="N584" t="s">
         <v>217</v>
       </c>
@@ -43027,6 +43037,9 @@
       <c r="L585" s="1">
         <v>46293</v>
       </c>
+      <c r="M585" t="s">
+        <v>204</v>
+      </c>
       <c r="N585" t="s">
         <v>217</v>
       </c>
@@ -43086,6 +43099,9 @@
       <c r="L586" s="1">
         <v>46293</v>
       </c>
+      <c r="M586" t="s">
+        <v>204</v>
+      </c>
       <c r="N586" t="s">
         <v>217</v>
       </c>
@@ -43145,6 +43161,9 @@
       <c r="L587" s="1">
         <v>46293</v>
       </c>
+      <c r="M587" t="s">
+        <v>204</v>
+      </c>
       <c r="N587" t="s">
         <v>217</v>
       </c>
@@ -43204,6 +43223,9 @@
       <c r="L588" s="1">
         <v>46293</v>
       </c>
+      <c r="M588" t="s">
+        <v>204</v>
+      </c>
       <c r="N588" t="s">
         <v>217</v>
       </c>
@@ -43263,6 +43285,9 @@
       <c r="L589" s="1">
         <v>46293</v>
       </c>
+      <c r="M589" t="s">
+        <v>204</v>
+      </c>
       <c r="N589" t="s">
         <v>217</v>
       </c>
@@ -43322,6 +43347,9 @@
       <c r="L590" s="1">
         <v>46293</v>
       </c>
+      <c r="M590" t="s">
+        <v>204</v>
+      </c>
       <c r="N590" t="s">
         <v>217</v>
       </c>
@@ -43381,6 +43409,9 @@
       <c r="L591" s="1">
         <v>46293</v>
       </c>
+      <c r="M591" t="s">
+        <v>204</v>
+      </c>
       <c r="N591" t="s">
         <v>217</v>
       </c>
@@ -43440,6 +43471,9 @@
       <c r="L592" s="1">
         <v>46293</v>
       </c>
+      <c r="M592" t="s">
+        <v>204</v>
+      </c>
       <c r="N592" t="s">
         <v>217</v>
       </c>
@@ -43499,6 +43533,9 @@
       <c r="L593" s="1">
         <v>46293</v>
       </c>
+      <c r="M593" t="s">
+        <v>204</v>
+      </c>
       <c r="N593" t="s">
         <v>217</v>
       </c>
@@ -43557,6 +43594,9 @@
       </c>
       <c r="L594" s="1">
         <v>46293</v>
+      </c>
+      <c r="M594" t="s">
+        <v>204</v>
       </c>
       <c r="N594" t="s">
         <v>217</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-29 14:48
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1075,9 +1075,6 @@
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/09/2026 - Data Comentário: 28/09/2026 11:14</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 29/09/2026 - Data Comentário: 28/09/2026 17:58</t>
-  </si>
-  <si>
     <t>Atraso da Operação, processo em elaboração conforme data prevista - Data Comentário: 28/09/2026 17:35</t>
   </si>
   <si>
@@ -1112,6 +1109,9 @@
   </si>
   <si>
     <t>Tarefa baixada automaticamente, cliente baixado com prejuizo na 1 Quota. - Data Comentário: 30/07/2026 12:07</t>
+  </si>
+  <si>
+    <t>Baixado via API integração MGC x Analise Balanço em 29/09/2026 14:12:54. - Data Comentário: 29/09/2026 14:07</t>
   </si>
   <si>
     <t>Baixado via API integração MGC x Analise Balanço em 24/09/2026 13:45:22. - Data Comentário: 24/09/2026 13:40</t>
@@ -23049,16 +23049,16 @@
     </row>
     <row r="303" spans="1:34">
       <c r="A303">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B303" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C303" t="s">
         <v>54</v>
       </c>
       <c r="D303" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E303" t="s">
         <v>58</v>
@@ -23067,7 +23067,7 @@
         <v>60</v>
       </c>
       <c r="G303">
-        <v>10988</v>
+        <v>7874</v>
       </c>
       <c r="H303">
         <v>0</v>
@@ -23076,19 +23076,16 @@
         <v>64</v>
       </c>
       <c r="J303" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L303" s="1">
         <v>46295</v>
       </c>
-      <c r="M303" t="s">
-        <v>189</v>
-      </c>
       <c r="N303" t="s">
         <v>202</v>
       </c>
       <c r="O303">
-        <v>18112918</v>
+        <v>18130463</v>
       </c>
       <c r="P303" t="s">
         <v>230</v>
@@ -23100,7 +23097,10 @@
         <v>-1</v>
       </c>
       <c r="T303" t="s">
-        <v>248</v>
+        <v>247</v>
+      </c>
+      <c r="V303" t="s">
+        <v>253</v>
       </c>
       <c r="W303" t="s">
         <v>344</v>
@@ -23117,10 +23117,10 @@
     </row>
     <row r="304" spans="1:34">
       <c r="A304">
-        <v>6486</v>
+        <v>6704</v>
       </c>
       <c r="B304" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C304" t="s">
         <v>54</v>
@@ -23153,10 +23153,10 @@
         <v>202</v>
       </c>
       <c r="O304">
-        <v>18130463</v>
+        <v>18096767</v>
       </c>
       <c r="P304" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="Q304" t="s">
         <v>239</v>
@@ -23165,14 +23165,11 @@
         <v>-1</v>
       </c>
       <c r="T304" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="V304" t="s">
         <v>253</v>
       </c>
-      <c r="W304" t="s">
-        <v>345</v>
-      </c>
       <c r="AA304">
         <v>0</v>
       </c>
@@ -23180,21 +23177,21 @@
         <v>471</v>
       </c>
       <c r="AH304" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="305" spans="1:34">
       <c r="A305">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B305" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C305" t="s">
         <v>54</v>
       </c>
       <c r="D305" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E305" t="s">
         <v>58</v>
@@ -23203,7 +23200,7 @@
         <v>60</v>
       </c>
       <c r="G305">
-        <v>7874</v>
+        <v>9762</v>
       </c>
       <c r="H305">
         <v>0</v>
@@ -23212,7 +23209,7 @@
         <v>64</v>
       </c>
       <c r="J305" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L305" s="1">
         <v>46295</v>
@@ -23221,7 +23218,7 @@
         <v>202</v>
       </c>
       <c r="O305">
-        <v>18096767</v>
+        <v>18096939</v>
       </c>
       <c r="P305" t="s">
         <v>212</v>
@@ -23235,9 +23232,6 @@
       <c r="T305" t="s">
         <v>246</v>
       </c>
-      <c r="V305" t="s">
-        <v>253</v>
-      </c>
       <c r="AA305">
         <v>0</v>
       </c>
@@ -23250,10 +23244,10 @@
     </row>
     <row r="306" spans="1:34">
       <c r="A306">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B306" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C306" t="s">
         <v>54</v>
@@ -23286,7 +23280,7 @@
         <v>202</v>
       </c>
       <c r="O306">
-        <v>18096939</v>
+        <v>18130484</v>
       </c>
       <c r="P306" t="s">
         <v>212</v>
@@ -23300,6 +23294,9 @@
       <c r="T306" t="s">
         <v>246</v>
       </c>
+      <c r="V306" t="s">
+        <v>253</v>
+      </c>
       <c r="AA306">
         <v>0</v>
       </c>
@@ -23312,16 +23309,16 @@
     </row>
     <row r="307" spans="1:34">
       <c r="A307">
-        <v>6779</v>
+        <v>5417</v>
       </c>
       <c r="B307" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C307" t="s">
         <v>54</v>
       </c>
       <c r="D307" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E307" t="s">
         <v>58</v>
@@ -23330,16 +23327,16 @@
         <v>60</v>
       </c>
       <c r="G307">
-        <v>9762</v>
+        <v>943</v>
       </c>
       <c r="H307">
         <v>0</v>
       </c>
       <c r="I307" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J307" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L307" s="1">
         <v>46295</v>
@@ -23348,10 +23345,10 @@
         <v>202</v>
       </c>
       <c r="O307">
-        <v>18130484</v>
+        <v>17398859</v>
       </c>
       <c r="P307" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="Q307" t="s">
         <v>239</v>
@@ -23360,10 +23357,7 @@
         <v>-1</v>
       </c>
       <c r="T307" t="s">
-        <v>246</v>
-      </c>
-      <c r="V307" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="AA307">
         <v>0</v>
@@ -23371,16 +23365,13 @@
       <c r="AG307" t="s">
         <v>471</v>
       </c>
-      <c r="AH307" t="s">
-        <v>475</v>
-      </c>
     </row>
     <row r="308" spans="1:34">
       <c r="A308">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B308" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C308" t="s">
         <v>54</v>
@@ -23413,7 +23404,7 @@
         <v>202</v>
       </c>
       <c r="O308">
-        <v>17398859</v>
+        <v>16975890</v>
       </c>
       <c r="P308" t="s">
         <v>227</v>
@@ -23425,7 +23416,10 @@
         <v>-1</v>
       </c>
       <c r="T308" t="s">
-        <v>245</v>
+        <v>247</v>
+      </c>
+      <c r="V308" t="s">
+        <v>253</v>
       </c>
       <c r="AA308">
         <v>0</v>
@@ -23436,16 +23430,16 @@
     </row>
     <row r="309" spans="1:34">
       <c r="A309">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B309" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C309" t="s">
         <v>54</v>
       </c>
       <c r="D309" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E309" t="s">
         <v>58</v>
@@ -23472,7 +23466,7 @@
         <v>202</v>
       </c>
       <c r="O309">
-        <v>16975890</v>
+        <v>17941122</v>
       </c>
       <c r="P309" t="s">
         <v>227</v>
@@ -23484,10 +23478,7 @@
         <v>-1</v>
       </c>
       <c r="T309" t="s">
-        <v>247</v>
-      </c>
-      <c r="V309" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="AA309">
         <v>0</v>
@@ -23498,16 +23489,16 @@
     </row>
     <row r="310" spans="1:34">
       <c r="A310">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B310" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C310" t="s">
         <v>54</v>
       </c>
       <c r="D310" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E310" t="s">
         <v>58</v>
@@ -23534,7 +23525,7 @@
         <v>202</v>
       </c>
       <c r="O310">
-        <v>17941122</v>
+        <v>17952314</v>
       </c>
       <c r="P310" t="s">
         <v>227</v>
@@ -23546,7 +23537,10 @@
         <v>-1</v>
       </c>
       <c r="T310" t="s">
-        <v>248</v>
+        <v>246</v>
+      </c>
+      <c r="V310" t="s">
+        <v>253</v>
       </c>
       <c r="AA310">
         <v>0</v>
@@ -23557,16 +23551,16 @@
     </row>
     <row r="311" spans="1:34">
       <c r="A311">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B311" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C311" t="s">
         <v>54</v>
       </c>
       <c r="D311" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E311" t="s">
         <v>58</v>
@@ -23593,7 +23587,7 @@
         <v>202</v>
       </c>
       <c r="O311">
-        <v>17952314</v>
+        <v>17952513</v>
       </c>
       <c r="P311" t="s">
         <v>227</v>
@@ -23607,9 +23601,6 @@
       <c r="T311" t="s">
         <v>246</v>
       </c>
-      <c r="V311" t="s">
-        <v>253</v>
-      </c>
       <c r="AA311">
         <v>0</v>
       </c>
@@ -23619,22 +23610,22 @@
     </row>
     <row r="312" spans="1:34">
       <c r="A312">
-        <v>6705</v>
+        <v>6949</v>
       </c>
       <c r="B312" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C312" t="s">
         <v>54</v>
       </c>
       <c r="D312" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E312" t="s">
         <v>58</v>
       </c>
       <c r="F312" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G312">
         <v>943</v>
@@ -23655,7 +23646,7 @@
         <v>202</v>
       </c>
       <c r="O312">
-        <v>17952513</v>
+        <v>18178126</v>
       </c>
       <c r="P312" t="s">
         <v>227</v>
@@ -23667,7 +23658,7 @@
         <v>-1</v>
       </c>
       <c r="T312" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="AA312">
         <v>0</v>
@@ -23678,16 +23669,16 @@
     </row>
     <row r="313" spans="1:34">
       <c r="A313">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B313" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C313" t="s">
         <v>54</v>
       </c>
       <c r="D313" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E313" t="s">
         <v>58</v>
@@ -23714,7 +23705,7 @@
         <v>202</v>
       </c>
       <c r="O313">
-        <v>18178126</v>
+        <v>18188710</v>
       </c>
       <c r="P313" t="s">
         <v>227</v>
@@ -23726,7 +23717,7 @@
         <v>-1</v>
       </c>
       <c r="T313" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AA313">
         <v>0</v>
@@ -23737,10 +23728,10 @@
     </row>
     <row r="314" spans="1:34">
       <c r="A314">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B314" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C314" t="s">
         <v>54</v>
@@ -23773,7 +23764,7 @@
         <v>202</v>
       </c>
       <c r="O314">
-        <v>18188710</v>
+        <v>18188616</v>
       </c>
       <c r="P314" t="s">
         <v>227</v>
@@ -23796,75 +23787,93 @@
     </row>
     <row r="315" spans="1:34">
       <c r="A315">
-        <v>6963</v>
+        <v>6627</v>
       </c>
       <c r="B315" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C315" t="s">
         <v>54</v>
       </c>
       <c r="D315" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E315" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F315" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G315">
-        <v>943</v>
+        <v>7869</v>
       </c>
       <c r="H315">
         <v>0</v>
       </c>
       <c r="I315" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J315" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L315" s="1">
-        <v>46295</v>
+        <v>46293</v>
+      </c>
+      <c r="M315" t="s">
+        <v>191</v>
       </c>
       <c r="N315" t="s">
         <v>202</v>
       </c>
       <c r="O315">
-        <v>18188616</v>
+        <v>17042546</v>
       </c>
       <c r="P315" t="s">
-        <v>227</v>
+        <v>208</v>
       </c>
       <c r="Q315" t="s">
-        <v>239</v>
+        <v>237</v>
+      </c>
+      <c r="R315" s="1">
+        <v>46288.76065641204</v>
       </c>
       <c r="S315">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T315" t="s">
-        <v>244</v>
+        <v>241</v>
+      </c>
+      <c r="V315" t="s">
+        <v>253</v>
+      </c>
+      <c r="W315" t="s">
+        <v>345</v>
       </c>
       <c r="AA315">
         <v>0</v>
+      </c>
+      <c r="AB315" t="s">
+        <v>466</v>
       </c>
       <c r="AG315" t="s">
         <v>471</v>
       </c>
+      <c r="AH315" t="s">
+        <v>474</v>
+      </c>
     </row>
     <row r="316" spans="1:34">
       <c r="A316">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B316" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C316" t="s">
         <v>54</v>
       </c>
       <c r="D316" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E316" t="s">
         <v>59</v>
@@ -23894,7 +23903,7 @@
         <v>202</v>
       </c>
       <c r="O316">
-        <v>17042546</v>
+        <v>16960048</v>
       </c>
       <c r="P316" t="s">
         <v>208</v>
@@ -23903,7 +23912,7 @@
         <v>237</v>
       </c>
       <c r="R316" s="1">
-        <v>46288.76065641204</v>
+        <v>46288.7606568287</v>
       </c>
       <c r="S316">
         <v>1</v>
@@ -23915,7 +23924,7 @@
         <v>253</v>
       </c>
       <c r="W316" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AA316">
         <v>0</v>
@@ -23932,22 +23941,22 @@
     </row>
     <row r="317" spans="1:34">
       <c r="A317">
-        <v>6628</v>
+        <v>6949</v>
       </c>
       <c r="B317" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C317" t="s">
         <v>54</v>
       </c>
       <c r="D317" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E317" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F317" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G317">
         <v>7869</v>
@@ -23971,28 +23980,25 @@
         <v>202</v>
       </c>
       <c r="O317">
-        <v>16960048</v>
+        <v>18178300</v>
       </c>
       <c r="P317" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q317" t="s">
         <v>237</v>
       </c>
       <c r="R317" s="1">
-        <v>46288.7606568287</v>
+        <v>46288.76066791666</v>
       </c>
       <c r="S317">
         <v>1</v>
       </c>
       <c r="T317" t="s">
-        <v>241</v>
-      </c>
-      <c r="V317" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="W317" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AA317">
         <v>0</v>
@@ -24004,30 +24010,30 @@
         <v>471</v>
       </c>
       <c r="AH317" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="318" spans="1:34">
       <c r="A318">
-        <v>6949</v>
+        <v>6628</v>
       </c>
       <c r="B318" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C318" t="s">
         <v>54</v>
       </c>
       <c r="D318" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E318" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F318" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G318">
-        <v>7869</v>
+        <v>1650</v>
       </c>
       <c r="H318">
         <v>0</v>
@@ -24036,57 +24042,54 @@
         <v>63</v>
       </c>
       <c r="J318" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L318" s="1">
         <v>46293</v>
       </c>
-      <c r="M318" t="s">
-        <v>191</v>
-      </c>
       <c r="N318" t="s">
         <v>202</v>
       </c>
       <c r="O318">
-        <v>18178300</v>
+        <v>16959974</v>
       </c>
       <c r="P318" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q318" t="s">
         <v>237</v>
       </c>
       <c r="R318" s="1">
-        <v>46288.76066791666</v>
+        <v>46265.00248284722</v>
       </c>
       <c r="S318">
         <v>1</v>
       </c>
       <c r="T318" t="s">
-        <v>243</v>
-      </c>
-      <c r="W318" t="s">
-        <v>346</v>
+        <v>241</v>
+      </c>
+      <c r="V318" t="s">
+        <v>253</v>
       </c>
       <c r="AA318">
         <v>0</v>
       </c>
       <c r="AB318" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="AG318" t="s">
         <v>471</v>
       </c>
       <c r="AH318" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="319" spans="1:34">
       <c r="A319">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B319" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C319" t="s">
         <v>54</v>
@@ -24095,10 +24098,10 @@
         <v>56</v>
       </c>
       <c r="E319" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F319" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G319">
         <v>1650</v>
@@ -24119,25 +24122,22 @@
         <v>202</v>
       </c>
       <c r="O319">
-        <v>16959974</v>
+        <v>18163667</v>
       </c>
       <c r="P319" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q319" t="s">
         <v>237</v>
       </c>
       <c r="R319" s="1">
-        <v>46265.00248284722</v>
+        <v>46265.00255472222</v>
       </c>
       <c r="S319">
         <v>1</v>
       </c>
       <c r="T319" t="s">
-        <v>241</v>
-      </c>
-      <c r="V319" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="AA319">
         <v>0</v>
@@ -24154,25 +24154,25 @@
     </row>
     <row r="320" spans="1:34">
       <c r="A320">
-        <v>6945</v>
+        <v>6548</v>
       </c>
       <c r="B320" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C320" t="s">
         <v>54</v>
       </c>
       <c r="D320" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E320" t="s">
         <v>58</v>
       </c>
       <c r="F320" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G320">
-        <v>1650</v>
+        <v>6892</v>
       </c>
       <c r="H320">
         <v>0</v>
@@ -24181,51 +24181,54 @@
         <v>63</v>
       </c>
       <c r="J320" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L320" s="1">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="N320" t="s">
         <v>202</v>
       </c>
       <c r="O320">
-        <v>18163667</v>
+        <v>17968017</v>
       </c>
       <c r="P320" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Q320" t="s">
         <v>237</v>
       </c>
       <c r="R320" s="1">
-        <v>46265.00255472222</v>
+        <v>46290.56449253472</v>
       </c>
       <c r="S320">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T320" t="s">
-        <v>242</v>
+        <v>240</v>
+      </c>
+      <c r="V320" t="s">
+        <v>253</v>
       </c>
       <c r="AA320">
         <v>0</v>
       </c>
       <c r="AB320" t="s">
-        <v>461</v>
+        <v>207</v>
       </c>
       <c r="AG320" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="AH320" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="321" spans="1:34">
       <c r="A321">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B321" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C321" t="s">
         <v>54</v>
@@ -24234,7 +24237,7 @@
         <v>55</v>
       </c>
       <c r="E321" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F321" t="s">
         <v>60</v>
@@ -24258,22 +24261,22 @@
         <v>202</v>
       </c>
       <c r="O321">
-        <v>17968017</v>
+        <v>17042486</v>
       </c>
       <c r="P321" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q321" t="s">
         <v>237</v>
       </c>
       <c r="R321" s="1">
-        <v>46290.56449253472</v>
+        <v>46290.56093913194</v>
       </c>
       <c r="S321">
         <v>4</v>
       </c>
       <c r="T321" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="V321" t="s">
         <v>253</v>
@@ -24282,27 +24285,27 @@
         <v>0</v>
       </c>
       <c r="AB321" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AG321" t="s">
         <v>473</v>
       </c>
       <c r="AH321" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="322" spans="1:34">
       <c r="A322">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B322" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C322" t="s">
         <v>54</v>
       </c>
       <c r="D322" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E322" t="s">
         <v>59</v>
@@ -24329,7 +24332,7 @@
         <v>202</v>
       </c>
       <c r="O322">
-        <v>17042486</v>
+        <v>16960024</v>
       </c>
       <c r="P322" t="s">
         <v>208</v>
@@ -24338,7 +24341,7 @@
         <v>237</v>
       </c>
       <c r="R322" s="1">
-        <v>46290.56093913194</v>
+        <v>46289.64172979166</v>
       </c>
       <c r="S322">
         <v>4</v>
@@ -24353,7 +24356,7 @@
         <v>0</v>
       </c>
       <c r="AB322" t="s">
-        <v>208</v>
+        <v>461</v>
       </c>
       <c r="AG322" t="s">
         <v>473</v>
@@ -24364,10 +24367,10 @@
     </row>
     <row r="323" spans="1:34">
       <c r="A323">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B323" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C323" t="s">
         <v>54</v>
@@ -24376,10 +24379,10 @@
         <v>56</v>
       </c>
       <c r="E323" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F323" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G323">
         <v>6892</v>
@@ -24396,35 +24399,38 @@
       <c r="L323" s="1">
         <v>46290</v>
       </c>
+      <c r="M323" t="s">
+        <v>190</v>
+      </c>
       <c r="N323" t="s">
         <v>202</v>
       </c>
       <c r="O323">
-        <v>16960024</v>
+        <v>18163676</v>
       </c>
       <c r="P323" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q323" t="s">
         <v>237</v>
       </c>
       <c r="R323" s="1">
-        <v>46289.64172979166</v>
+        <v>46289.56480809028</v>
       </c>
       <c r="S323">
         <v>4</v>
       </c>
       <c r="T323" t="s">
-        <v>241</v>
-      </c>
-      <c r="V323" t="s">
-        <v>253</v>
+        <v>242</v>
+      </c>
+      <c r="W323" t="s">
+        <v>346</v>
       </c>
       <c r="AA323">
         <v>0</v>
       </c>
       <c r="AB323" t="s">
-        <v>461</v>
+        <v>209</v>
       </c>
       <c r="AG323" t="s">
         <v>473</v>
@@ -24435,16 +24441,16 @@
     </row>
     <row r="324" spans="1:34">
       <c r="A324">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B324" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C324" t="s">
         <v>54</v>
       </c>
       <c r="D324" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E324" t="s">
         <v>58</v>
@@ -24467,58 +24473,52 @@
       <c r="L324" s="1">
         <v>46290</v>
       </c>
-      <c r="M324" t="s">
-        <v>190</v>
-      </c>
       <c r="N324" t="s">
         <v>202</v>
       </c>
       <c r="O324">
-        <v>18163676</v>
+        <v>18178288</v>
       </c>
       <c r="P324" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Q324" t="s">
         <v>237</v>
       </c>
       <c r="R324" s="1">
-        <v>46289.56480809028</v>
+        <v>46290.56969825231</v>
       </c>
       <c r="S324">
         <v>4</v>
       </c>
       <c r="T324" t="s">
-        <v>242</v>
-      </c>
-      <c r="W324" t="s">
-        <v>347</v>
+        <v>243</v>
       </c>
       <c r="AA324">
         <v>0</v>
       </c>
       <c r="AB324" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="AG324" t="s">
         <v>473</v>
       </c>
       <c r="AH324" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="325" spans="1:34">
       <c r="A325">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B325" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C325" t="s">
         <v>54</v>
       </c>
       <c r="D325" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E325" t="s">
         <v>58</v>
@@ -24545,42 +24545,42 @@
         <v>202</v>
       </c>
       <c r="O325">
-        <v>18178288</v>
+        <v>18187955</v>
       </c>
       <c r="P325" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Q325" t="s">
         <v>237</v>
       </c>
       <c r="R325" s="1">
-        <v>46290.56969825231</v>
+        <v>46290.481633125</v>
       </c>
       <c r="S325">
         <v>4</v>
       </c>
       <c r="T325" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AA325">
         <v>0</v>
       </c>
       <c r="AB325" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AG325" t="s">
         <v>473</v>
       </c>
       <c r="AH325" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="326" spans="1:34">
       <c r="A326">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B326" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C326" t="s">
         <v>54</v>
@@ -24613,7 +24613,7 @@
         <v>202</v>
       </c>
       <c r="O326">
-        <v>18187955</v>
+        <v>18187893</v>
       </c>
       <c r="P326" t="s">
         <v>210</v>
@@ -24622,7 +24622,7 @@
         <v>237</v>
       </c>
       <c r="R326" s="1">
-        <v>46290.481633125</v>
+        <v>46290.48190942129</v>
       </c>
       <c r="S326">
         <v>4</v>
@@ -24645,25 +24645,25 @@
     </row>
     <row r="327" spans="1:34">
       <c r="A327">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B327" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C327" t="s">
         <v>54</v>
       </c>
       <c r="D327" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E327" t="s">
         <v>58</v>
       </c>
       <c r="F327" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G327">
-        <v>6892</v>
+        <v>1652</v>
       </c>
       <c r="H327">
         <v>0</v>
@@ -24672,51 +24672,57 @@
         <v>63</v>
       </c>
       <c r="J327" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L327" s="1">
         <v>46290</v>
       </c>
       <c r="N327" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="O327">
-        <v>18187893</v>
+        <v>17967989</v>
       </c>
       <c r="P327" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="Q327" t="s">
         <v>237</v>
       </c>
       <c r="R327" s="1">
-        <v>46290.48190942129</v>
+        <v>46234.66180127315</v>
       </c>
       <c r="S327">
         <v>4</v>
       </c>
       <c r="T327" t="s">
-        <v>244</v>
+        <v>240</v>
+      </c>
+      <c r="V327" t="s">
+        <v>253</v>
+      </c>
+      <c r="W327" t="s">
+        <v>347</v>
       </c>
       <c r="AA327">
         <v>0</v>
       </c>
       <c r="AB327" t="s">
-        <v>210</v>
+        <v>461</v>
       </c>
       <c r="AG327" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="AH327" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="328" spans="1:34">
       <c r="A328">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B328" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C328" t="s">
         <v>54</v>
@@ -24725,7 +24731,7 @@
         <v>55</v>
       </c>
       <c r="E328" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F328" t="s">
         <v>60</v>
@@ -24749,22 +24755,22 @@
         <v>205</v>
       </c>
       <c r="O328">
-        <v>17967989</v>
+        <v>17042389</v>
       </c>
       <c r="P328" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q328" t="s">
         <v>237</v>
       </c>
       <c r="R328" s="1">
-        <v>46234.66180127315</v>
+        <v>46245.76585582176</v>
       </c>
       <c r="S328">
         <v>4</v>
       </c>
       <c r="T328" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="V328" t="s">
         <v>253</v>
@@ -24782,15 +24788,15 @@
         <v>472</v>
       </c>
       <c r="AH328" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="329" spans="1:34">
       <c r="A329">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B329" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C329" t="s">
         <v>54</v>
@@ -24799,13 +24805,13 @@
         <v>55</v>
       </c>
       <c r="E329" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F329" t="s">
         <v>60</v>
       </c>
       <c r="G329">
-        <v>1652</v>
+        <v>11516</v>
       </c>
       <c r="H329">
         <v>0</v>
@@ -24814,57 +24820,54 @@
         <v>63</v>
       </c>
       <c r="J329" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L329" s="1">
         <v>46290</v>
       </c>
       <c r="N329" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="O329">
-        <v>17042389</v>
+        <v>17968053</v>
       </c>
       <c r="P329" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q329" t="s">
         <v>237</v>
       </c>
       <c r="R329" s="1">
-        <v>46245.76585582176</v>
+        <v>46290.564674375</v>
       </c>
       <c r="S329">
         <v>4</v>
       </c>
       <c r="T329" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="V329" t="s">
         <v>253</v>
       </c>
-      <c r="W329" t="s">
-        <v>349</v>
-      </c>
       <c r="AA329">
         <v>0</v>
       </c>
       <c r="AB329" t="s">
-        <v>461</v>
+        <v>207</v>
       </c>
       <c r="AG329" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AH329" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="330" spans="1:34">
       <c r="A330">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B330" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C330" t="s">
         <v>54</v>
@@ -24873,7 +24876,7 @@
         <v>55</v>
       </c>
       <c r="E330" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F330" t="s">
         <v>60</v>
@@ -24897,22 +24900,22 @@
         <v>202</v>
       </c>
       <c r="O330">
-        <v>17968053</v>
+        <v>17042662</v>
       </c>
       <c r="P330" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q330" t="s">
         <v>237</v>
       </c>
       <c r="R330" s="1">
-        <v>46290.564674375</v>
+        <v>46290.56113170139</v>
       </c>
       <c r="S330">
         <v>4</v>
       </c>
       <c r="T330" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="V330" t="s">
         <v>253</v>
@@ -24921,21 +24924,21 @@
         <v>0</v>
       </c>
       <c r="AB330" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AG330" t="s">
         <v>473</v>
       </c>
       <c r="AH330" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="331" spans="1:34">
       <c r="A331">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B331" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C331" t="s">
         <v>54</v>
@@ -24944,10 +24947,10 @@
         <v>55</v>
       </c>
       <c r="E331" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F331" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G331">
         <v>11516</v>
@@ -24968,51 +24971,48 @@
         <v>202</v>
       </c>
       <c r="O331">
-        <v>17042662</v>
+        <v>18178314</v>
       </c>
       <c r="P331" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q331" t="s">
         <v>237</v>
       </c>
       <c r="R331" s="1">
-        <v>46290.56113170139</v>
+        <v>46290.56957094908</v>
       </c>
       <c r="S331">
         <v>4</v>
       </c>
       <c r="T331" t="s">
-        <v>241</v>
-      </c>
-      <c r="V331" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="AA331">
         <v>0</v>
       </c>
       <c r="AB331" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AG331" t="s">
         <v>473</v>
       </c>
       <c r="AH331" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="332" spans="1:34">
       <c r="A332">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B332" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C332" t="s">
         <v>54</v>
       </c>
       <c r="D332" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E332" t="s">
         <v>58</v>
@@ -25039,42 +25039,42 @@
         <v>202</v>
       </c>
       <c r="O332">
-        <v>18178314</v>
+        <v>18187985</v>
       </c>
       <c r="P332" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Q332" t="s">
         <v>237</v>
       </c>
       <c r="R332" s="1">
-        <v>46290.56957094908</v>
+        <v>46290.40572291666</v>
       </c>
       <c r="S332">
         <v>4</v>
       </c>
       <c r="T332" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AA332">
         <v>0</v>
       </c>
       <c r="AB332" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AG332" t="s">
         <v>473</v>
       </c>
       <c r="AH332" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="333" spans="1:34">
       <c r="A333">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B333" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C333" t="s">
         <v>54</v>
@@ -25107,7 +25107,7 @@
         <v>202</v>
       </c>
       <c r="O333">
-        <v>18187985</v>
+        <v>18241255</v>
       </c>
       <c r="P333" t="s">
         <v>210</v>
@@ -25116,7 +25116,7 @@
         <v>237</v>
       </c>
       <c r="R333" s="1">
-        <v>46290.40572291666</v>
+        <v>46290.40597356481</v>
       </c>
       <c r="S333">
         <v>4</v>
@@ -25139,10 +25139,10 @@
     </row>
     <row r="334" spans="1:34">
       <c r="A334">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B334" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C334" t="s">
         <v>54</v>
@@ -25157,7 +25157,7 @@
         <v>61</v>
       </c>
       <c r="G334">
-        <v>11516</v>
+        <v>10992</v>
       </c>
       <c r="H334">
         <v>0</v>
@@ -25166,16 +25166,16 @@
         <v>63</v>
       </c>
       <c r="J334" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="L334" s="1">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="N334" t="s">
         <v>202</v>
       </c>
       <c r="O334">
-        <v>18241255</v>
+        <v>18249084</v>
       </c>
       <c r="P334" t="s">
         <v>210</v>
@@ -25184,14 +25184,17 @@
         <v>237</v>
       </c>
       <c r="R334" s="1">
-        <v>46290.40597356481</v>
+        <v>46293.54930709491</v>
       </c>
       <c r="S334">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="T334" t="s">
         <v>244</v>
       </c>
+      <c r="W334" t="s">
+        <v>349</v>
+      </c>
       <c r="AA334">
         <v>0</v>
       </c>
@@ -25199,7 +25202,7 @@
         <v>210</v>
       </c>
       <c r="AG334" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AH334" t="s">
         <v>474</v>
@@ -25207,10 +25210,10 @@
     </row>
     <row r="335" spans="1:34">
       <c r="A335">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B335" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C335" t="s">
         <v>54</v>
@@ -25243,7 +25246,7 @@
         <v>202</v>
       </c>
       <c r="O335">
-        <v>18249084</v>
+        <v>18249092</v>
       </c>
       <c r="P335" t="s">
         <v>210</v>
@@ -25252,7 +25255,7 @@
         <v>237</v>
       </c>
       <c r="R335" s="1">
-        <v>46293.54930709491</v>
+        <v>46293.5514684838</v>
       </c>
       <c r="S335">
         <v>-1</v>
@@ -25261,7 +25264,7 @@
         <v>244</v>
       </c>
       <c r="W335" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AA335">
         <v>0</v>
@@ -25278,10 +25281,10 @@
     </row>
     <row r="336" spans="1:34">
       <c r="A336">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B336" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C336" t="s">
         <v>54</v>
@@ -25296,7 +25299,7 @@
         <v>61</v>
       </c>
       <c r="G336">
-        <v>10992</v>
+        <v>7875</v>
       </c>
       <c r="H336">
         <v>0</v>
@@ -25305,7 +25308,7 @@
         <v>63</v>
       </c>
       <c r="J336" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L336" s="1">
         <v>46295</v>
@@ -25314,7 +25317,7 @@
         <v>202</v>
       </c>
       <c r="O336">
-        <v>18249092</v>
+        <v>18200037</v>
       </c>
       <c r="P336" t="s">
         <v>210</v>
@@ -25323,7 +25326,7 @@
         <v>237</v>
       </c>
       <c r="R336" s="1">
-        <v>46293.5514684838</v>
+        <v>46293.54923961806</v>
       </c>
       <c r="S336">
         <v>-1</v>
@@ -25338,7 +25341,7 @@
         <v>0</v>
       </c>
       <c r="AB336" t="s">
-        <v>210</v>
+        <v>461</v>
       </c>
       <c r="AG336" t="s">
         <v>471</v>
@@ -25349,10 +25352,10 @@
     </row>
     <row r="337" spans="1:34">
       <c r="A337">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B337" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C337" t="s">
         <v>54</v>
@@ -25385,7 +25388,7 @@
         <v>202</v>
       </c>
       <c r="O337">
-        <v>18200037</v>
+        <v>18200056</v>
       </c>
       <c r="P337" t="s">
         <v>210</v>
@@ -25394,7 +25397,7 @@
         <v>237</v>
       </c>
       <c r="R337" s="1">
-        <v>46293.54923961806</v>
+        <v>46293.5514659375</v>
       </c>
       <c r="S337">
         <v>-1</v>
@@ -25420,16 +25423,16 @@
     </row>
     <row r="338" spans="1:34">
       <c r="A338">
-        <v>6963</v>
+        <v>6945</v>
       </c>
       <c r="B338" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C338" t="s">
         <v>54</v>
       </c>
       <c r="D338" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E338" t="s">
         <v>58</v>
@@ -25438,7 +25441,7 @@
         <v>61</v>
       </c>
       <c r="G338">
-        <v>7875</v>
+        <v>9764</v>
       </c>
       <c r="H338">
         <v>0</v>
@@ -25447,7 +25450,7 @@
         <v>63</v>
       </c>
       <c r="J338" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L338" s="1">
         <v>46295</v>
@@ -25456,22 +25459,22 @@
         <v>202</v>
       </c>
       <c r="O338">
-        <v>18200056</v>
+        <v>18200045</v>
       </c>
       <c r="P338" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Q338" t="s">
         <v>237</v>
       </c>
       <c r="R338" s="1">
-        <v>46293.5514659375</v>
+        <v>46288.43167056713</v>
       </c>
       <c r="S338">
         <v>-1</v>
       </c>
       <c r="T338" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="W338" t="s">
         <v>352</v>
@@ -25491,81 +25494,81 @@
     </row>
     <row r="339" spans="1:34">
       <c r="A339">
-        <v>6945</v>
+        <v>6548</v>
       </c>
       <c r="B339" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C339" t="s">
         <v>54</v>
       </c>
       <c r="D339" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E339" t="s">
         <v>58</v>
       </c>
       <c r="F339" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G339">
-        <v>9764</v>
+        <v>1697</v>
       </c>
       <c r="H339">
-        <v>0</v>
+        <v>1650</v>
       </c>
       <c r="I339" t="s">
         <v>63</v>
       </c>
       <c r="J339" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="L339" s="1">
-        <v>46295</v>
+        <v>46286</v>
       </c>
       <c r="N339" t="s">
         <v>202</v>
       </c>
       <c r="O339">
-        <v>18200045</v>
+        <v>17968001</v>
       </c>
       <c r="P339" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Q339" t="s">
         <v>237</v>
       </c>
       <c r="R339" s="1">
-        <v>46288.43167056713</v>
+        <v>46282.62254486111</v>
       </c>
       <c r="S339">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T339" t="s">
-        <v>242</v>
-      </c>
-      <c r="W339" t="s">
-        <v>353</v>
+        <v>240</v>
+      </c>
+      <c r="V339" t="s">
+        <v>253</v>
       </c>
       <c r="AA339">
         <v>0</v>
       </c>
       <c r="AB339" t="s">
-        <v>461</v>
+        <v>207</v>
       </c>
       <c r="AG339" t="s">
         <v>471</v>
       </c>
       <c r="AH339" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="340" spans="1:34">
       <c r="A340">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B340" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C340" t="s">
         <v>54</v>
@@ -25574,7 +25577,7 @@
         <v>55</v>
       </c>
       <c r="E340" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F340" t="s">
         <v>60</v>
@@ -25594,49 +25597,55 @@
       <c r="L340" s="1">
         <v>46286</v>
       </c>
+      <c r="M340" t="s">
+        <v>192</v>
+      </c>
       <c r="N340" t="s">
         <v>202</v>
       </c>
       <c r="O340">
-        <v>17968001</v>
+        <v>17042403</v>
       </c>
       <c r="P340" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q340" t="s">
         <v>237</v>
       </c>
       <c r="R340" s="1">
-        <v>46282.62254486111</v>
+        <v>46286.64173940972</v>
       </c>
       <c r="S340">
         <v>8</v>
       </c>
       <c r="T340" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="V340" t="s">
         <v>253</v>
       </c>
+      <c r="W340" t="s">
+        <v>353</v>
+      </c>
       <c r="AA340">
         <v>0</v>
       </c>
       <c r="AB340" t="s">
-        <v>207</v>
+        <v>467</v>
       </c>
       <c r="AG340" t="s">
         <v>471</v>
       </c>
       <c r="AH340" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="341" spans="1:34">
       <c r="A341">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B341" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C341" t="s">
         <v>54</v>
@@ -25645,10 +25654,10 @@
         <v>55</v>
       </c>
       <c r="E341" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F341" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G341">
         <v>1697</v>
@@ -25665,55 +25674,46 @@
       <c r="L341" s="1">
         <v>46286</v>
       </c>
-      <c r="M341" t="s">
-        <v>192</v>
-      </c>
       <c r="N341" t="s">
         <v>202</v>
       </c>
       <c r="O341">
-        <v>17042403</v>
+        <v>18178280</v>
       </c>
       <c r="P341" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q341" t="s">
         <v>237</v>
       </c>
       <c r="R341" s="1">
-        <v>46286.64173940972</v>
+        <v>46283.44840582176</v>
       </c>
       <c r="S341">
         <v>8</v>
       </c>
       <c r="T341" t="s">
-        <v>241</v>
-      </c>
-      <c r="V341" t="s">
-        <v>253</v>
-      </c>
-      <c r="W341" t="s">
-        <v>354</v>
+        <v>243</v>
       </c>
       <c r="AA341">
         <v>0</v>
       </c>
       <c r="AB341" t="s">
-        <v>467</v>
+        <v>207</v>
       </c>
       <c r="AG341" t="s">
         <v>471</v>
       </c>
       <c r="AH341" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="342" spans="1:34">
       <c r="A342">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B342" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C342" t="s">
         <v>54</v>
@@ -25725,63 +25725,63 @@
         <v>58</v>
       </c>
       <c r="F342" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G342">
-        <v>1697</v>
+        <v>7868</v>
       </c>
       <c r="H342">
-        <v>1650</v>
+        <v>0</v>
       </c>
       <c r="I342" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J342" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="L342" s="1">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="N342" t="s">
         <v>202</v>
       </c>
       <c r="O342">
-        <v>18178280</v>
+        <v>17399310</v>
       </c>
       <c r="P342" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="Q342" t="s">
         <v>237</v>
       </c>
       <c r="R342" s="1">
-        <v>46283.44840582176</v>
+        <v>46293.61969709491</v>
       </c>
       <c r="S342">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="T342" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AA342">
         <v>0</v>
       </c>
       <c r="AB342" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="AG342" t="s">
         <v>471</v>
       </c>
       <c r="AH342" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="343" spans="1:34">
       <c r="A343">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B343" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C343" t="s">
         <v>54</v>
@@ -25814,28 +25814,31 @@
         <v>202</v>
       </c>
       <c r="O343">
-        <v>17399310</v>
+        <v>18114218</v>
       </c>
       <c r="P343" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="Q343" t="s">
         <v>237</v>
       </c>
       <c r="R343" s="1">
-        <v>46293.61969709491</v>
+        <v>46293.61789920139</v>
       </c>
       <c r="S343">
         <v>1</v>
       </c>
       <c r="T343" t="s">
-        <v>245</v>
+        <v>247</v>
+      </c>
+      <c r="V343" t="s">
+        <v>253</v>
       </c>
       <c r="AA343">
         <v>0</v>
       </c>
       <c r="AB343" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="AG343" t="s">
         <v>471</v>
@@ -25846,10 +25849,10 @@
     </row>
     <row r="344" spans="1:34">
       <c r="A344">
-        <v>6486</v>
+        <v>6704</v>
       </c>
       <c r="B344" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C344" t="s">
         <v>54</v>
@@ -25882,22 +25885,22 @@
         <v>202</v>
       </c>
       <c r="O344">
-        <v>18114218</v>
+        <v>17955421</v>
       </c>
       <c r="P344" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="Q344" t="s">
         <v>237</v>
       </c>
       <c r="R344" s="1">
-        <v>46293.61789920139</v>
+        <v>46267.47365627315</v>
       </c>
       <c r="S344">
         <v>1</v>
       </c>
       <c r="T344" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="V344" t="s">
         <v>253</v>
@@ -25906,21 +25909,21 @@
         <v>0</v>
       </c>
       <c r="AB344" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="AG344" t="s">
         <v>471</v>
       </c>
       <c r="AH344" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="345" spans="1:34">
       <c r="A345">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B345" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C345" t="s">
         <v>54</v>
@@ -25935,7 +25938,7 @@
         <v>60</v>
       </c>
       <c r="G345">
-        <v>7868</v>
+        <v>6890</v>
       </c>
       <c r="H345">
         <v>0</v>
@@ -25944,60 +25947,63 @@
         <v>64</v>
       </c>
       <c r="J345" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="L345" s="1">
-        <v>46293</v>
+        <v>46290</v>
+      </c>
+      <c r="M345" t="s">
+        <v>193</v>
       </c>
       <c r="N345" t="s">
         <v>202</v>
       </c>
       <c r="O345">
-        <v>17955421</v>
+        <v>17399260</v>
       </c>
       <c r="P345" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q345" t="s">
         <v>237</v>
       </c>
       <c r="R345" s="1">
-        <v>46267.47365627315</v>
+        <v>46287.48052434028</v>
       </c>
       <c r="S345">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T345" t="s">
-        <v>246</v>
-      </c>
-      <c r="V345" t="s">
-        <v>253</v>
+        <v>245</v>
+      </c>
+      <c r="W345" t="s">
+        <v>354</v>
       </c>
       <c r="AA345">
         <v>0</v>
       </c>
       <c r="AB345" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AG345" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="AH345" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="346" spans="1:34">
       <c r="A346">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B346" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C346" t="s">
         <v>54</v>
       </c>
       <c r="D346" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E346" t="s">
         <v>58</v>
@@ -26027,51 +26033,51 @@
         <v>202</v>
       </c>
       <c r="O346">
-        <v>17399260</v>
+        <v>16962328</v>
       </c>
       <c r="P346" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="Q346" t="s">
         <v>237</v>
       </c>
       <c r="R346" s="1">
-        <v>46287.48052434028</v>
+        <v>46289.41381568287</v>
       </c>
       <c r="S346">
         <v>4</v>
       </c>
       <c r="T346" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="W346" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AA346">
         <v>0</v>
       </c>
       <c r="AB346" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="AG346" t="s">
         <v>473</v>
       </c>
       <c r="AH346" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="347" spans="1:34">
       <c r="A347">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B347" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C347" t="s">
         <v>54</v>
       </c>
       <c r="D347" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E347" t="s">
         <v>58</v>
@@ -26094,58 +26100,55 @@
       <c r="L347" s="1">
         <v>46290</v>
       </c>
-      <c r="M347" t="s">
-        <v>193</v>
-      </c>
       <c r="N347" t="s">
         <v>202</v>
       </c>
       <c r="O347">
-        <v>16962328</v>
+        <v>18152538</v>
       </c>
       <c r="P347" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q347" t="s">
         <v>237</v>
       </c>
       <c r="R347" s="1">
-        <v>46289.41381568287</v>
+        <v>46289.44878592592</v>
       </c>
       <c r="S347">
         <v>4</v>
       </c>
       <c r="T347" t="s">
-        <v>249</v>
-      </c>
-      <c r="W347" t="s">
-        <v>355</v>
+        <v>247</v>
+      </c>
+      <c r="V347" t="s">
+        <v>253</v>
       </c>
       <c r="AA347">
         <v>0</v>
       </c>
       <c r="AB347" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AG347" t="s">
         <v>473</v>
       </c>
       <c r="AH347" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="348" spans="1:34">
       <c r="A348">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B348" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C348" t="s">
         <v>54</v>
       </c>
       <c r="D348" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E348" t="s">
         <v>58</v>
@@ -26172,7 +26175,7 @@
         <v>202</v>
       </c>
       <c r="O348">
-        <v>18152538</v>
+        <v>17955186</v>
       </c>
       <c r="P348" t="s">
         <v>230</v>
@@ -26181,16 +26184,13 @@
         <v>237</v>
       </c>
       <c r="R348" s="1">
-        <v>46289.44878592592</v>
+        <v>46289.44878644676</v>
       </c>
       <c r="S348">
         <v>4</v>
       </c>
       <c r="T348" t="s">
-        <v>247</v>
-      </c>
-      <c r="V348" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="AA348">
         <v>0</v>
@@ -26207,16 +26207,16 @@
     </row>
     <row r="349" spans="1:34">
       <c r="A349">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B349" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C349" t="s">
         <v>54</v>
       </c>
       <c r="D349" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E349" t="s">
         <v>58</v>
@@ -26243,48 +26243,51 @@
         <v>202</v>
       </c>
       <c r="O349">
-        <v>17955186</v>
+        <v>17955399</v>
       </c>
       <c r="P349" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="Q349" t="s">
         <v>237</v>
       </c>
       <c r="R349" s="1">
-        <v>46289.44878644676</v>
+        <v>46290.67269146991</v>
       </c>
       <c r="S349">
         <v>4</v>
       </c>
       <c r="T349" t="s">
-        <v>248</v>
+        <v>246</v>
+      </c>
+      <c r="V349" t="s">
+        <v>253</v>
       </c>
       <c r="AA349">
         <v>0</v>
       </c>
       <c r="AB349" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="AG349" t="s">
         <v>473</v>
       </c>
       <c r="AH349" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="350" spans="1:34">
       <c r="A350">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B350" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C350" t="s">
         <v>54</v>
       </c>
       <c r="D350" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E350" t="s">
         <v>58</v>
@@ -26311,7 +26314,7 @@
         <v>202</v>
       </c>
       <c r="O350">
-        <v>17955399</v>
+        <v>17955249</v>
       </c>
       <c r="P350" t="s">
         <v>212</v>
@@ -26320,7 +26323,7 @@
         <v>237</v>
       </c>
       <c r="R350" s="1">
-        <v>46290.67269146991</v>
+        <v>46289.64049288195</v>
       </c>
       <c r="S350">
         <v>4</v>
@@ -26328,14 +26331,11 @@
       <c r="T350" t="s">
         <v>246</v>
       </c>
-      <c r="V350" t="s">
-        <v>253</v>
-      </c>
       <c r="AA350">
         <v>0</v>
       </c>
       <c r="AB350" t="s">
-        <v>212</v>
+        <v>461</v>
       </c>
       <c r="AG350" t="s">
         <v>473</v>
@@ -26346,10 +26346,10 @@
     </row>
     <row r="351" spans="1:34">
       <c r="A351">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B351" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C351" t="s">
         <v>54</v>
@@ -26382,7 +26382,7 @@
         <v>202</v>
       </c>
       <c r="O351">
-        <v>17955249</v>
+        <v>18056769</v>
       </c>
       <c r="P351" t="s">
         <v>212</v>
@@ -26391,7 +26391,7 @@
         <v>237</v>
       </c>
       <c r="R351" s="1">
-        <v>46289.64049288195</v>
+        <v>46289.64073386574</v>
       </c>
       <c r="S351">
         <v>4</v>
@@ -26399,6 +26399,9 @@
       <c r="T351" t="s">
         <v>246</v>
       </c>
+      <c r="V351" t="s">
+        <v>253</v>
+      </c>
       <c r="AA351">
         <v>0</v>
       </c>
@@ -26414,16 +26417,16 @@
     </row>
     <row r="352" spans="1:34">
       <c r="A352">
-        <v>6779</v>
+        <v>5417</v>
       </c>
       <c r="B352" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C352" t="s">
         <v>54</v>
       </c>
       <c r="D352" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E352" t="s">
         <v>58</v>
@@ -26432,7 +26435,7 @@
         <v>60</v>
       </c>
       <c r="G352">
-        <v>6890</v>
+        <v>11276</v>
       </c>
       <c r="H352">
         <v>0</v>
@@ -26441,54 +26444,51 @@
         <v>64</v>
       </c>
       <c r="J352" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="L352" s="1">
-        <v>46290</v>
+        <v>46283</v>
       </c>
       <c r="N352" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="O352">
-        <v>18056769</v>
+        <v>17399423</v>
       </c>
       <c r="P352" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q352" t="s">
         <v>237</v>
       </c>
       <c r="R352" s="1">
-        <v>46289.64073386574</v>
+        <v>46266.47620831019</v>
       </c>
       <c r="S352">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="T352" t="s">
-        <v>246</v>
-      </c>
-      <c r="V352" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="AA352">
         <v>0</v>
       </c>
       <c r="AB352" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="AG352" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AH352" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="353" spans="1:34">
       <c r="A353">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B353" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C353" t="s">
         <v>54</v>
@@ -26521,28 +26521,31 @@
         <v>204</v>
       </c>
       <c r="O353">
-        <v>17399423</v>
+        <v>18152557</v>
       </c>
       <c r="P353" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="Q353" t="s">
         <v>237</v>
       </c>
       <c r="R353" s="1">
-        <v>46266.47620831019</v>
+        <v>46267.57586420139</v>
       </c>
       <c r="S353">
         <v>11</v>
       </c>
       <c r="T353" t="s">
-        <v>245</v>
+        <v>247</v>
+      </c>
+      <c r="V353" t="s">
+        <v>253</v>
       </c>
       <c r="AA353">
         <v>0</v>
       </c>
       <c r="AB353" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="AG353" t="s">
         <v>471</v>
@@ -26553,10 +26556,10 @@
     </row>
     <row r="354" spans="1:34">
       <c r="A354">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B354" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C354" t="s">
         <v>54</v>
@@ -26571,7 +26574,7 @@
         <v>60</v>
       </c>
       <c r="G354">
-        <v>11276</v>
+        <v>1583</v>
       </c>
       <c r="H354">
         <v>0</v>
@@ -26580,43 +26583,40 @@
         <v>64</v>
       </c>
       <c r="J354" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="L354" s="1">
-        <v>46283</v>
+        <v>46290</v>
       </c>
       <c r="N354" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="O354">
-        <v>18152557</v>
+        <v>17398917</v>
       </c>
       <c r="P354" t="s">
-        <v>230</v>
+        <v>211</v>
       </c>
       <c r="Q354" t="s">
         <v>237</v>
       </c>
       <c r="R354" s="1">
-        <v>46267.57586420139</v>
+        <v>46233.72355880787</v>
       </c>
       <c r="S354">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="T354" t="s">
-        <v>247</v>
-      </c>
-      <c r="V354" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="AA354">
         <v>0</v>
       </c>
       <c r="AB354" t="s">
-        <v>469</v>
+        <v>211</v>
       </c>
       <c r="AG354" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AH354" t="s">
         <v>469</v>
@@ -26624,10 +26624,10 @@
     </row>
     <row r="355" spans="1:34">
       <c r="A355">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B355" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C355" t="s">
         <v>54</v>
@@ -26660,42 +26660,36 @@
         <v>205</v>
       </c>
       <c r="O355">
-        <v>17398917</v>
-      </c>
-      <c r="P355" t="s">
-        <v>211</v>
+        <v>17407553</v>
       </c>
       <c r="Q355" t="s">
         <v>237</v>
       </c>
       <c r="R355" s="1">
-        <v>46233.72355880787</v>
+        <v>46261.36669849537</v>
       </c>
       <c r="S355">
         <v>4</v>
       </c>
       <c r="T355" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="AA355">
         <v>0</v>
       </c>
       <c r="AB355" t="s">
-        <v>211</v>
+        <v>461</v>
       </c>
       <c r="AG355" t="s">
         <v>472</v>
       </c>
-      <c r="AH355" t="s">
-        <v>469</v>
-      </c>
     </row>
     <row r="356" spans="1:34">
       <c r="A356">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B356" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C356" t="s">
         <v>54</v>
@@ -26707,7 +26701,7 @@
         <v>58</v>
       </c>
       <c r="F356" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G356">
         <v>1583</v>
@@ -26728,13 +26722,13 @@
         <v>205</v>
       </c>
       <c r="O356">
-        <v>17407553</v>
+        <v>17688645</v>
       </c>
       <c r="Q356" t="s">
         <v>237</v>
       </c>
       <c r="R356" s="1">
-        <v>46261.36669849537</v>
+        <v>46266.44156952546</v>
       </c>
       <c r="S356">
         <v>4</v>
@@ -26742,11 +26736,14 @@
       <c r="T356" t="s">
         <v>250</v>
       </c>
+      <c r="V356" t="s">
+        <v>253</v>
+      </c>
       <c r="AA356">
         <v>0</v>
       </c>
       <c r="AB356" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="AG356" t="s">
         <v>472</v>
@@ -26754,10 +26751,10 @@
     </row>
     <row r="357" spans="1:34">
       <c r="A357">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B357" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C357" t="s">
         <v>54</v>
@@ -26769,7 +26766,7 @@
         <v>58</v>
       </c>
       <c r="F357" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G357">
         <v>1583</v>
@@ -26790,28 +26787,31 @@
         <v>205</v>
       </c>
       <c r="O357">
-        <v>17688645</v>
+        <v>18166312</v>
       </c>
       <c r="Q357" t="s">
         <v>237</v>
       </c>
       <c r="R357" s="1">
-        <v>46266.44156952546</v>
+        <v>46233.50562820602</v>
       </c>
       <c r="S357">
         <v>4</v>
       </c>
       <c r="T357" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="V357" t="s">
         <v>253</v>
       </c>
+      <c r="W357" t="s">
+        <v>355</v>
+      </c>
       <c r="AA357">
         <v>0</v>
       </c>
       <c r="AB357" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="AG357" t="s">
         <v>472</v>
@@ -26819,10 +26819,10 @@
     </row>
     <row r="358" spans="1:34">
       <c r="A358">
-        <v>6278</v>
+        <v>6486</v>
       </c>
       <c r="B358" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C358" t="s">
         <v>54</v>
@@ -26855,42 +26855,45 @@
         <v>205</v>
       </c>
       <c r="O358">
-        <v>18166312</v>
+        <v>18114208</v>
+      </c>
+      <c r="P358" t="s">
+        <v>230</v>
       </c>
       <c r="Q358" t="s">
         <v>237</v>
       </c>
       <c r="R358" s="1">
-        <v>46233.50562820602</v>
+        <v>46233.80164280093</v>
       </c>
       <c r="S358">
         <v>4</v>
       </c>
       <c r="T358" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="V358" t="s">
         <v>253</v>
       </c>
-      <c r="W358" t="s">
-        <v>356</v>
-      </c>
       <c r="AA358">
         <v>0</v>
       </c>
       <c r="AB358" t="s">
-        <v>461</v>
+        <v>230</v>
       </c>
       <c r="AG358" t="s">
         <v>472</v>
       </c>
+      <c r="AH358" t="s">
+        <v>469</v>
+      </c>
     </row>
     <row r="359" spans="1:34">
       <c r="A359">
-        <v>6486</v>
+        <v>6704</v>
       </c>
       <c r="B359" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C359" t="s">
         <v>54</v>
@@ -26923,22 +26926,22 @@
         <v>205</v>
       </c>
       <c r="O359">
-        <v>18114208</v>
+        <v>17955373</v>
       </c>
       <c r="P359" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="Q359" t="s">
         <v>237</v>
       </c>
       <c r="R359" s="1">
-        <v>46233.80164280093</v>
+        <v>46232.72913953703</v>
       </c>
       <c r="S359">
         <v>4</v>
       </c>
       <c r="T359" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="V359" t="s">
         <v>253</v>
@@ -26947,21 +26950,21 @@
         <v>0</v>
       </c>
       <c r="AB359" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="AG359" t="s">
         <v>472</v>
       </c>
       <c r="AH359" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="360" spans="1:34">
       <c r="A360">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B360" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C360" t="s">
         <v>54</v>
@@ -26976,7 +26979,7 @@
         <v>60</v>
       </c>
       <c r="G360">
-        <v>1583</v>
+        <v>11514</v>
       </c>
       <c r="H360">
         <v>0</v>
@@ -26985,60 +26988,63 @@
         <v>64</v>
       </c>
       <c r="J360" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L360" s="1">
         <v>46290</v>
       </c>
+      <c r="M360" t="s">
+        <v>193</v>
+      </c>
       <c r="N360" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="O360">
-        <v>17955373</v>
+        <v>17399465</v>
       </c>
       <c r="P360" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q360" t="s">
         <v>237</v>
       </c>
       <c r="R360" s="1">
-        <v>46232.72913953703</v>
+        <v>46287.48083141204</v>
       </c>
       <c r="S360">
         <v>4</v>
       </c>
       <c r="T360" t="s">
-        <v>246</v>
-      </c>
-      <c r="V360" t="s">
-        <v>253</v>
+        <v>245</v>
+      </c>
+      <c r="W360" t="s">
+        <v>354</v>
       </c>
       <c r="AA360">
         <v>0</v>
       </c>
       <c r="AB360" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AG360" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AH360" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="361" spans="1:34">
       <c r="A361">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B361" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C361" t="s">
         <v>54</v>
       </c>
       <c r="D361" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E361" t="s">
         <v>58</v>
@@ -27068,51 +27074,51 @@
         <v>202</v>
       </c>
       <c r="O361">
-        <v>17399465</v>
+        <v>16962474</v>
       </c>
       <c r="P361" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="Q361" t="s">
         <v>237</v>
       </c>
       <c r="R361" s="1">
-        <v>46287.48083141204</v>
+        <v>46289.40860091435</v>
       </c>
       <c r="S361">
         <v>4</v>
       </c>
       <c r="T361" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="W361" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AA361">
         <v>0</v>
       </c>
       <c r="AB361" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="AG361" t="s">
         <v>473</v>
       </c>
       <c r="AH361" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="362" spans="1:34">
       <c r="A362">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B362" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C362" t="s">
         <v>54</v>
       </c>
       <c r="D362" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E362" t="s">
         <v>58</v>
@@ -27135,58 +27141,55 @@
       <c r="L362" s="1">
         <v>46290</v>
       </c>
-      <c r="M362" t="s">
-        <v>193</v>
-      </c>
       <c r="N362" t="s">
         <v>202</v>
       </c>
       <c r="O362">
-        <v>16962474</v>
+        <v>18114227</v>
       </c>
       <c r="P362" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q362" t="s">
         <v>237</v>
       </c>
       <c r="R362" s="1">
-        <v>46289.40860091435</v>
+        <v>46289.44826453704</v>
       </c>
       <c r="S362">
         <v>4</v>
       </c>
       <c r="T362" t="s">
-        <v>249</v>
-      </c>
-      <c r="W362" t="s">
-        <v>355</v>
+        <v>247</v>
+      </c>
+      <c r="V362" t="s">
+        <v>253</v>
       </c>
       <c r="AA362">
         <v>0</v>
       </c>
       <c r="AB362" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AG362" t="s">
         <v>473</v>
       </c>
       <c r="AH362" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="363" spans="1:34">
       <c r="A363">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B363" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C363" t="s">
         <v>54</v>
       </c>
       <c r="D363" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E363" t="s">
         <v>58</v>
@@ -27213,7 +27216,7 @@
         <v>202</v>
       </c>
       <c r="O363">
-        <v>18114227</v>
+        <v>17955212</v>
       </c>
       <c r="P363" t="s">
         <v>230</v>
@@ -27222,16 +27225,13 @@
         <v>237</v>
       </c>
       <c r="R363" s="1">
-        <v>46289.44826453704</v>
+        <v>46289.4482663426</v>
       </c>
       <c r="S363">
         <v>4</v>
       </c>
       <c r="T363" t="s">
-        <v>247</v>
-      </c>
-      <c r="V363" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="AA363">
         <v>0</v>
@@ -27248,16 +27248,16 @@
     </row>
     <row r="364" spans="1:34">
       <c r="A364">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B364" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C364" t="s">
         <v>54</v>
       </c>
       <c r="D364" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E364" t="s">
         <v>58</v>
@@ -27284,48 +27284,51 @@
         <v>202</v>
       </c>
       <c r="O364">
-        <v>17955212</v>
+        <v>17955445</v>
       </c>
       <c r="P364" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="Q364" t="s">
         <v>237</v>
       </c>
       <c r="R364" s="1">
-        <v>46289.4482663426</v>
+        <v>46290.67373011574</v>
       </c>
       <c r="S364">
         <v>4</v>
       </c>
       <c r="T364" t="s">
-        <v>248</v>
+        <v>246</v>
+      </c>
+      <c r="V364" t="s">
+        <v>253</v>
       </c>
       <c r="AA364">
         <v>0</v>
       </c>
       <c r="AB364" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="AG364" t="s">
         <v>473</v>
       </c>
       <c r="AH364" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="365" spans="1:34">
       <c r="A365">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B365" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C365" t="s">
         <v>54</v>
       </c>
       <c r="D365" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E365" t="s">
         <v>58</v>
@@ -27334,7 +27337,7 @@
         <v>60</v>
       </c>
       <c r="G365">
-        <v>11514</v>
+        <v>10988</v>
       </c>
       <c r="H365">
         <v>0</v>
@@ -27343,46 +27346,46 @@
         <v>64</v>
       </c>
       <c r="J365" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="L365" s="1">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="N365" t="s">
         <v>202</v>
       </c>
       <c r="O365">
-        <v>17955445</v>
+        <v>18112918</v>
       </c>
       <c r="P365" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="Q365" t="s">
         <v>237</v>
       </c>
       <c r="R365" s="1">
-        <v>46290.67373011574</v>
+        <v>46294.58957913194</v>
       </c>
       <c r="S365">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="T365" t="s">
-        <v>246</v>
-      </c>
-      <c r="V365" t="s">
-        <v>253</v>
+        <v>248</v>
+      </c>
+      <c r="W365" t="s">
+        <v>356</v>
       </c>
       <c r="AA365">
         <v>0</v>
       </c>
       <c r="AB365" t="s">
-        <v>212</v>
+        <v>461</v>
       </c>
       <c r="AG365" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AH365" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="366" spans="1:34">
@@ -33131,7 +33134,7 @@
         <v>253</v>
       </c>
       <c r="W445" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AA445">
         <v>0</v>
@@ -33205,7 +33208,7 @@
         <v>243</v>
       </c>
       <c r="W446" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AA446">
         <v>0</v>
@@ -34581,7 +34584,7 @@
         <v>243</v>
       </c>
       <c r="W465" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AA465">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-29 18:45
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -583,40 +583,40 @@
     <t>15/09/2026</t>
   </si>
   <si>
+    <t>30/09/2026</t>
+  </si>
+  <si>
+    <t>02/10/2026</t>
+  </si>
+  <si>
+    <t>28/09/2026</t>
+  </si>
+  <si>
+    <t>21/09/2026</t>
+  </si>
+  <si>
+    <t>25/09/2026</t>
+  </si>
+  <si>
+    <t>16/09/2026</t>
+  </si>
+  <si>
+    <t>18/09/2026</t>
+  </si>
+  <si>
+    <t>17/09/2026</t>
+  </si>
+  <si>
+    <t>22/09/2026</t>
+  </si>
+  <si>
+    <t>23/09/2026</t>
+  </si>
+  <si>
+    <t>24/09/2026</t>
+  </si>
+  <si>
     <t>29/09/2026</t>
-  </si>
-  <si>
-    <t>30/09/2026</t>
-  </si>
-  <si>
-    <t>28/09/2026</t>
-  </si>
-  <si>
-    <t>21/09/2026</t>
-  </si>
-  <si>
-    <t>25/09/2026</t>
-  </si>
-  <si>
-    <t>16/09/2026</t>
-  </si>
-  <si>
-    <t>18/09/2026</t>
-  </si>
-  <si>
-    <t>17/09/2026</t>
-  </si>
-  <si>
-    <t>22/09/2026</t>
-  </si>
-  <si>
-    <t>23/09/2026</t>
-  </si>
-  <si>
-    <t>24/09/2026</t>
-  </si>
-  <si>
-    <t>02/10/2026</t>
   </si>
   <si>
     <t>09/10/2026</t>
@@ -1048,14 +1048,14 @@
 Reunião confirmada pelo cliente - Data Comentário: 04/09/2026 11:03</t>
   </si>
   <si>
-    <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 29/09/2026 - Data Comentário: 28/09/2026 16:40</t>
+    <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 30/09/2026 - Data Comentário: 29/09/2026 17:51</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/09/2026 
 Aguardando envio do cliente. - Data Comentário: 29/09/2026 10:31</t>
   </si>
   <si>
-    <t>Reaberto via API integração MGC x Analise Balanço em 24/09/2026 13:41:29. - Data Comentário: 28/09/2026 18:32</t>
+    <t>Reaberto via API integração MGC x Analise Balanço em 24/09/2026 13:41:29. - Data Comentário: 29/09/2026 18:31</t>
   </si>
   <si>
     <t>Atraso da Operação, processo em elaboração conforme data prevista   
@@ -22532,7 +22532,7 @@
         <v>46293</v>
       </c>
       <c r="M295" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N295" t="s">
         <v>203</v>
@@ -22603,7 +22603,7 @@
         <v>46290</v>
       </c>
       <c r="M296" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N296" t="s">
         <v>202</v>
@@ -22736,7 +22736,7 @@
         <v>46295</v>
       </c>
       <c r="M298" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N298" t="s">
         <v>202</v>
@@ -22934,7 +22934,7 @@
         <v>46295</v>
       </c>
       <c r="M301" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N301" t="s">
         <v>202</v>
@@ -24255,7 +24255,7 @@
         <v>46290</v>
       </c>
       <c r="M321" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N321" t="s">
         <v>202</v>
@@ -35528,7 +35528,7 @@
         <v>46293</v>
       </c>
       <c r="M478" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="N478" t="s">
         <v>205</v>
@@ -42324,7 +42324,7 @@
         <v>46287</v>
       </c>
       <c r="M573" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="N573" t="s">
         <v>202</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-30 14:42
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1058,9 +1058,6 @@
     <t>Reaberto via API integração MGC x Analise Balanço em 29/09/2026 20:27:46. - Data Comentário: 29/09/2026 20:26</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/09/2026 - Data Comentário: 28/09/2026 11:12</t>
-  </si>
-  <si>
     <t>Comentário Colaborador + Previsão de Conclusão. Previsto para: 28/09/2026 - Data Comentário: 18/09/2026 15:26</t>
   </si>
   <si>
@@ -1077,6 +1074,9 @@
   </si>
   <si>
     <t>Baixado via API integração MGC x Analise Balanço em 30/09/2026 09:46:04. - Data Comentário: 30/09/2026 09:41</t>
+  </si>
+  <si>
+    <t>Baixado via API integração MGC x Analise Balanço em 30/09/2026 14:10:10. - Data Comentário: 30/09/2026 14:05</t>
   </si>
   <si>
     <t>Baixado via API integração MGC x Analise Balanço em 30/09/2026 09:47:08. - Data Comentário: 30/09/2026 09:42</t>
@@ -22702,49 +22702,46 @@
     </row>
     <row r="298" spans="1:34">
       <c r="A298">
-        <v>6627</v>
+        <v>6404</v>
       </c>
       <c r="B298" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C298" t="s">
         <v>54</v>
       </c>
       <c r="D298" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E298" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F298" t="s">
         <v>60</v>
       </c>
       <c r="G298">
-        <v>7875</v>
+        <v>10988</v>
       </c>
       <c r="H298">
         <v>0</v>
       </c>
       <c r="I298" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J298" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="L298" s="1">
         <v>46295</v>
       </c>
-      <c r="M298" t="s">
-        <v>189</v>
-      </c>
       <c r="N298" t="s">
         <v>202</v>
       </c>
       <c r="O298">
-        <v>18096487</v>
+        <v>16962444</v>
       </c>
       <c r="P298" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="Q298" t="s">
         <v>237</v>
@@ -22753,13 +22750,7 @@
         <v>0</v>
       </c>
       <c r="T298" t="s">
-        <v>239</v>
-      </c>
-      <c r="V298" t="s">
-        <v>251</v>
-      </c>
-      <c r="W298" t="s">
-        <v>339</v>
+        <v>247</v>
       </c>
       <c r="AA298">
         <v>0</v>
@@ -22768,21 +22759,21 @@
         <v>469</v>
       </c>
       <c r="AH298" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="299" spans="1:34">
       <c r="A299">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B299" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C299" t="s">
         <v>54</v>
       </c>
       <c r="D299" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E299" t="s">
         <v>58</v>
@@ -22791,7 +22782,7 @@
         <v>60</v>
       </c>
       <c r="G299">
-        <v>10988</v>
+        <v>7874</v>
       </c>
       <c r="H299">
         <v>0</v>
@@ -22800,7 +22791,7 @@
         <v>64</v>
       </c>
       <c r="J299" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L299" s="1">
         <v>46295</v>
@@ -22809,10 +22800,10 @@
         <v>202</v>
       </c>
       <c r="O299">
-        <v>16962444</v>
+        <v>18096767</v>
       </c>
       <c r="P299" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="Q299" t="s">
         <v>237</v>
@@ -22821,7 +22812,10 @@
         <v>0</v>
       </c>
       <c r="T299" t="s">
-        <v>247</v>
+        <v>244</v>
+      </c>
+      <c r="V299" t="s">
+        <v>251</v>
       </c>
       <c r="AA299">
         <v>0</v>
@@ -22835,10 +22829,10 @@
     </row>
     <row r="300" spans="1:34">
       <c r="A300">
-        <v>6704</v>
+        <v>6627</v>
       </c>
       <c r="B300" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C300" t="s">
         <v>54</v>
@@ -22847,69 +22841,81 @@
         <v>55</v>
       </c>
       <c r="E300" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F300" t="s">
         <v>60</v>
       </c>
       <c r="G300">
-        <v>7874</v>
+        <v>7869</v>
       </c>
       <c r="H300">
         <v>0</v>
       </c>
       <c r="I300" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J300" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="L300" s="1">
-        <v>46295</v>
+        <v>46293</v>
+      </c>
+      <c r="M300" t="s">
+        <v>191</v>
       </c>
       <c r="N300" t="s">
         <v>202</v>
       </c>
       <c r="O300">
-        <v>18096767</v>
+        <v>17042546</v>
       </c>
       <c r="P300" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="Q300" t="s">
-        <v>237</v>
+        <v>235</v>
+      </c>
+      <c r="R300" s="1">
+        <v>46288.76065641204</v>
       </c>
       <c r="S300">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T300" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="V300" t="s">
         <v>251</v>
       </c>
+      <c r="W300" t="s">
+        <v>339</v>
+      </c>
       <c r="AA300">
         <v>0</v>
+      </c>
+      <c r="AB300" t="s">
+        <v>463</v>
       </c>
       <c r="AG300" t="s">
         <v>469</v>
       </c>
       <c r="AH300" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="301" spans="1:34">
       <c r="A301">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B301" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C301" t="s">
         <v>54</v>
       </c>
       <c r="D301" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E301" t="s">
         <v>59</v>
@@ -22939,7 +22945,7 @@
         <v>202</v>
       </c>
       <c r="O301">
-        <v>17042546</v>
+        <v>16960048</v>
       </c>
       <c r="P301" t="s">
         <v>208</v>
@@ -22948,7 +22954,7 @@
         <v>235</v>
       </c>
       <c r="R301" s="1">
-        <v>46288.76065641204</v>
+        <v>46288.7606568287</v>
       </c>
       <c r="S301">
         <v>2</v>
@@ -22960,7 +22966,7 @@
         <v>251</v>
       </c>
       <c r="W301" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AA301">
         <v>0</v>
@@ -22977,22 +22983,22 @@
     </row>
     <row r="302" spans="1:34">
       <c r="A302">
-        <v>6628</v>
+        <v>6949</v>
       </c>
       <c r="B302" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C302" t="s">
         <v>54</v>
       </c>
       <c r="D302" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E302" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F302" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G302">
         <v>7869</v>
@@ -23016,28 +23022,25 @@
         <v>202</v>
       </c>
       <c r="O302">
-        <v>16960048</v>
+        <v>18178300</v>
       </c>
       <c r="P302" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q302" t="s">
         <v>235</v>
       </c>
       <c r="R302" s="1">
-        <v>46288.7606568287</v>
+        <v>46288.76066791666</v>
       </c>
       <c r="S302">
         <v>2</v>
       </c>
       <c r="T302" t="s">
-        <v>239</v>
-      </c>
-      <c r="V302" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="W302" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AA302">
         <v>0</v>
@@ -23049,30 +23052,30 @@
         <v>469</v>
       </c>
       <c r="AH302" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="303" spans="1:34">
       <c r="A303">
-        <v>6949</v>
+        <v>6628</v>
       </c>
       <c r="B303" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C303" t="s">
         <v>54</v>
       </c>
       <c r="D303" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E303" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F303" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G303">
-        <v>7869</v>
+        <v>1650</v>
       </c>
       <c r="H303">
         <v>0</v>
@@ -23081,57 +23084,54 @@
         <v>63</v>
       </c>
       <c r="J303" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L303" s="1">
         <v>46293</v>
       </c>
-      <c r="M303" t="s">
-        <v>191</v>
-      </c>
       <c r="N303" t="s">
         <v>202</v>
       </c>
       <c r="O303">
-        <v>18178300</v>
+        <v>16959974</v>
       </c>
       <c r="P303" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q303" t="s">
         <v>235</v>
       </c>
       <c r="R303" s="1">
-        <v>46288.76066791666</v>
+        <v>46265.00248284722</v>
       </c>
       <c r="S303">
         <v>2</v>
       </c>
       <c r="T303" t="s">
-        <v>241</v>
-      </c>
-      <c r="W303" t="s">
-        <v>340</v>
+        <v>239</v>
+      </c>
+      <c r="V303" t="s">
+        <v>251</v>
       </c>
       <c r="AA303">
         <v>0</v>
       </c>
       <c r="AB303" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="AG303" t="s">
         <v>469</v>
       </c>
       <c r="AH303" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="304" spans="1:34">
       <c r="A304">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B304" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C304" t="s">
         <v>54</v>
@@ -23140,10 +23140,10 @@
         <v>56</v>
       </c>
       <c r="E304" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F304" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G304">
         <v>1650</v>
@@ -23164,25 +23164,22 @@
         <v>202</v>
       </c>
       <c r="O304">
-        <v>16959974</v>
+        <v>18163667</v>
       </c>
       <c r="P304" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q304" t="s">
         <v>235</v>
       </c>
       <c r="R304" s="1">
-        <v>46265.00248284722</v>
+        <v>46265.00255472222</v>
       </c>
       <c r="S304">
         <v>2</v>
       </c>
       <c r="T304" t="s">
-        <v>239</v>
-      </c>
-      <c r="V304" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="AA304">
         <v>0</v>
@@ -23199,25 +23196,25 @@
     </row>
     <row r="305" spans="1:34">
       <c r="A305">
-        <v>6945</v>
+        <v>6548</v>
       </c>
       <c r="B305" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C305" t="s">
         <v>54</v>
       </c>
       <c r="D305" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E305" t="s">
         <v>58</v>
       </c>
       <c r="F305" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G305">
-        <v>1650</v>
+        <v>6892</v>
       </c>
       <c r="H305">
         <v>0</v>
@@ -23226,51 +23223,54 @@
         <v>63</v>
       </c>
       <c r="J305" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L305" s="1">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="N305" t="s">
         <v>202</v>
       </c>
       <c r="O305">
-        <v>18163667</v>
+        <v>17968017</v>
       </c>
       <c r="P305" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Q305" t="s">
         <v>235</v>
       </c>
       <c r="R305" s="1">
-        <v>46265.00255472222</v>
+        <v>46290.56449253472</v>
       </c>
       <c r="S305">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T305" t="s">
-        <v>240</v>
+        <v>238</v>
+      </c>
+      <c r="V305" t="s">
+        <v>251</v>
       </c>
       <c r="AA305">
         <v>0</v>
       </c>
       <c r="AB305" t="s">
-        <v>458</v>
+        <v>207</v>
       </c>
       <c r="AG305" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="AH305" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="306" spans="1:34">
       <c r="A306">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B306" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C306" t="s">
         <v>54</v>
@@ -23279,7 +23279,7 @@
         <v>55</v>
       </c>
       <c r="E306" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F306" t="s">
         <v>60</v>
@@ -23303,22 +23303,22 @@
         <v>202</v>
       </c>
       <c r="O306">
-        <v>17968017</v>
+        <v>17042486</v>
       </c>
       <c r="P306" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q306" t="s">
         <v>235</v>
       </c>
       <c r="R306" s="1">
-        <v>46290.56449253472</v>
+        <v>46290.56093913194</v>
       </c>
       <c r="S306">
         <v>5</v>
       </c>
       <c r="T306" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="V306" t="s">
         <v>251</v>
@@ -23327,27 +23327,27 @@
         <v>0</v>
       </c>
       <c r="AB306" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AG306" t="s">
         <v>471</v>
       </c>
       <c r="AH306" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="307" spans="1:34">
       <c r="A307">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B307" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C307" t="s">
         <v>54</v>
       </c>
       <c r="D307" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E307" t="s">
         <v>59</v>
@@ -23374,7 +23374,7 @@
         <v>202</v>
       </c>
       <c r="O307">
-        <v>17042486</v>
+        <v>16960024</v>
       </c>
       <c r="P307" t="s">
         <v>208</v>
@@ -23383,7 +23383,7 @@
         <v>235</v>
       </c>
       <c r="R307" s="1">
-        <v>46290.56093913194</v>
+        <v>46289.64172979166</v>
       </c>
       <c r="S307">
         <v>5</v>
@@ -23398,7 +23398,7 @@
         <v>0</v>
       </c>
       <c r="AB307" t="s">
-        <v>208</v>
+        <v>458</v>
       </c>
       <c r="AG307" t="s">
         <v>471</v>
@@ -23409,10 +23409,10 @@
     </row>
     <row r="308" spans="1:34">
       <c r="A308">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B308" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C308" t="s">
         <v>54</v>
@@ -23421,10 +23421,10 @@
         <v>56</v>
       </c>
       <c r="E308" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F308" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G308">
         <v>6892</v>
@@ -23441,35 +23441,38 @@
       <c r="L308" s="1">
         <v>46290</v>
       </c>
+      <c r="M308" t="s">
+        <v>189</v>
+      </c>
       <c r="N308" t="s">
         <v>202</v>
       </c>
       <c r="O308">
-        <v>16960024</v>
+        <v>18163676</v>
       </c>
       <c r="P308" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q308" t="s">
         <v>235</v>
       </c>
       <c r="R308" s="1">
-        <v>46289.64172979166</v>
+        <v>46289.56480809028</v>
       </c>
       <c r="S308">
         <v>5</v>
       </c>
       <c r="T308" t="s">
-        <v>239</v>
-      </c>
-      <c r="V308" t="s">
-        <v>251</v>
+        <v>240</v>
+      </c>
+      <c r="W308" t="s">
+        <v>340</v>
       </c>
       <c r="AA308">
         <v>0</v>
       </c>
       <c r="AB308" t="s">
-        <v>458</v>
+        <v>209</v>
       </c>
       <c r="AG308" t="s">
         <v>471</v>
@@ -23480,16 +23483,16 @@
     </row>
     <row r="309" spans="1:34">
       <c r="A309">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B309" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C309" t="s">
         <v>54</v>
       </c>
       <c r="D309" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E309" t="s">
         <v>58</v>
@@ -23512,58 +23515,52 @@
       <c r="L309" s="1">
         <v>46290</v>
       </c>
-      <c r="M309" t="s">
-        <v>189</v>
-      </c>
       <c r="N309" t="s">
         <v>202</v>
       </c>
       <c r="O309">
-        <v>18163676</v>
+        <v>18178288</v>
       </c>
       <c r="P309" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Q309" t="s">
         <v>235</v>
       </c>
       <c r="R309" s="1">
-        <v>46289.56480809028</v>
+        <v>46290.56969825231</v>
       </c>
       <c r="S309">
         <v>5</v>
       </c>
       <c r="T309" t="s">
-        <v>240</v>
-      </c>
-      <c r="W309" t="s">
-        <v>341</v>
+        <v>241</v>
       </c>
       <c r="AA309">
         <v>0</v>
       </c>
       <c r="AB309" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="AG309" t="s">
         <v>471</v>
       </c>
       <c r="AH309" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="310" spans="1:34">
       <c r="A310">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B310" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C310" t="s">
         <v>54</v>
       </c>
       <c r="D310" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E310" t="s">
         <v>58</v>
@@ -23590,42 +23587,42 @@
         <v>202</v>
       </c>
       <c r="O310">
-        <v>18178288</v>
+        <v>18187955</v>
       </c>
       <c r="P310" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Q310" t="s">
         <v>235</v>
       </c>
       <c r="R310" s="1">
-        <v>46290.56969825231</v>
+        <v>46290.481633125</v>
       </c>
       <c r="S310">
         <v>5</v>
       </c>
       <c r="T310" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AA310">
         <v>0</v>
       </c>
       <c r="AB310" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AG310" t="s">
         <v>471</v>
       </c>
       <c r="AH310" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="311" spans="1:34">
       <c r="A311">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B311" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C311" t="s">
         <v>54</v>
@@ -23658,7 +23655,7 @@
         <v>202</v>
       </c>
       <c r="O311">
-        <v>18187955</v>
+        <v>18187893</v>
       </c>
       <c r="P311" t="s">
         <v>210</v>
@@ -23667,7 +23664,7 @@
         <v>235</v>
       </c>
       <c r="R311" s="1">
-        <v>46290.481633125</v>
+        <v>46290.48190942129</v>
       </c>
       <c r="S311">
         <v>5</v>
@@ -23690,25 +23687,25 @@
     </row>
     <row r="312" spans="1:34">
       <c r="A312">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B312" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C312" t="s">
         <v>54</v>
       </c>
       <c r="D312" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E312" t="s">
         <v>58</v>
       </c>
       <c r="F312" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G312">
-        <v>6892</v>
+        <v>1652</v>
       </c>
       <c r="H312">
         <v>0</v>
@@ -23717,51 +23714,57 @@
         <v>63</v>
       </c>
       <c r="J312" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L312" s="1">
         <v>46290</v>
       </c>
       <c r="N312" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="O312">
-        <v>18187893</v>
+        <v>17967989</v>
       </c>
       <c r="P312" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="Q312" t="s">
         <v>235</v>
       </c>
       <c r="R312" s="1">
-        <v>46290.48190942129</v>
+        <v>46234.66180127315</v>
       </c>
       <c r="S312">
         <v>5</v>
       </c>
       <c r="T312" t="s">
-        <v>242</v>
+        <v>238</v>
+      </c>
+      <c r="V312" t="s">
+        <v>251</v>
+      </c>
+      <c r="W312" t="s">
+        <v>341</v>
       </c>
       <c r="AA312">
         <v>0</v>
       </c>
       <c r="AB312" t="s">
-        <v>210</v>
+        <v>458</v>
       </c>
       <c r="AG312" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="AH312" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="313" spans="1:34">
       <c r="A313">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B313" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C313" t="s">
         <v>54</v>
@@ -23770,7 +23773,7 @@
         <v>55</v>
       </c>
       <c r="E313" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F313" t="s">
         <v>60</v>
@@ -23794,22 +23797,22 @@
         <v>204</v>
       </c>
       <c r="O313">
-        <v>17967989</v>
+        <v>17042389</v>
       </c>
       <c r="P313" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q313" t="s">
         <v>235</v>
       </c>
       <c r="R313" s="1">
-        <v>46234.66180127315</v>
+        <v>46245.76585582176</v>
       </c>
       <c r="S313">
         <v>5</v>
       </c>
       <c r="T313" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="V313" t="s">
         <v>251</v>
@@ -23827,15 +23830,15 @@
         <v>470</v>
       </c>
       <c r="AH313" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="314" spans="1:34">
       <c r="A314">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B314" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C314" t="s">
         <v>54</v>
@@ -23844,13 +23847,13 @@
         <v>55</v>
       </c>
       <c r="E314" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F314" t="s">
         <v>60</v>
       </c>
       <c r="G314">
-        <v>1652</v>
+        <v>11516</v>
       </c>
       <c r="H314">
         <v>0</v>
@@ -23859,57 +23862,54 @@
         <v>63</v>
       </c>
       <c r="J314" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L314" s="1">
         <v>46290</v>
       </c>
       <c r="N314" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="O314">
-        <v>17042389</v>
+        <v>17968053</v>
       </c>
       <c r="P314" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q314" t="s">
         <v>235</v>
       </c>
       <c r="R314" s="1">
-        <v>46245.76585582176</v>
+        <v>46290.564674375</v>
       </c>
       <c r="S314">
         <v>5</v>
       </c>
       <c r="T314" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V314" t="s">
         <v>251</v>
       </c>
-      <c r="W314" t="s">
-        <v>343</v>
-      </c>
       <c r="AA314">
         <v>0</v>
       </c>
       <c r="AB314" t="s">
-        <v>458</v>
+        <v>207</v>
       </c>
       <c r="AG314" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AH314" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="315" spans="1:34">
       <c r="A315">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B315" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C315" t="s">
         <v>54</v>
@@ -23918,7 +23918,7 @@
         <v>55</v>
       </c>
       <c r="E315" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F315" t="s">
         <v>60</v>
@@ -23942,22 +23942,22 @@
         <v>202</v>
       </c>
       <c r="O315">
-        <v>17968053</v>
+        <v>17042662</v>
       </c>
       <c r="P315" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q315" t="s">
         <v>235</v>
       </c>
       <c r="R315" s="1">
-        <v>46290.564674375</v>
+        <v>46290.56113170139</v>
       </c>
       <c r="S315">
         <v>5</v>
       </c>
       <c r="T315" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="V315" t="s">
         <v>251</v>
@@ -23966,21 +23966,21 @@
         <v>0</v>
       </c>
       <c r="AB315" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AG315" t="s">
         <v>471</v>
       </c>
       <c r="AH315" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="316" spans="1:34">
       <c r="A316">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B316" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C316" t="s">
         <v>54</v>
@@ -23989,10 +23989,10 @@
         <v>55</v>
       </c>
       <c r="E316" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F316" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G316">
         <v>11516</v>
@@ -24013,51 +24013,48 @@
         <v>202</v>
       </c>
       <c r="O316">
-        <v>17042662</v>
+        <v>18178314</v>
       </c>
       <c r="P316" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q316" t="s">
         <v>235</v>
       </c>
       <c r="R316" s="1">
-        <v>46290.56113170139</v>
+        <v>46290.56957094908</v>
       </c>
       <c r="S316">
         <v>5</v>
       </c>
       <c r="T316" t="s">
-        <v>239</v>
-      </c>
-      <c r="V316" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="AA316">
         <v>0</v>
       </c>
       <c r="AB316" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AG316" t="s">
         <v>471</v>
       </c>
       <c r="AH316" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="317" spans="1:34">
       <c r="A317">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B317" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C317" t="s">
         <v>54</v>
       </c>
       <c r="D317" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E317" t="s">
         <v>58</v>
@@ -24084,42 +24081,42 @@
         <v>202</v>
       </c>
       <c r="O317">
-        <v>18178314</v>
+        <v>18187985</v>
       </c>
       <c r="P317" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Q317" t="s">
         <v>235</v>
       </c>
       <c r="R317" s="1">
-        <v>46290.56957094908</v>
+        <v>46290.40572291666</v>
       </c>
       <c r="S317">
         <v>5</v>
       </c>
       <c r="T317" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AA317">
         <v>0</v>
       </c>
       <c r="AB317" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AG317" t="s">
         <v>471</v>
       </c>
       <c r="AH317" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="318" spans="1:34">
       <c r="A318">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B318" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C318" t="s">
         <v>54</v>
@@ -24152,7 +24149,7 @@
         <v>202</v>
       </c>
       <c r="O318">
-        <v>18187985</v>
+        <v>18241255</v>
       </c>
       <c r="P318" t="s">
         <v>210</v>
@@ -24161,7 +24158,7 @@
         <v>235</v>
       </c>
       <c r="R318" s="1">
-        <v>46290.40572291666</v>
+        <v>46290.40597356481</v>
       </c>
       <c r="S318">
         <v>5</v>
@@ -24184,10 +24181,10 @@
     </row>
     <row r="319" spans="1:34">
       <c r="A319">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B319" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C319" t="s">
         <v>54</v>
@@ -24202,7 +24199,7 @@
         <v>61</v>
       </c>
       <c r="G319">
-        <v>11516</v>
+        <v>10992</v>
       </c>
       <c r="H319">
         <v>0</v>
@@ -24211,16 +24208,16 @@
         <v>63</v>
       </c>
       <c r="J319" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="L319" s="1">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="N319" t="s">
         <v>202</v>
       </c>
       <c r="O319">
-        <v>18241255</v>
+        <v>18249084</v>
       </c>
       <c r="P319" t="s">
         <v>210</v>
@@ -24229,14 +24226,17 @@
         <v>235</v>
       </c>
       <c r="R319" s="1">
-        <v>46290.40597356481</v>
+        <v>46293.54930709491</v>
       </c>
       <c r="S319">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T319" t="s">
         <v>242</v>
       </c>
+      <c r="W319" t="s">
+        <v>343</v>
+      </c>
       <c r="AA319">
         <v>0</v>
       </c>
@@ -24244,7 +24244,7 @@
         <v>210</v>
       </c>
       <c r="AG319" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="AH319" t="s">
         <v>472</v>
@@ -24252,10 +24252,10 @@
     </row>
     <row r="320" spans="1:34">
       <c r="A320">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B320" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C320" t="s">
         <v>54</v>
@@ -24288,7 +24288,7 @@
         <v>202</v>
       </c>
       <c r="O320">
-        <v>18249084</v>
+        <v>18249092</v>
       </c>
       <c r="P320" t="s">
         <v>210</v>
@@ -24297,7 +24297,7 @@
         <v>235</v>
       </c>
       <c r="R320" s="1">
-        <v>46293.54930709491</v>
+        <v>46293.5514684838</v>
       </c>
       <c r="S320">
         <v>0</v>
@@ -24306,7 +24306,7 @@
         <v>242</v>
       </c>
       <c r="W320" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AA320">
         <v>0</v>
@@ -24323,25 +24323,25 @@
     </row>
     <row r="321" spans="1:34">
       <c r="A321">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B321" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C321" t="s">
         <v>54</v>
       </c>
       <c r="D321" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E321" t="s">
         <v>58</v>
       </c>
       <c r="F321" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G321">
-        <v>10992</v>
+        <v>7875</v>
       </c>
       <c r="H321">
         <v>0</v>
@@ -24350,7 +24350,7 @@
         <v>63</v>
       </c>
       <c r="J321" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L321" s="1">
         <v>46295</v>
@@ -24359,22 +24359,25 @@
         <v>202</v>
       </c>
       <c r="O321">
-        <v>18249092</v>
+        <v>18096234</v>
       </c>
       <c r="P321" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="Q321" t="s">
         <v>235</v>
       </c>
       <c r="R321" s="1">
-        <v>46293.5514684838</v>
+        <v>46295.40666767361</v>
       </c>
       <c r="S321">
         <v>0</v>
       </c>
       <c r="T321" t="s">
-        <v>242</v>
+        <v>238</v>
+      </c>
+      <c r="V321" t="s">
+        <v>251</v>
       </c>
       <c r="W321" t="s">
         <v>344</v>
@@ -24383,21 +24386,21 @@
         <v>0</v>
       </c>
       <c r="AB321" t="s">
-        <v>210</v>
+        <v>458</v>
       </c>
       <c r="AG321" t="s">
         <v>469</v>
       </c>
       <c r="AH321" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="322" spans="1:34">
       <c r="A322">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B322" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C322" t="s">
         <v>54</v>
@@ -24406,7 +24409,7 @@
         <v>55</v>
       </c>
       <c r="E322" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F322" t="s">
         <v>60</v>
@@ -24430,22 +24433,22 @@
         <v>202</v>
       </c>
       <c r="O322">
-        <v>18096234</v>
+        <v>18096487</v>
       </c>
       <c r="P322" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q322" t="s">
         <v>235</v>
       </c>
       <c r="R322" s="1">
-        <v>46295.40666767361</v>
+        <v>46295.58573206019</v>
       </c>
       <c r="S322">
         <v>0</v>
       </c>
       <c r="T322" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="V322" t="s">
         <v>251</v>
@@ -24463,7 +24466,7 @@
         <v>469</v>
       </c>
       <c r="AH322" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="323" spans="1:34">

</xml_diff>

<commit_message>
Atualização automática: 2026-10-02 16:03
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9346" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9307" uniqueCount="363">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1452,7 +1452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH690"/>
+  <dimension ref="A1:AH687"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:34">
@@ -40370,7 +40370,7 @@
         <v>18291927</v>
       </c>
       <c r="P604" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q604" t="s">
         <v>258</v>
@@ -40429,7 +40429,7 @@
         <v>18291511</v>
       </c>
       <c r="P605" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q605" t="s">
         <v>258</v>
@@ -40606,7 +40606,7 @@
         <v>18291919</v>
       </c>
       <c r="P608" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q608" t="s">
         <v>258</v>
@@ -40665,7 +40665,7 @@
         <v>18291503</v>
       </c>
       <c r="P609" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q609" t="s">
         <v>258</v>
@@ -40842,7 +40842,7 @@
         <v>18291923</v>
       </c>
       <c r="P612" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q612" t="s">
         <v>258</v>
@@ -40901,7 +40901,7 @@
         <v>18291507</v>
       </c>
       <c r="P613" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q613" t="s">
         <v>258</v>
@@ -41196,7 +41196,7 @@
         <v>18291931</v>
       </c>
       <c r="P618" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q618" t="s">
         <v>258</v>
@@ -41255,7 +41255,7 @@
         <v>18291515</v>
       </c>
       <c r="P619" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q619" t="s">
         <v>258</v>
@@ -41452,16 +41452,16 @@
     </row>
     <row r="623" spans="1:34">
       <c r="A623">
-        <v>7095</v>
+        <v>7048</v>
       </c>
       <c r="B623" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C623" t="s">
         <v>61</v>
       </c>
       <c r="D623" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E623" t="s">
         <v>65</v>
@@ -41470,16 +41470,16 @@
         <v>68</v>
       </c>
       <c r="G623">
-        <v>11756</v>
+        <v>6221</v>
       </c>
       <c r="H623">
-        <v>11755</v>
+        <v>6220</v>
       </c>
       <c r="I623" t="s">
         <v>73</v>
       </c>
       <c r="J623" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L623" s="1">
         <v>46297</v>
@@ -41488,7 +41488,7 @@
         <v>219</v>
       </c>
       <c r="O623">
-        <v>18292337</v>
+        <v>18291881</v>
       </c>
       <c r="P623" t="s">
         <v>244</v>
@@ -41500,7 +41500,7 @@
         <v>0</v>
       </c>
       <c r="T623" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="AG623" t="s">
         <v>350</v>
@@ -41511,16 +41511,16 @@
     </row>
     <row r="624" spans="1:34">
       <c r="A624">
-        <v>7048</v>
+        <v>7049</v>
       </c>
       <c r="B624" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C624" t="s">
         <v>61</v>
       </c>
       <c r="D624" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E624" t="s">
         <v>65</v>
@@ -41547,10 +41547,10 @@
         <v>219</v>
       </c>
       <c r="O624">
-        <v>18291881</v>
+        <v>18291487</v>
       </c>
       <c r="P624" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q624" t="s">
         <v>258</v>
@@ -41570,10 +41570,10 @@
     </row>
     <row r="625" spans="1:34">
       <c r="A625">
-        <v>7049</v>
+        <v>7066</v>
       </c>
       <c r="B625" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C625" t="s">
         <v>61</v>
@@ -41606,7 +41606,7 @@
         <v>219</v>
       </c>
       <c r="O625">
-        <v>18291487</v>
+        <v>18292372</v>
       </c>
       <c r="P625" t="s">
         <v>256</v>
@@ -41618,7 +41618,7 @@
         <v>0</v>
       </c>
       <c r="T625" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="AG625" t="s">
         <v>350</v>
@@ -41629,16 +41629,16 @@
     </row>
     <row r="626" spans="1:34">
       <c r="A626">
-        <v>7066</v>
+        <v>7048</v>
       </c>
       <c r="B626" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C626" t="s">
         <v>61</v>
       </c>
       <c r="D626" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E626" t="s">
         <v>65</v>
@@ -41647,16 +41647,16 @@
         <v>68</v>
       </c>
       <c r="G626">
-        <v>6221</v>
+        <v>6223</v>
       </c>
       <c r="H626">
-        <v>6220</v>
+        <v>6222</v>
       </c>
       <c r="I626" t="s">
         <v>73</v>
       </c>
       <c r="J626" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L626" s="1">
         <v>46297</v>
@@ -41665,10 +41665,10 @@
         <v>219</v>
       </c>
       <c r="O626">
-        <v>18292372</v>
+        <v>18291885</v>
       </c>
       <c r="P626" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q626" t="s">
         <v>258</v>
@@ -41677,7 +41677,7 @@
         <v>0</v>
       </c>
       <c r="T626" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="AG626" t="s">
         <v>350</v>
@@ -41688,10 +41688,10 @@
     </row>
     <row r="627" spans="1:34">
       <c r="A627">
-        <v>7095</v>
+        <v>7049</v>
       </c>
       <c r="B627" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C627" t="s">
         <v>61</v>
@@ -41706,16 +41706,16 @@
         <v>68</v>
       </c>
       <c r="G627">
-        <v>6221</v>
+        <v>6223</v>
       </c>
       <c r="H627">
-        <v>6220</v>
+        <v>6222</v>
       </c>
       <c r="I627" t="s">
         <v>73</v>
       </c>
       <c r="J627" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L627" s="1">
         <v>46297</v>
@@ -41724,7 +41724,7 @@
         <v>219</v>
       </c>
       <c r="O627">
-        <v>18292305</v>
+        <v>18291491</v>
       </c>
       <c r="P627" t="s">
         <v>244</v>
@@ -41736,7 +41736,7 @@
         <v>0</v>
       </c>
       <c r="T627" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="AG627" t="s">
         <v>350</v>
@@ -41747,16 +41747,16 @@
     </row>
     <row r="628" spans="1:34">
       <c r="A628">
-        <v>7048</v>
+        <v>7066</v>
       </c>
       <c r="B628" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C628" t="s">
         <v>61</v>
       </c>
       <c r="D628" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E628" t="s">
         <v>65</v>
@@ -41783,7 +41783,7 @@
         <v>219</v>
       </c>
       <c r="O628">
-        <v>18291885</v>
+        <v>18292376</v>
       </c>
       <c r="P628" t="s">
         <v>256</v>
@@ -41795,7 +41795,7 @@
         <v>0</v>
       </c>
       <c r="T628" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="AG628" t="s">
         <v>350</v>
@@ -41806,16 +41806,16 @@
     </row>
     <row r="629" spans="1:34">
       <c r="A629">
-        <v>7049</v>
+        <v>7048</v>
       </c>
       <c r="B629" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C629" t="s">
         <v>61</v>
       </c>
       <c r="D629" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E629" t="s">
         <v>65</v>
@@ -41824,16 +41824,16 @@
         <v>68</v>
       </c>
       <c r="G629">
-        <v>6223</v>
+        <v>11766</v>
       </c>
       <c r="H629">
-        <v>6222</v>
+        <v>11765</v>
       </c>
       <c r="I629" t="s">
         <v>73</v>
       </c>
       <c r="J629" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L629" s="1">
         <v>46297</v>
@@ -41842,10 +41842,10 @@
         <v>219</v>
       </c>
       <c r="O629">
-        <v>18291491</v>
+        <v>18291935</v>
       </c>
       <c r="P629" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q629" t="s">
         <v>258</v>
@@ -41865,10 +41865,10 @@
     </row>
     <row r="630" spans="1:34">
       <c r="A630">
-        <v>7066</v>
+        <v>7049</v>
       </c>
       <c r="B630" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C630" t="s">
         <v>61</v>
@@ -41883,16 +41883,16 @@
         <v>68</v>
       </c>
       <c r="G630">
-        <v>6223</v>
+        <v>11766</v>
       </c>
       <c r="H630">
-        <v>6222</v>
+        <v>11765</v>
       </c>
       <c r="I630" t="s">
         <v>73</v>
       </c>
       <c r="J630" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L630" s="1">
         <v>46297</v>
@@ -41901,10 +41901,10 @@
         <v>219</v>
       </c>
       <c r="O630">
-        <v>18292376</v>
+        <v>18291519</v>
       </c>
       <c r="P630" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q630" t="s">
         <v>258</v>
@@ -41913,7 +41913,7 @@
         <v>0</v>
       </c>
       <c r="T630" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="AG630" t="s">
         <v>350</v>
@@ -41924,10 +41924,10 @@
     </row>
     <row r="631" spans="1:34">
       <c r="A631">
-        <v>7095</v>
+        <v>7066</v>
       </c>
       <c r="B631" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C631" t="s">
         <v>61</v>
@@ -41942,16 +41942,16 @@
         <v>68</v>
       </c>
       <c r="G631">
-        <v>6223</v>
+        <v>11766</v>
       </c>
       <c r="H631">
-        <v>6222</v>
+        <v>11765</v>
       </c>
       <c r="I631" t="s">
         <v>73</v>
       </c>
       <c r="J631" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L631" s="1">
         <v>46297</v>
@@ -41960,10 +41960,10 @@
         <v>219</v>
       </c>
       <c r="O631">
-        <v>18292309</v>
+        <v>18292412</v>
       </c>
       <c r="P631" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="Q631" t="s">
         <v>258</v>
@@ -41972,7 +41972,7 @@
         <v>0</v>
       </c>
       <c r="T631" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AG631" t="s">
         <v>350</v>
@@ -41983,16 +41983,16 @@
     </row>
     <row r="632" spans="1:34">
       <c r="A632">
-        <v>7048</v>
+        <v>7095</v>
       </c>
       <c r="B632" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C632" t="s">
         <v>61</v>
       </c>
       <c r="D632" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E632" t="s">
         <v>65</v>
@@ -42019,10 +42019,10 @@
         <v>219</v>
       </c>
       <c r="O632">
-        <v>18291935</v>
+        <v>18292349</v>
       </c>
       <c r="P632" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q632" t="s">
         <v>258</v>
@@ -42031,7 +42031,7 @@
         <v>0</v>
       </c>
       <c r="T632" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="AG632" t="s">
         <v>350</v>
@@ -42042,16 +42042,16 @@
     </row>
     <row r="633" spans="1:34">
       <c r="A633">
-        <v>7049</v>
+        <v>7048</v>
       </c>
       <c r="B633" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C633" t="s">
         <v>61</v>
       </c>
       <c r="D633" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E633" t="s">
         <v>65</v>
@@ -42060,16 +42060,16 @@
         <v>68</v>
       </c>
       <c r="G633">
-        <v>11766</v>
+        <v>11768</v>
       </c>
       <c r="H633">
-        <v>11765</v>
+        <v>11767</v>
       </c>
       <c r="I633" t="s">
         <v>73</v>
       </c>
       <c r="J633" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L633" s="1">
         <v>46297</v>
@@ -42078,10 +42078,10 @@
         <v>219</v>
       </c>
       <c r="O633">
-        <v>18291519</v>
+        <v>18291939</v>
       </c>
       <c r="P633" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q633" t="s">
         <v>258</v>
@@ -42101,10 +42101,10 @@
     </row>
     <row r="634" spans="1:34">
       <c r="A634">
-        <v>7066</v>
+        <v>7049</v>
       </c>
       <c r="B634" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C634" t="s">
         <v>61</v>
@@ -42119,16 +42119,16 @@
         <v>68</v>
       </c>
       <c r="G634">
-        <v>11766</v>
+        <v>11768</v>
       </c>
       <c r="H634">
-        <v>11765</v>
+        <v>11767</v>
       </c>
       <c r="I634" t="s">
         <v>73</v>
       </c>
       <c r="J634" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L634" s="1">
         <v>46297</v>
@@ -42137,10 +42137,10 @@
         <v>219</v>
       </c>
       <c r="O634">
-        <v>18292412</v>
+        <v>18291523</v>
       </c>
       <c r="P634" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q634" t="s">
         <v>258</v>
@@ -42149,7 +42149,7 @@
         <v>0</v>
       </c>
       <c r="T634" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="AG634" t="s">
         <v>350</v>
@@ -42160,10 +42160,10 @@
     </row>
     <row r="635" spans="1:34">
       <c r="A635">
-        <v>7095</v>
+        <v>7066</v>
       </c>
       <c r="B635" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C635" t="s">
         <v>61</v>
@@ -42178,16 +42178,16 @@
         <v>68</v>
       </c>
       <c r="G635">
-        <v>11766</v>
+        <v>11768</v>
       </c>
       <c r="H635">
-        <v>11765</v>
+        <v>11767</v>
       </c>
       <c r="I635" t="s">
         <v>73</v>
       </c>
       <c r="J635" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L635" s="1">
         <v>46297</v>
@@ -42196,10 +42196,10 @@
         <v>219</v>
       </c>
       <c r="O635">
-        <v>18292349</v>
+        <v>18292416</v>
       </c>
       <c r="P635" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="Q635" t="s">
         <v>258</v>
@@ -42208,7 +42208,7 @@
         <v>0</v>
       </c>
       <c r="T635" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AG635" t="s">
         <v>350</v>
@@ -42219,16 +42219,16 @@
     </row>
     <row r="636" spans="1:34">
       <c r="A636">
-        <v>7048</v>
+        <v>7095</v>
       </c>
       <c r="B636" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C636" t="s">
         <v>61</v>
       </c>
       <c r="D636" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E636" t="s">
         <v>65</v>
@@ -42255,10 +42255,10 @@
         <v>219</v>
       </c>
       <c r="O636">
-        <v>18291939</v>
+        <v>18292353</v>
       </c>
       <c r="P636" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Q636" t="s">
         <v>258</v>
@@ -42267,7 +42267,7 @@
         <v>0</v>
       </c>
       <c r="T636" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="AG636" t="s">
         <v>350</v>
@@ -42278,10 +42278,10 @@
     </row>
     <row r="637" spans="1:34">
       <c r="A637">
-        <v>7049</v>
+        <v>7095</v>
       </c>
       <c r="B637" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C637" t="s">
         <v>61</v>
@@ -42296,28 +42296,31 @@
         <v>68</v>
       </c>
       <c r="G637">
-        <v>11768</v>
+        <v>11686</v>
       </c>
       <c r="H637">
-        <v>11767</v>
+        <v>11685</v>
       </c>
       <c r="I637" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J637" t="s">
-        <v>133</v>
+        <v>195</v>
       </c>
       <c r="L637" s="1">
         <v>46297</v>
       </c>
+      <c r="M637" t="s">
+        <v>209</v>
+      </c>
       <c r="N637" t="s">
         <v>219</v>
       </c>
       <c r="O637">
-        <v>18291523</v>
+        <v>18273891</v>
       </c>
       <c r="P637" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="Q637" t="s">
         <v>258</v>
@@ -42326,27 +42329,27 @@
         <v>0</v>
       </c>
       <c r="T637" t="s">
-        <v>273</v>
+        <v>264</v>
+      </c>
+      <c r="W637" t="s">
+        <v>345</v>
       </c>
       <c r="AG637" t="s">
         <v>350</v>
       </c>
-      <c r="AH637" t="s">
-        <v>361</v>
-      </c>
     </row>
     <row r="638" spans="1:34">
       <c r="A638">
-        <v>7066</v>
+        <v>7106</v>
       </c>
       <c r="B638" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C638" t="s">
         <v>61</v>
       </c>
       <c r="D638" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E638" t="s">
         <v>65</v>
@@ -42355,16 +42358,16 @@
         <v>68</v>
       </c>
       <c r="G638">
-        <v>11768</v>
+        <v>11686</v>
       </c>
       <c r="H638">
-        <v>11767</v>
+        <v>11685</v>
       </c>
       <c r="I638" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J638" t="s">
-        <v>133</v>
+        <v>195</v>
       </c>
       <c r="L638" s="1">
         <v>46297</v>
@@ -42373,10 +42376,10 @@
         <v>219</v>
       </c>
       <c r="O638">
-        <v>18292416</v>
+        <v>18286174</v>
       </c>
       <c r="P638" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="Q638" t="s">
         <v>258</v>
@@ -42385,21 +42388,21 @@
         <v>0</v>
       </c>
       <c r="T638" t="s">
-        <v>265</v>
+        <v>271</v>
+      </c>
+      <c r="W638" t="s">
+        <v>346</v>
       </c>
       <c r="AG638" t="s">
         <v>350</v>
       </c>
-      <c r="AH638" t="s">
-        <v>361</v>
-      </c>
     </row>
     <row r="639" spans="1:34">
       <c r="A639">
-        <v>7095</v>
+        <v>7107</v>
       </c>
       <c r="B639" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C639" t="s">
         <v>61</v>
@@ -42414,16 +42417,16 @@
         <v>68</v>
       </c>
       <c r="G639">
-        <v>11768</v>
+        <v>11686</v>
       </c>
       <c r="H639">
-        <v>11767</v>
+        <v>11685</v>
       </c>
       <c r="I639" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J639" t="s">
-        <v>133</v>
+        <v>195</v>
       </c>
       <c r="L639" s="1">
         <v>46297</v>
@@ -42432,10 +42435,10 @@
         <v>219</v>
       </c>
       <c r="O639">
-        <v>18292353</v>
+        <v>18286179</v>
       </c>
       <c r="P639" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="Q639" t="s">
         <v>258</v>
@@ -42444,13 +42447,13 @@
         <v>0</v>
       </c>
       <c r="T639" t="s">
-        <v>264</v>
+        <v>271</v>
+      </c>
+      <c r="W639" t="s">
+        <v>346</v>
       </c>
       <c r="AG639" t="s">
         <v>350</v>
-      </c>
-      <c r="AH639" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="640" spans="1:34">
@@ -42473,7 +42476,7 @@
         <v>68</v>
       </c>
       <c r="G640">
-        <v>11686</v>
+        <v>11687</v>
       </c>
       <c r="H640">
         <v>11685</v>
@@ -42482,7 +42485,7 @@
         <v>75</v>
       </c>
       <c r="J640" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L640" s="1">
         <v>46297</v>
@@ -42494,7 +42497,7 @@
         <v>219</v>
       </c>
       <c r="O640">
-        <v>18273891</v>
+        <v>18273892</v>
       </c>
       <c r="P640" t="s">
         <v>246</v>
@@ -42535,7 +42538,7 @@
         <v>68</v>
       </c>
       <c r="G641">
-        <v>11686</v>
+        <v>11687</v>
       </c>
       <c r="H641">
         <v>11685</v>
@@ -42544,7 +42547,7 @@
         <v>75</v>
       </c>
       <c r="J641" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L641" s="1">
         <v>46297</v>
@@ -42553,7 +42556,7 @@
         <v>219</v>
       </c>
       <c r="O641">
-        <v>18286174</v>
+        <v>18286175</v>
       </c>
       <c r="P641" t="s">
         <v>246</v>
@@ -42594,7 +42597,7 @@
         <v>68</v>
       </c>
       <c r="G642">
-        <v>11686</v>
+        <v>11687</v>
       </c>
       <c r="H642">
         <v>11685</v>
@@ -42603,7 +42606,7 @@
         <v>75</v>
       </c>
       <c r="J642" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L642" s="1">
         <v>46297</v>
@@ -42612,7 +42615,7 @@
         <v>219</v>
       </c>
       <c r="O642">
-        <v>18286179</v>
+        <v>18286180</v>
       </c>
       <c r="P642" t="s">
         <v>246</v>
@@ -42653,7 +42656,7 @@
         <v>68</v>
       </c>
       <c r="G643">
-        <v>11687</v>
+        <v>11688</v>
       </c>
       <c r="H643">
         <v>11685</v>
@@ -42662,7 +42665,7 @@
         <v>75</v>
       </c>
       <c r="J643" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L643" s="1">
         <v>46297</v>
@@ -42674,7 +42677,7 @@
         <v>219</v>
       </c>
       <c r="O643">
-        <v>18273892</v>
+        <v>18273893</v>
       </c>
       <c r="P643" t="s">
         <v>246</v>
@@ -42715,7 +42718,7 @@
         <v>68</v>
       </c>
       <c r="G644">
-        <v>11687</v>
+        <v>11688</v>
       </c>
       <c r="H644">
         <v>11685</v>
@@ -42724,7 +42727,7 @@
         <v>75</v>
       </c>
       <c r="J644" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L644" s="1">
         <v>46297</v>
@@ -42733,7 +42736,7 @@
         <v>219</v>
       </c>
       <c r="O644">
-        <v>18286175</v>
+        <v>18286176</v>
       </c>
       <c r="P644" t="s">
         <v>246</v>
@@ -42774,7 +42777,7 @@
         <v>68</v>
       </c>
       <c r="G645">
-        <v>11687</v>
+        <v>11688</v>
       </c>
       <c r="H645">
         <v>11685</v>
@@ -42783,7 +42786,7 @@
         <v>75</v>
       </c>
       <c r="J645" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L645" s="1">
         <v>46297</v>
@@ -42792,7 +42795,7 @@
         <v>219</v>
       </c>
       <c r="O645">
-        <v>18286180</v>
+        <v>18286181</v>
       </c>
       <c r="P645" t="s">
         <v>246</v>
@@ -42833,7 +42836,7 @@
         <v>68</v>
       </c>
       <c r="G646">
-        <v>11688</v>
+        <v>11689</v>
       </c>
       <c r="H646">
         <v>11685</v>
@@ -42842,7 +42845,7 @@
         <v>75</v>
       </c>
       <c r="J646" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L646" s="1">
         <v>46297</v>
@@ -42854,7 +42857,7 @@
         <v>219</v>
       </c>
       <c r="O646">
-        <v>18273893</v>
+        <v>18273894</v>
       </c>
       <c r="P646" t="s">
         <v>246</v>
@@ -42895,7 +42898,7 @@
         <v>68</v>
       </c>
       <c r="G647">
-        <v>11688</v>
+        <v>11689</v>
       </c>
       <c r="H647">
         <v>11685</v>
@@ -42904,7 +42907,7 @@
         <v>75</v>
       </c>
       <c r="J647" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L647" s="1">
         <v>46297</v>
@@ -42913,7 +42916,7 @@
         <v>219</v>
       </c>
       <c r="O647">
-        <v>18286176</v>
+        <v>18286177</v>
       </c>
       <c r="P647" t="s">
         <v>246</v>
@@ -42954,7 +42957,7 @@
         <v>68</v>
       </c>
       <c r="G648">
-        <v>11688</v>
+        <v>11689</v>
       </c>
       <c r="H648">
         <v>11685</v>
@@ -42963,7 +42966,7 @@
         <v>75</v>
       </c>
       <c r="J648" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L648" s="1">
         <v>46297</v>
@@ -42972,7 +42975,7 @@
         <v>219</v>
       </c>
       <c r="O648">
-        <v>18286181</v>
+        <v>18286182</v>
       </c>
       <c r="P648" t="s">
         <v>246</v>
@@ -43013,16 +43016,16 @@
         <v>68</v>
       </c>
       <c r="G649">
-        <v>11689</v>
+        <v>11070</v>
       </c>
       <c r="H649">
-        <v>11685</v>
+        <v>0</v>
       </c>
       <c r="I649" t="s">
         <v>75</v>
       </c>
       <c r="J649" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L649" s="1">
         <v>46297</v>
@@ -43034,7 +43037,7 @@
         <v>219</v>
       </c>
       <c r="O649">
-        <v>18273894</v>
+        <v>18273878</v>
       </c>
       <c r="P649" t="s">
         <v>246</v>
@@ -43075,16 +43078,16 @@
         <v>68</v>
       </c>
       <c r="G650">
-        <v>11689</v>
+        <v>11070</v>
       </c>
       <c r="H650">
-        <v>11685</v>
+        <v>0</v>
       </c>
       <c r="I650" t="s">
         <v>75</v>
       </c>
       <c r="J650" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L650" s="1">
         <v>46297</v>
@@ -43093,7 +43096,7 @@
         <v>219</v>
       </c>
       <c r="O650">
-        <v>18286177</v>
+        <v>18286149</v>
       </c>
       <c r="P650" t="s">
         <v>246</v>
@@ -43134,16 +43137,16 @@
         <v>68</v>
       </c>
       <c r="G651">
-        <v>11689</v>
+        <v>11070</v>
       </c>
       <c r="H651">
-        <v>11685</v>
+        <v>0</v>
       </c>
       <c r="I651" t="s">
         <v>75</v>
       </c>
       <c r="J651" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L651" s="1">
         <v>46297</v>
@@ -43152,7 +43155,7 @@
         <v>219</v>
       </c>
       <c r="O651">
-        <v>18286182</v>
+        <v>18286150</v>
       </c>
       <c r="P651" t="s">
         <v>246</v>
@@ -43175,16 +43178,16 @@
     </row>
     <row r="652" spans="1:33">
       <c r="A652">
-        <v>7095</v>
+        <v>7106</v>
       </c>
       <c r="B652" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C652" t="s">
         <v>61</v>
       </c>
       <c r="D652" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E652" t="s">
         <v>65</v>
@@ -43193,28 +43196,25 @@
         <v>68</v>
       </c>
       <c r="G652">
-        <v>11070</v>
+        <v>11872</v>
       </c>
       <c r="H652">
-        <v>0</v>
+        <v>11869</v>
       </c>
       <c r="I652" t="s">
         <v>75</v>
       </c>
       <c r="J652" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L652" s="1">
         <v>46297</v>
       </c>
-      <c r="M652" t="s">
-        <v>209</v>
-      </c>
       <c r="N652" t="s">
         <v>219</v>
       </c>
       <c r="O652">
-        <v>18273878</v>
+        <v>18286154</v>
       </c>
       <c r="P652" t="s">
         <v>246</v>
@@ -43226,10 +43226,10 @@
         <v>0</v>
       </c>
       <c r="T652" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="W652" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="AG652" t="s">
         <v>350</v>
@@ -43237,16 +43237,16 @@
     </row>
     <row r="653" spans="1:33">
       <c r="A653">
-        <v>7106</v>
+        <v>7107</v>
       </c>
       <c r="B653" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C653" t="s">
         <v>61</v>
       </c>
       <c r="D653" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E653" t="s">
         <v>65</v>
@@ -43255,16 +43255,16 @@
         <v>68</v>
       </c>
       <c r="G653">
-        <v>11070</v>
+        <v>11872</v>
       </c>
       <c r="H653">
-        <v>0</v>
+        <v>11869</v>
       </c>
       <c r="I653" t="s">
         <v>75</v>
       </c>
       <c r="J653" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L653" s="1">
         <v>46297</v>
@@ -43273,7 +43273,7 @@
         <v>219</v>
       </c>
       <c r="O653">
-        <v>18286149</v>
+        <v>18286158</v>
       </c>
       <c r="P653" t="s">
         <v>246</v>
@@ -43296,10 +43296,10 @@
     </row>
     <row r="654" spans="1:33">
       <c r="A654">
-        <v>7107</v>
+        <v>7095</v>
       </c>
       <c r="B654" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C654" t="s">
         <v>61</v>
@@ -43314,25 +43314,28 @@
         <v>68</v>
       </c>
       <c r="G654">
-        <v>11070</v>
+        <v>11870</v>
       </c>
       <c r="H654">
-        <v>0</v>
+        <v>11869</v>
       </c>
       <c r="I654" t="s">
         <v>75</v>
       </c>
       <c r="J654" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L654" s="1">
         <v>46297</v>
       </c>
+      <c r="M654" t="s">
+        <v>209</v>
+      </c>
       <c r="N654" t="s">
         <v>219</v>
       </c>
       <c r="O654">
-        <v>18286150</v>
+        <v>18273880</v>
       </c>
       <c r="P654" t="s">
         <v>246</v>
@@ -43344,10 +43347,10 @@
         <v>0</v>
       </c>
       <c r="T654" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="W654" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AG654" t="s">
         <v>350</v>
@@ -43373,7 +43376,7 @@
         <v>68</v>
       </c>
       <c r="G655">
-        <v>11872</v>
+        <v>11870</v>
       </c>
       <c r="H655">
         <v>11869</v>
@@ -43382,7 +43385,7 @@
         <v>75</v>
       </c>
       <c r="J655" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L655" s="1">
         <v>46297</v>
@@ -43391,7 +43394,7 @@
         <v>219</v>
       </c>
       <c r="O655">
-        <v>18286154</v>
+        <v>18286152</v>
       </c>
       <c r="P655" t="s">
         <v>246</v>
@@ -43432,7 +43435,7 @@
         <v>68</v>
       </c>
       <c r="G656">
-        <v>11872</v>
+        <v>11870</v>
       </c>
       <c r="H656">
         <v>11869</v>
@@ -43441,7 +43444,7 @@
         <v>75</v>
       </c>
       <c r="J656" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L656" s="1">
         <v>46297</v>
@@ -43450,7 +43453,7 @@
         <v>219</v>
       </c>
       <c r="O656">
-        <v>18286158</v>
+        <v>18286156</v>
       </c>
       <c r="P656" t="s">
         <v>246</v>
@@ -43491,7 +43494,7 @@
         <v>68</v>
       </c>
       <c r="G657">
-        <v>11870</v>
+        <v>11871</v>
       </c>
       <c r="H657">
         <v>11869</v>
@@ -43500,7 +43503,7 @@
         <v>75</v>
       </c>
       <c r="J657" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L657" s="1">
         <v>46297</v>
@@ -43512,7 +43515,7 @@
         <v>219</v>
       </c>
       <c r="O657">
-        <v>18273880</v>
+        <v>18273881</v>
       </c>
       <c r="P657" t="s">
         <v>246</v>
@@ -43553,7 +43556,7 @@
         <v>68</v>
       </c>
       <c r="G658">
-        <v>11870</v>
+        <v>11871</v>
       </c>
       <c r="H658">
         <v>11869</v>
@@ -43562,7 +43565,7 @@
         <v>75</v>
       </c>
       <c r="J658" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L658" s="1">
         <v>46297</v>
@@ -43571,7 +43574,7 @@
         <v>219</v>
       </c>
       <c r="O658">
-        <v>18286152</v>
+        <v>18286153</v>
       </c>
       <c r="P658" t="s">
         <v>246</v>
@@ -43612,7 +43615,7 @@
         <v>68</v>
       </c>
       <c r="G659">
-        <v>11870</v>
+        <v>11871</v>
       </c>
       <c r="H659">
         <v>11869</v>
@@ -43621,7 +43624,7 @@
         <v>75</v>
       </c>
       <c r="J659" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L659" s="1">
         <v>46297</v>
@@ -43630,7 +43633,7 @@
         <v>219</v>
       </c>
       <c r="O659">
-        <v>18286156</v>
+        <v>18286157</v>
       </c>
       <c r="P659" t="s">
         <v>246</v>
@@ -43653,10 +43656,10 @@
     </row>
     <row r="660" spans="1:33">
       <c r="A660">
-        <v>7095</v>
+        <v>6966</v>
       </c>
       <c r="B660" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C660" t="s">
         <v>61</v>
@@ -43671,28 +43674,25 @@
         <v>68</v>
       </c>
       <c r="G660">
-        <v>11871</v>
+        <v>5989</v>
       </c>
       <c r="H660">
-        <v>11869</v>
+        <v>0</v>
       </c>
       <c r="I660" t="s">
         <v>75</v>
       </c>
       <c r="J660" t="s">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="L660" s="1">
         <v>46297</v>
       </c>
-      <c r="M660" t="s">
-        <v>209</v>
-      </c>
       <c r="N660" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O660">
-        <v>18273881</v>
+        <v>18189348</v>
       </c>
       <c r="P660" t="s">
         <v>246</v>
@@ -43704,27 +43704,24 @@
         <v>0</v>
       </c>
       <c r="T660" t="s">
-        <v>264</v>
-      </c>
-      <c r="W660" t="s">
-        <v>345</v>
+        <v>274</v>
       </c>
       <c r="AG660" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="661" spans="1:33">
       <c r="A661">
-        <v>7106</v>
+        <v>6967</v>
       </c>
       <c r="B661" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="C661" t="s">
         <v>61</v>
       </c>
       <c r="D661" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E661" t="s">
         <v>65</v>
@@ -43733,25 +43730,25 @@
         <v>68</v>
       </c>
       <c r="G661">
-        <v>11871</v>
+        <v>5989</v>
       </c>
       <c r="H661">
-        <v>11869</v>
+        <v>0</v>
       </c>
       <c r="I661" t="s">
         <v>75</v>
       </c>
       <c r="J661" t="s">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="L661" s="1">
         <v>46297</v>
       </c>
       <c r="N661" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O661">
-        <v>18286153</v>
+        <v>18189277</v>
       </c>
       <c r="P661" t="s">
         <v>246</v>
@@ -43763,27 +43760,24 @@
         <v>0</v>
       </c>
       <c r="T661" t="s">
-        <v>271</v>
-      </c>
-      <c r="W661" t="s">
-        <v>346</v>
+        <v>274</v>
       </c>
       <c r="AG661" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="662" spans="1:33">
       <c r="A662">
-        <v>7107</v>
+        <v>6981</v>
       </c>
       <c r="B662" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C662" t="s">
         <v>61</v>
       </c>
       <c r="D662" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E662" t="s">
         <v>65</v>
@@ -43792,25 +43786,25 @@
         <v>68</v>
       </c>
       <c r="G662">
-        <v>11871</v>
+        <v>5989</v>
       </c>
       <c r="H662">
-        <v>11869</v>
+        <v>0</v>
       </c>
       <c r="I662" t="s">
         <v>75</v>
       </c>
       <c r="J662" t="s">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="L662" s="1">
         <v>46297</v>
       </c>
       <c r="N662" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O662">
-        <v>18286157</v>
+        <v>18199134</v>
       </c>
       <c r="P662" t="s">
         <v>246</v>
@@ -43822,27 +43816,24 @@
         <v>0</v>
       </c>
       <c r="T662" t="s">
-        <v>271</v>
-      </c>
-      <c r="W662" t="s">
-        <v>346</v>
+        <v>272</v>
       </c>
       <c r="AG662" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="663" spans="1:33">
       <c r="A663">
-        <v>6966</v>
+        <v>6992</v>
       </c>
       <c r="B663" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C663" t="s">
         <v>61</v>
       </c>
       <c r="D663" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E663" t="s">
         <v>65</v>
@@ -43869,7 +43860,7 @@
         <v>220</v>
       </c>
       <c r="O663">
-        <v>18189348</v>
+        <v>18211351</v>
       </c>
       <c r="P663" t="s">
         <v>246</v>
@@ -43881,7 +43872,7 @@
         <v>0</v>
       </c>
       <c r="T663" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AG663" t="s">
         <v>352</v>
@@ -43889,10 +43880,10 @@
     </row>
     <row r="664" spans="1:33">
       <c r="A664">
-        <v>6967</v>
+        <v>6993</v>
       </c>
       <c r="B664" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C664" t="s">
         <v>61</v>
@@ -43904,7 +43895,7 @@
         <v>65</v>
       </c>
       <c r="F664" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G664">
         <v>5989</v>
@@ -43925,7 +43916,7 @@
         <v>220</v>
       </c>
       <c r="O664">
-        <v>18189277</v>
+        <v>18211400</v>
       </c>
       <c r="P664" t="s">
         <v>246</v>
@@ -43937,7 +43928,7 @@
         <v>0</v>
       </c>
       <c r="T664" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AG664" t="s">
         <v>352</v>
@@ -43945,16 +43936,16 @@
     </row>
     <row r="665" spans="1:33">
       <c r="A665">
-        <v>6981</v>
+        <v>7041</v>
       </c>
       <c r="B665" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C665" t="s">
         <v>61</v>
       </c>
       <c r="D665" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E665" t="s">
         <v>65</v>
@@ -43981,7 +43972,7 @@
         <v>220</v>
       </c>
       <c r="O665">
-        <v>18199134</v>
+        <v>18241157</v>
       </c>
       <c r="P665" t="s">
         <v>246</v>
@@ -43993,7 +43984,7 @@
         <v>0</v>
       </c>
       <c r="T665" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="AG665" t="s">
         <v>352</v>
@@ -44001,10 +43992,10 @@
     </row>
     <row r="666" spans="1:33">
       <c r="A666">
-        <v>6992</v>
+        <v>7048</v>
       </c>
       <c r="B666" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C666" t="s">
         <v>61</v>
@@ -44037,7 +44028,7 @@
         <v>220</v>
       </c>
       <c r="O666">
-        <v>18211351</v>
+        <v>18247538</v>
       </c>
       <c r="P666" t="s">
         <v>246</v>
@@ -44049,7 +44040,7 @@
         <v>0</v>
       </c>
       <c r="T666" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AG666" t="s">
         <v>352</v>
@@ -44057,10 +44048,10 @@
     </row>
     <row r="667" spans="1:33">
       <c r="A667">
-        <v>6993</v>
+        <v>7049</v>
       </c>
       <c r="B667" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C667" t="s">
         <v>61</v>
@@ -44072,7 +44063,7 @@
         <v>65</v>
       </c>
       <c r="F667" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G667">
         <v>5989</v>
@@ -44093,7 +44084,7 @@
         <v>220</v>
       </c>
       <c r="O667">
-        <v>18211400</v>
+        <v>18247602</v>
       </c>
       <c r="P667" t="s">
         <v>246</v>
@@ -44105,7 +44096,7 @@
         <v>0</v>
       </c>
       <c r="T667" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AG667" t="s">
         <v>352</v>
@@ -44113,10 +44104,10 @@
     </row>
     <row r="668" spans="1:33">
       <c r="A668">
-        <v>7041</v>
+        <v>7066</v>
       </c>
       <c r="B668" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C668" t="s">
         <v>61</v>
@@ -44149,7 +44140,7 @@
         <v>220</v>
       </c>
       <c r="O668">
-        <v>18241157</v>
+        <v>18254499</v>
       </c>
       <c r="P668" t="s">
         <v>246</v>
@@ -44161,7 +44152,7 @@
         <v>0</v>
       </c>
       <c r="T668" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="AG668" t="s">
         <v>352</v>
@@ -44169,16 +44160,16 @@
     </row>
     <row r="669" spans="1:33">
       <c r="A669">
-        <v>7048</v>
+        <v>7095</v>
       </c>
       <c r="B669" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C669" t="s">
         <v>61</v>
       </c>
       <c r="D669" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E669" t="s">
         <v>65</v>
@@ -44205,7 +44196,7 @@
         <v>220</v>
       </c>
       <c r="O669">
-        <v>18247538</v>
+        <v>18274349</v>
       </c>
       <c r="P669" t="s">
         <v>246</v>
@@ -44217,7 +44208,7 @@
         <v>0</v>
       </c>
       <c r="T669" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="AG669" t="s">
         <v>352</v>
@@ -44225,10 +44216,10 @@
     </row>
     <row r="670" spans="1:33">
       <c r="A670">
-        <v>7049</v>
+        <v>7095</v>
       </c>
       <c r="B670" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C670" t="s">
         <v>61</v>
@@ -44243,7 +44234,7 @@
         <v>68</v>
       </c>
       <c r="G670">
-        <v>5989</v>
+        <v>11868</v>
       </c>
       <c r="H670">
         <v>0</v>
@@ -44252,16 +44243,19 @@
         <v>75</v>
       </c>
       <c r="J670" t="s">
-        <v>116</v>
+        <v>203</v>
       </c>
       <c r="L670" s="1">
         <v>46297</v>
       </c>
+      <c r="M670" t="s">
+        <v>209</v>
+      </c>
       <c r="N670" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="O670">
-        <v>18247602</v>
+        <v>18273883</v>
       </c>
       <c r="P670" t="s">
         <v>246</v>
@@ -44273,24 +44267,27 @@
         <v>0</v>
       </c>
       <c r="T670" t="s">
-        <v>273</v>
+        <v>264</v>
+      </c>
+      <c r="W670" t="s">
+        <v>345</v>
       </c>
       <c r="AG670" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="671" spans="1:33">
       <c r="A671">
-        <v>7066</v>
+        <v>7106</v>
       </c>
       <c r="B671" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C671" t="s">
         <v>61</v>
       </c>
       <c r="D671" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E671" t="s">
         <v>65</v>
@@ -44299,7 +44296,7 @@
         <v>68</v>
       </c>
       <c r="G671">
-        <v>5989</v>
+        <v>11868</v>
       </c>
       <c r="H671">
         <v>0</v>
@@ -44308,16 +44305,16 @@
         <v>75</v>
       </c>
       <c r="J671" t="s">
-        <v>116</v>
+        <v>203</v>
       </c>
       <c r="L671" s="1">
         <v>46297</v>
       </c>
       <c r="N671" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="O671">
-        <v>18254499</v>
+        <v>18286159</v>
       </c>
       <c r="P671" t="s">
         <v>246</v>
@@ -44329,18 +44326,21 @@
         <v>0</v>
       </c>
       <c r="T671" t="s">
-        <v>265</v>
+        <v>271</v>
+      </c>
+      <c r="W671" t="s">
+        <v>346</v>
       </c>
       <c r="AG671" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="672" spans="1:33">
       <c r="A672">
-        <v>7095</v>
+        <v>7107</v>
       </c>
       <c r="B672" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C672" t="s">
         <v>61</v>
@@ -44355,7 +44355,7 @@
         <v>68</v>
       </c>
       <c r="G672">
-        <v>5989</v>
+        <v>11868</v>
       </c>
       <c r="H672">
         <v>0</v>
@@ -44364,16 +44364,16 @@
         <v>75</v>
       </c>
       <c r="J672" t="s">
-        <v>116</v>
+        <v>203</v>
       </c>
       <c r="L672" s="1">
         <v>46297</v>
       </c>
       <c r="N672" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="O672">
-        <v>18274349</v>
+        <v>18286160</v>
       </c>
       <c r="P672" t="s">
         <v>246</v>
@@ -44385,10 +44385,13 @@
         <v>0</v>
       </c>
       <c r="T672" t="s">
-        <v>264</v>
+        <v>271</v>
+      </c>
+      <c r="W672" t="s">
+        <v>346</v>
       </c>
       <c r="AG672" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="673" spans="1:33">
@@ -44411,16 +44414,16 @@
         <v>68</v>
       </c>
       <c r="G673">
-        <v>11868</v>
+        <v>11684</v>
       </c>
       <c r="H673">
-        <v>0</v>
+        <v>11679</v>
       </c>
       <c r="I673" t="s">
         <v>75</v>
       </c>
       <c r="J673" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L673" s="1">
         <v>46297</v>
@@ -44432,7 +44435,7 @@
         <v>219</v>
       </c>
       <c r="O673">
-        <v>18273883</v>
+        <v>18273889</v>
       </c>
       <c r="P673" t="s">
         <v>246</v>
@@ -44473,16 +44476,16 @@
         <v>68</v>
       </c>
       <c r="G674">
-        <v>11868</v>
+        <v>11684</v>
       </c>
       <c r="H674">
-        <v>0</v>
+        <v>11679</v>
       </c>
       <c r="I674" t="s">
         <v>75</v>
       </c>
       <c r="J674" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L674" s="1">
         <v>46297</v>
@@ -44491,7 +44494,7 @@
         <v>219</v>
       </c>
       <c r="O674">
-        <v>18286159</v>
+        <v>18286166</v>
       </c>
       <c r="P674" t="s">
         <v>246</v>
@@ -44532,16 +44535,16 @@
         <v>68</v>
       </c>
       <c r="G675">
-        <v>11868</v>
+        <v>11684</v>
       </c>
       <c r="H675">
-        <v>0</v>
+        <v>11679</v>
       </c>
       <c r="I675" t="s">
         <v>75</v>
       </c>
       <c r="J675" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L675" s="1">
         <v>46297</v>
@@ -44550,7 +44553,7 @@
         <v>219</v>
       </c>
       <c r="O675">
-        <v>18286160</v>
+        <v>18286172</v>
       </c>
       <c r="P675" t="s">
         <v>246</v>
@@ -44591,7 +44594,7 @@
         <v>68</v>
       </c>
       <c r="G676">
-        <v>11684</v>
+        <v>11681</v>
       </c>
       <c r="H676">
         <v>11679</v>
@@ -44600,7 +44603,7 @@
         <v>75</v>
       </c>
       <c r="J676" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L676" s="1">
         <v>46297</v>
@@ -44612,7 +44615,7 @@
         <v>219</v>
       </c>
       <c r="O676">
-        <v>18273889</v>
+        <v>18273886</v>
       </c>
       <c r="P676" t="s">
         <v>246</v>
@@ -44653,7 +44656,7 @@
         <v>68</v>
       </c>
       <c r="G677">
-        <v>11684</v>
+        <v>11681</v>
       </c>
       <c r="H677">
         <v>11679</v>
@@ -44662,7 +44665,7 @@
         <v>75</v>
       </c>
       <c r="J677" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L677" s="1">
         <v>46297</v>
@@ -44671,7 +44674,7 @@
         <v>219</v>
       </c>
       <c r="O677">
-        <v>18286166</v>
+        <v>18286163</v>
       </c>
       <c r="P677" t="s">
         <v>246</v>
@@ -44712,7 +44715,7 @@
         <v>68</v>
       </c>
       <c r="G678">
-        <v>11684</v>
+        <v>11681</v>
       </c>
       <c r="H678">
         <v>11679</v>
@@ -44721,7 +44724,7 @@
         <v>75</v>
       </c>
       <c r="J678" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L678" s="1">
         <v>46297</v>
@@ -44730,7 +44733,7 @@
         <v>219</v>
       </c>
       <c r="O678">
-        <v>18286172</v>
+        <v>18286169</v>
       </c>
       <c r="P678" t="s">
         <v>246</v>
@@ -44771,7 +44774,7 @@
         <v>68</v>
       </c>
       <c r="G679">
-        <v>11681</v>
+        <v>11680</v>
       </c>
       <c r="H679">
         <v>11679</v>
@@ -44780,7 +44783,7 @@
         <v>75</v>
       </c>
       <c r="J679" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L679" s="1">
         <v>46297</v>
@@ -44792,7 +44795,7 @@
         <v>219</v>
       </c>
       <c r="O679">
-        <v>18273886</v>
+        <v>18273885</v>
       </c>
       <c r="P679" t="s">
         <v>246</v>
@@ -44833,7 +44836,7 @@
         <v>68</v>
       </c>
       <c r="G680">
-        <v>11681</v>
+        <v>11680</v>
       </c>
       <c r="H680">
         <v>11679</v>
@@ -44842,7 +44845,7 @@
         <v>75</v>
       </c>
       <c r="J680" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L680" s="1">
         <v>46297</v>
@@ -44851,7 +44854,7 @@
         <v>219</v>
       </c>
       <c r="O680">
-        <v>18286163</v>
+        <v>18286162</v>
       </c>
       <c r="P680" t="s">
         <v>246</v>
@@ -44892,7 +44895,7 @@
         <v>68</v>
       </c>
       <c r="G681">
-        <v>11681</v>
+        <v>11680</v>
       </c>
       <c r="H681">
         <v>11679</v>
@@ -44901,7 +44904,7 @@
         <v>75</v>
       </c>
       <c r="J681" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L681" s="1">
         <v>46297</v>
@@ -44910,7 +44913,7 @@
         <v>219</v>
       </c>
       <c r="O681">
-        <v>18286169</v>
+        <v>18286168</v>
       </c>
       <c r="P681" t="s">
         <v>246</v>
@@ -44951,7 +44954,7 @@
         <v>68</v>
       </c>
       <c r="G682">
-        <v>11680</v>
+        <v>11683</v>
       </c>
       <c r="H682">
         <v>11679</v>
@@ -44960,7 +44963,7 @@
         <v>75</v>
       </c>
       <c r="J682" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L682" s="1">
         <v>46297</v>
@@ -44972,7 +44975,7 @@
         <v>219</v>
       </c>
       <c r="O682">
-        <v>18273885</v>
+        <v>18273888</v>
       </c>
       <c r="P682" t="s">
         <v>246</v>
@@ -45013,7 +45016,7 @@
         <v>68</v>
       </c>
       <c r="G683">
-        <v>11680</v>
+        <v>11683</v>
       </c>
       <c r="H683">
         <v>11679</v>
@@ -45022,7 +45025,7 @@
         <v>75</v>
       </c>
       <c r="J683" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L683" s="1">
         <v>46297</v>
@@ -45031,7 +45034,7 @@
         <v>219</v>
       </c>
       <c r="O683">
-        <v>18286162</v>
+        <v>18286165</v>
       </c>
       <c r="P683" t="s">
         <v>246</v>
@@ -45072,7 +45075,7 @@
         <v>68</v>
       </c>
       <c r="G684">
-        <v>11680</v>
+        <v>11683</v>
       </c>
       <c r="H684">
         <v>11679</v>
@@ -45081,7 +45084,7 @@
         <v>75</v>
       </c>
       <c r="J684" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L684" s="1">
         <v>46297</v>
@@ -45090,7 +45093,7 @@
         <v>219</v>
       </c>
       <c r="O684">
-        <v>18286168</v>
+        <v>18286171</v>
       </c>
       <c r="P684" t="s">
         <v>246</v>
@@ -45131,7 +45134,7 @@
         <v>68</v>
       </c>
       <c r="G685">
-        <v>11683</v>
+        <v>11682</v>
       </c>
       <c r="H685">
         <v>11679</v>
@@ -45140,7 +45143,7 @@
         <v>75</v>
       </c>
       <c r="J685" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="L685" s="1">
         <v>46297</v>
@@ -45152,7 +45155,7 @@
         <v>219</v>
       </c>
       <c r="O685">
-        <v>18273888</v>
+        <v>18273887</v>
       </c>
       <c r="P685" t="s">
         <v>246</v>
@@ -45193,7 +45196,7 @@
         <v>68</v>
       </c>
       <c r="G686">
-        <v>11683</v>
+        <v>11682</v>
       </c>
       <c r="H686">
         <v>11679</v>
@@ -45202,7 +45205,7 @@
         <v>75</v>
       </c>
       <c r="J686" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="L686" s="1">
         <v>46297</v>
@@ -45211,7 +45214,7 @@
         <v>219</v>
       </c>
       <c r="O686">
-        <v>18286165</v>
+        <v>18286164</v>
       </c>
       <c r="P686" t="s">
         <v>246</v>
@@ -45252,7 +45255,7 @@
         <v>68</v>
       </c>
       <c r="G687">
-        <v>11683</v>
+        <v>11682</v>
       </c>
       <c r="H687">
         <v>11679</v>
@@ -45261,7 +45264,7 @@
         <v>75</v>
       </c>
       <c r="J687" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="L687" s="1">
         <v>46297</v>
@@ -45270,7 +45273,7 @@
         <v>219</v>
       </c>
       <c r="O687">
-        <v>18286171</v>
+        <v>18286170</v>
       </c>
       <c r="P687" t="s">
         <v>246</v>
@@ -45288,186 +45291,6 @@
         <v>346</v>
       </c>
       <c r="AG687" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="688" spans="1:33">
-      <c r="A688">
-        <v>7095</v>
-      </c>
-      <c r="B688" t="s">
-        <v>51</v>
-      </c>
-      <c r="C688" t="s">
-        <v>61</v>
-      </c>
-      <c r="D688" t="s">
-        <v>63</v>
-      </c>
-      <c r="E688" t="s">
-        <v>65</v>
-      </c>
-      <c r="F688" t="s">
-        <v>68</v>
-      </c>
-      <c r="G688">
-        <v>11682</v>
-      </c>
-      <c r="H688">
-        <v>11679</v>
-      </c>
-      <c r="I688" t="s">
-        <v>75</v>
-      </c>
-      <c r="J688" t="s">
-        <v>208</v>
-      </c>
-      <c r="L688" s="1">
-        <v>46297</v>
-      </c>
-      <c r="M688" t="s">
-        <v>209</v>
-      </c>
-      <c r="N688" t="s">
-        <v>219</v>
-      </c>
-      <c r="O688">
-        <v>18273887</v>
-      </c>
-      <c r="P688" t="s">
-        <v>246</v>
-      </c>
-      <c r="Q688" t="s">
-        <v>258</v>
-      </c>
-      <c r="S688">
-        <v>0</v>
-      </c>
-      <c r="T688" t="s">
-        <v>264</v>
-      </c>
-      <c r="W688" t="s">
-        <v>345</v>
-      </c>
-      <c r="AG688" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="689" spans="1:33">
-      <c r="A689">
-        <v>7106</v>
-      </c>
-      <c r="B689" t="s">
-        <v>49</v>
-      </c>
-      <c r="C689" t="s">
-        <v>61</v>
-      </c>
-      <c r="D689" t="s">
-        <v>62</v>
-      </c>
-      <c r="E689" t="s">
-        <v>65</v>
-      </c>
-      <c r="F689" t="s">
-        <v>68</v>
-      </c>
-      <c r="G689">
-        <v>11682</v>
-      </c>
-      <c r="H689">
-        <v>11679</v>
-      </c>
-      <c r="I689" t="s">
-        <v>75</v>
-      </c>
-      <c r="J689" t="s">
-        <v>208</v>
-      </c>
-      <c r="L689" s="1">
-        <v>46297</v>
-      </c>
-      <c r="N689" t="s">
-        <v>219</v>
-      </c>
-      <c r="O689">
-        <v>18286164</v>
-      </c>
-      <c r="P689" t="s">
-        <v>246</v>
-      </c>
-      <c r="Q689" t="s">
-        <v>258</v>
-      </c>
-      <c r="S689">
-        <v>0</v>
-      </c>
-      <c r="T689" t="s">
-        <v>271</v>
-      </c>
-      <c r="W689" t="s">
-        <v>346</v>
-      </c>
-      <c r="AG689" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="690" spans="1:33">
-      <c r="A690">
-        <v>7107</v>
-      </c>
-      <c r="B690" t="s">
-        <v>50</v>
-      </c>
-      <c r="C690" t="s">
-        <v>61</v>
-      </c>
-      <c r="D690" t="s">
-        <v>63</v>
-      </c>
-      <c r="E690" t="s">
-        <v>65</v>
-      </c>
-      <c r="F690" t="s">
-        <v>68</v>
-      </c>
-      <c r="G690">
-        <v>11682</v>
-      </c>
-      <c r="H690">
-        <v>11679</v>
-      </c>
-      <c r="I690" t="s">
-        <v>75</v>
-      </c>
-      <c r="J690" t="s">
-        <v>208</v>
-      </c>
-      <c r="L690" s="1">
-        <v>46297</v>
-      </c>
-      <c r="N690" t="s">
-        <v>219</v>
-      </c>
-      <c r="O690">
-        <v>18286170</v>
-      </c>
-      <c r="P690" t="s">
-        <v>246</v>
-      </c>
-      <c r="Q690" t="s">
-        <v>258</v>
-      </c>
-      <c r="S690">
-        <v>0</v>
-      </c>
-      <c r="T690" t="s">
-        <v>271</v>
-      </c>
-      <c r="W690" t="s">
-        <v>346</v>
-      </c>
-      <c r="AG690" t="s">
         <v>350</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-08 09:44
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -867,10 +867,6 @@
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/10/2026 - Data Comentário: 05/10/2026 17:05</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/10/2026 
-Previsão de conclusão em 08/10 - Data Comentário: 05/10/2026 17:59</t>
-  </si>
-  <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/10/2026 - Data Comentário: 05/10/2026 17:07</t>
   </si>
   <si>
@@ -881,6 +877,9 @@
   </si>
   <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-07/10/2026 10:49:56.. - Data Comentário: 07/10/2026 10:44</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-08/10/2026 08:54:54.. - Data Comentário: 08/10/2026 08:49</t>
   </si>
   <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-06/10/2026 14:49:58.. - Data Comentário: 06/10/2026 14:44</t>
@@ -1024,6 +1023,10 @@
     <t>Imposto enviado via SCI Report - Data Comentário: 07/10/2026 09:22</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/10/2026 
+Previsão de conclusão em 08/10 - Data Comentário: 05/10/2026 17:59</t>
+  </si>
+  <si>
     <t>Imposto enviado via SCI Report - Data Comentário: 06/10/2026 12:39</t>
   </si>
   <si>
@@ -1037,9 +1040,6 @@
   </si>
   <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1792]. - Data Comentário: 01/10/2026 09:00</t>
-  </si>
-  <si>
-    <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1867]. - Data Comentário: 01/10/2026 09:01</t>
   </si>
   <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1793]. - Data Comentário: 01/10/2026 09:02</t>
@@ -3601,22 +3601,22 @@
     </row>
     <row r="32" spans="1:34">
       <c r="A32">
-        <v>6548</v>
+        <v>6962</v>
       </c>
       <c r="B32" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C32" t="s">
         <v>57</v>
       </c>
       <c r="D32" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E32" t="s">
         <v>61</v>
       </c>
       <c r="F32" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G32">
         <v>1867</v>
@@ -3640,10 +3640,10 @@
         <v>221</v>
       </c>
       <c r="O32">
-        <v>17988544</v>
+        <v>18186954</v>
       </c>
       <c r="P32" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="Q32" t="s">
         <v>257</v>
@@ -3652,10 +3652,7 @@
         <v>-1</v>
       </c>
       <c r="T32" t="s">
-        <v>261</v>
-      </c>
-      <c r="V32" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="W32" t="s">
         <v>283</v>
@@ -3672,16 +3669,16 @@
     </row>
     <row r="33" spans="1:34">
       <c r="A33">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C33" t="s">
         <v>57</v>
       </c>
       <c r="D33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E33" t="s">
         <v>61</v>
@@ -3690,49 +3687,43 @@
         <v>63</v>
       </c>
       <c r="G33">
-        <v>1867</v>
+        <v>6886</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>1862</v>
       </c>
       <c r="I33" t="s">
         <v>67</v>
       </c>
       <c r="J33" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L33" s="1">
-        <v>46304</v>
-      </c>
-      <c r="M33" t="s">
-        <v>208</v>
+        <v>46308</v>
       </c>
       <c r="N33" t="s">
         <v>221</v>
       </c>
       <c r="O33">
-        <v>18186954</v>
+        <v>18214908</v>
       </c>
       <c r="P33" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Q33" t="s">
         <v>257</v>
       </c>
       <c r="S33">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="T33" t="s">
-        <v>267</v>
-      </c>
-      <c r="W33" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
       <c r="AA33">
         <v>0</v>
       </c>
       <c r="AG33" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AH33" t="s">
         <v>371</v>
@@ -3740,10 +3731,10 @@
     </row>
     <row r="34" spans="1:34">
       <c r="A34">
-        <v>6949</v>
+        <v>6627</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C34" t="s">
         <v>57</v>
@@ -3752,31 +3743,31 @@
         <v>59</v>
       </c>
       <c r="E34" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F34" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G34">
-        <v>6886</v>
+        <v>10674</v>
       </c>
       <c r="H34">
-        <v>1862</v>
+        <v>0</v>
       </c>
       <c r="I34" t="s">
         <v>67</v>
       </c>
       <c r="J34" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L34" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N34" t="s">
         <v>221</v>
       </c>
       <c r="O34">
-        <v>18214908</v>
+        <v>17968446</v>
       </c>
       <c r="P34" t="s">
         <v>235</v>
@@ -3785,10 +3776,13 @@
         <v>257</v>
       </c>
       <c r="S34">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="T34" t="s">
-        <v>265</v>
+        <v>262</v>
+      </c>
+      <c r="V34" t="s">
+        <v>274</v>
       </c>
       <c r="AA34">
         <v>0</v>
@@ -3802,22 +3796,22 @@
     </row>
     <row r="35" spans="1:34">
       <c r="A35">
-        <v>6627</v>
+        <v>6945</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C35" t="s">
         <v>57</v>
       </c>
       <c r="D35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G35">
         <v>10674</v>
@@ -3838,7 +3832,7 @@
         <v>221</v>
       </c>
       <c r="O35">
-        <v>17968446</v>
+        <v>18220234</v>
       </c>
       <c r="P35" t="s">
         <v>235</v>
@@ -3850,10 +3844,7 @@
         <v>-7</v>
       </c>
       <c r="T35" t="s">
-        <v>262</v>
-      </c>
-      <c r="V35" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="AA35">
         <v>0</v>
@@ -3867,16 +3858,16 @@
     </row>
     <row r="36" spans="1:34">
       <c r="A36">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B36" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
         <v>57</v>
       </c>
       <c r="D36" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E36" t="s">
         <v>61</v>
@@ -3903,7 +3894,7 @@
         <v>221</v>
       </c>
       <c r="O36">
-        <v>18220234</v>
+        <v>18214920</v>
       </c>
       <c r="P36" t="s">
         <v>235</v>
@@ -3915,7 +3906,7 @@
         <v>-7</v>
       </c>
       <c r="T36" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="AA36">
         <v>0</v>
@@ -3929,10 +3920,10 @@
     </row>
     <row r="37" spans="1:34">
       <c r="A37">
-        <v>6949</v>
+        <v>6486</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C37" t="s">
         <v>57</v>
@@ -3944,19 +3935,19 @@
         <v>61</v>
       </c>
       <c r="F37" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G37">
-        <v>10674</v>
+        <v>1837</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I37" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J37" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L37" s="1">
         <v>46310</v>
@@ -3965,10 +3956,10 @@
         <v>221</v>
       </c>
       <c r="O37">
-        <v>18214920</v>
+        <v>16975984</v>
       </c>
       <c r="P37" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="Q37" t="s">
         <v>257</v>
@@ -3977,7 +3968,10 @@
         <v>-7</v>
       </c>
       <c r="T37" t="s">
-        <v>265</v>
+        <v>266</v>
+      </c>
+      <c r="V37" t="s">
+        <v>274</v>
       </c>
       <c r="AA37">
         <v>0</v>
@@ -3986,21 +3980,21 @@
         <v>378</v>
       </c>
       <c r="AH37" t="s">
-        <v>371</v>
+        <v>384</v>
       </c>
     </row>
     <row r="38" spans="1:34">
       <c r="A38">
-        <v>6486</v>
+        <v>6779</v>
       </c>
       <c r="B38" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
         <v>57</v>
       </c>
       <c r="D38" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E38" t="s">
         <v>61</v>
@@ -4009,25 +4003,25 @@
         <v>64</v>
       </c>
       <c r="G38">
-        <v>1837</v>
+        <v>11636</v>
       </c>
       <c r="H38">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I38" t="s">
         <v>68</v>
       </c>
       <c r="J38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L38" s="1">
-        <v>46310</v>
+        <v>46303</v>
       </c>
       <c r="N38" t="s">
         <v>221</v>
       </c>
       <c r="O38">
-        <v>16975984</v>
+        <v>18085089</v>
       </c>
       <c r="P38" t="s">
         <v>238</v>
@@ -4036,10 +4030,10 @@
         <v>257</v>
       </c>
       <c r="S38">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="T38" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="V38" t="s">
         <v>274</v>
@@ -4056,10 +4050,10 @@
     </row>
     <row r="39" spans="1:34">
       <c r="A39">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C39" t="s">
         <v>57</v>
@@ -4074,7 +4068,7 @@
         <v>64</v>
       </c>
       <c r="G39">
-        <v>11636</v>
+        <v>6298</v>
       </c>
       <c r="H39">
         <v>0</v>
@@ -4083,16 +4077,16 @@
         <v>68</v>
       </c>
       <c r="J39" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="L39" s="1">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="N39" t="s">
         <v>221</v>
       </c>
       <c r="O39">
-        <v>18085089</v>
+        <v>17949010</v>
       </c>
       <c r="P39" t="s">
         <v>238</v>
@@ -4101,19 +4095,16 @@
         <v>257</v>
       </c>
       <c r="S39">
-        <v>0</v>
+        <v>-7</v>
       </c>
       <c r="T39" t="s">
         <v>264</v>
       </c>
-      <c r="V39" t="s">
-        <v>274</v>
-      </c>
       <c r="AA39">
         <v>0</v>
       </c>
       <c r="AG39" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="AH39" t="s">
         <v>384</v>
@@ -4121,16 +4112,16 @@
     </row>
     <row r="40" spans="1:34">
       <c r="A40">
-        <v>6705</v>
+        <v>5417</v>
       </c>
       <c r="B40" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C40" t="s">
         <v>57</v>
       </c>
       <c r="D40" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E40" t="s">
         <v>61</v>
@@ -4139,7 +4130,7 @@
         <v>64</v>
       </c>
       <c r="G40">
-        <v>6298</v>
+        <v>6806</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -4148,16 +4139,16 @@
         <v>68</v>
       </c>
       <c r="J40" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L40" s="1">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="N40" t="s">
         <v>221</v>
       </c>
       <c r="O40">
-        <v>17949010</v>
+        <v>17399231</v>
       </c>
       <c r="P40" t="s">
         <v>238</v>
@@ -4166,10 +4157,10 @@
         <v>257</v>
       </c>
       <c r="S40">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="T40" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="AA40">
         <v>0</v>
@@ -4183,16 +4174,16 @@
     </row>
     <row r="41" spans="1:34">
       <c r="A41">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B41" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C41" t="s">
         <v>57</v>
       </c>
       <c r="D41" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E41" t="s">
         <v>61</v>
@@ -4219,7 +4210,7 @@
         <v>221</v>
       </c>
       <c r="O41">
-        <v>17399231</v>
+        <v>16962309</v>
       </c>
       <c r="P41" t="s">
         <v>238</v>
@@ -4231,7 +4222,7 @@
         <v>-5</v>
       </c>
       <c r="T41" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="AA41">
         <v>0</v>
@@ -4245,16 +4236,16 @@
     </row>
     <row r="42" spans="1:34">
       <c r="A42">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B42" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C42" t="s">
         <v>57</v>
       </c>
       <c r="D42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E42" t="s">
         <v>61</v>
@@ -4281,7 +4272,7 @@
         <v>221</v>
       </c>
       <c r="O42">
-        <v>16962309</v>
+        <v>16976188</v>
       </c>
       <c r="P42" t="s">
         <v>238</v>
@@ -4293,7 +4284,10 @@
         <v>-5</v>
       </c>
       <c r="T42" t="s">
-        <v>268</v>
+        <v>266</v>
+      </c>
+      <c r="V42" t="s">
+        <v>274</v>
       </c>
       <c r="AA42">
         <v>0</v>
@@ -4307,16 +4301,16 @@
     </row>
     <row r="43" spans="1:34">
       <c r="A43">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C43" t="s">
         <v>57</v>
       </c>
       <c r="D43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E43" t="s">
         <v>61</v>
@@ -4343,7 +4337,7 @@
         <v>221</v>
       </c>
       <c r="O43">
-        <v>16976188</v>
+        <v>17948859</v>
       </c>
       <c r="P43" t="s">
         <v>238</v>
@@ -4355,10 +4349,7 @@
         <v>-5</v>
       </c>
       <c r="T43" t="s">
-        <v>266</v>
-      </c>
-      <c r="V43" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="AA43">
         <v>0</v>
@@ -4372,16 +4363,16 @@
     </row>
     <row r="44" spans="1:34">
       <c r="A44">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C44" t="s">
         <v>57</v>
       </c>
       <c r="D44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E44" t="s">
         <v>61</v>
@@ -4408,7 +4399,7 @@
         <v>221</v>
       </c>
       <c r="O44">
-        <v>17948859</v>
+        <v>18085298</v>
       </c>
       <c r="P44" t="s">
         <v>238</v>
@@ -4420,7 +4411,10 @@
         <v>-5</v>
       </c>
       <c r="T44" t="s">
-        <v>263</v>
+        <v>264</v>
+      </c>
+      <c r="V44" t="s">
+        <v>274</v>
       </c>
       <c r="AA44">
         <v>0</v>
@@ -4434,16 +4428,16 @@
     </row>
     <row r="45" spans="1:34">
       <c r="A45">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B45" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C45" t="s">
         <v>57</v>
       </c>
       <c r="D45" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E45" t="s">
         <v>61</v>
@@ -4470,7 +4464,7 @@
         <v>221</v>
       </c>
       <c r="O45">
-        <v>18085298</v>
+        <v>17949030</v>
       </c>
       <c r="P45" t="s">
         <v>238</v>
@@ -4484,9 +4478,6 @@
       <c r="T45" t="s">
         <v>264</v>
       </c>
-      <c r="V45" t="s">
-        <v>274</v>
-      </c>
       <c r="AA45">
         <v>0</v>
       </c>
@@ -4499,10 +4490,10 @@
     </row>
     <row r="46" spans="1:34">
       <c r="A46">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B46" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C46" t="s">
         <v>57</v>
@@ -4535,7 +4526,7 @@
         <v>221</v>
       </c>
       <c r="O46">
-        <v>17949030</v>
+        <v>18085067</v>
       </c>
       <c r="P46" t="s">
         <v>238</v>
@@ -4549,6 +4540,9 @@
       <c r="T46" t="s">
         <v>264</v>
       </c>
+      <c r="V46" t="s">
+        <v>274</v>
+      </c>
       <c r="AA46">
         <v>0</v>
       </c>
@@ -4561,16 +4555,16 @@
     </row>
     <row r="47" spans="1:34">
       <c r="A47">
-        <v>6779</v>
+        <v>5417</v>
       </c>
       <c r="B47" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C47" t="s">
         <v>57</v>
       </c>
       <c r="D47" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E47" t="s">
         <v>61</v>
@@ -4579,25 +4573,25 @@
         <v>64</v>
       </c>
       <c r="G47">
-        <v>6806</v>
+        <v>7884</v>
       </c>
       <c r="H47">
-        <v>0</v>
+        <v>9114</v>
       </c>
       <c r="I47" t="s">
         <v>68</v>
       </c>
       <c r="J47" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="L47" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N47" t="s">
         <v>221</v>
       </c>
       <c r="O47">
-        <v>18085067</v>
+        <v>17399341</v>
       </c>
       <c r="P47" t="s">
         <v>238</v>
@@ -4606,19 +4600,19 @@
         <v>257</v>
       </c>
       <c r="S47">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="T47" t="s">
-        <v>264</v>
-      </c>
-      <c r="V47" t="s">
-        <v>274</v>
+        <v>260</v>
+      </c>
+      <c r="W47" t="s">
+        <v>284</v>
       </c>
       <c r="AA47">
         <v>0</v>
       </c>
       <c r="AG47" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="AH47" t="s">
         <v>384</v>
@@ -4626,16 +4620,16 @@
     </row>
     <row r="48" spans="1:34">
       <c r="A48">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B48" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C48" t="s">
         <v>57</v>
       </c>
       <c r="D48" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E48" t="s">
         <v>61</v>
@@ -4644,25 +4638,25 @@
         <v>64</v>
       </c>
       <c r="G48">
-        <v>7884</v>
+        <v>1792</v>
       </c>
       <c r="H48">
-        <v>9114</v>
+        <v>0</v>
       </c>
       <c r="I48" t="s">
         <v>68</v>
       </c>
       <c r="J48" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="L48" s="1">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="N48" t="s">
         <v>221</v>
       </c>
       <c r="O48">
-        <v>17399341</v>
+        <v>16962152</v>
       </c>
       <c r="P48" t="s">
         <v>238</v>
@@ -4671,19 +4665,16 @@
         <v>257</v>
       </c>
       <c r="S48">
-        <v>-7</v>
+        <v>-1</v>
       </c>
       <c r="T48" t="s">
-        <v>260</v>
-      </c>
-      <c r="W48" t="s">
-        <v>285</v>
+        <v>268</v>
       </c>
       <c r="AA48">
         <v>0</v>
       </c>
       <c r="AG48" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="AH48" t="s">
         <v>384</v>
@@ -4691,10 +4682,10 @@
     </row>
     <row r="49" spans="1:34">
       <c r="A49">
-        <v>6404</v>
+        <v>6703</v>
       </c>
       <c r="B49" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C49" t="s">
         <v>57</v>
@@ -4727,7 +4718,7 @@
         <v>221</v>
       </c>
       <c r="O49">
-        <v>16962152</v>
+        <v>17948757</v>
       </c>
       <c r="P49" t="s">
         <v>238</v>
@@ -4739,7 +4730,7 @@
         <v>-1</v>
       </c>
       <c r="T49" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="AA49">
         <v>0</v>
@@ -4753,16 +4744,16 @@
     </row>
     <row r="50" spans="1:34">
       <c r="A50">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B50" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C50" t="s">
         <v>57</v>
       </c>
       <c r="D50" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E50" t="s">
         <v>61</v>
@@ -4789,7 +4780,7 @@
         <v>221</v>
       </c>
       <c r="O50">
-        <v>17948757</v>
+        <v>18085144</v>
       </c>
       <c r="P50" t="s">
         <v>238</v>
@@ -4801,7 +4792,10 @@
         <v>-1</v>
       </c>
       <c r="T50" t="s">
-        <v>263</v>
+        <v>264</v>
+      </c>
+      <c r="V50" t="s">
+        <v>274</v>
       </c>
       <c r="AA50">
         <v>0</v>
@@ -4815,16 +4809,16 @@
     </row>
     <row r="51" spans="1:34">
       <c r="A51">
-        <v>6704</v>
+        <v>6404</v>
       </c>
       <c r="B51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C51" t="s">
         <v>57</v>
       </c>
       <c r="D51" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E51" t="s">
         <v>61</v>
@@ -4833,7 +4827,7 @@
         <v>64</v>
       </c>
       <c r="G51">
-        <v>1792</v>
+        <v>1793</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -4842,7 +4836,7 @@
         <v>68</v>
       </c>
       <c r="J51" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L51" s="1">
         <v>46304</v>
@@ -4851,7 +4845,7 @@
         <v>221</v>
       </c>
       <c r="O51">
-        <v>18085144</v>
+        <v>16962162</v>
       </c>
       <c r="P51" t="s">
         <v>238</v>
@@ -4863,10 +4857,7 @@
         <v>-1</v>
       </c>
       <c r="T51" t="s">
-        <v>264</v>
-      </c>
-      <c r="V51" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="AA51">
         <v>0</v>
@@ -4880,16 +4871,16 @@
     </row>
     <row r="52" spans="1:34">
       <c r="A52">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B52" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C52" t="s">
         <v>57</v>
       </c>
       <c r="D52" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E52" t="s">
         <v>61</v>
@@ -4916,7 +4907,7 @@
         <v>221</v>
       </c>
       <c r="O52">
-        <v>16962162</v>
+        <v>16975953</v>
       </c>
       <c r="P52" t="s">
         <v>238</v>
@@ -4928,7 +4919,10 @@
         <v>-1</v>
       </c>
       <c r="T52" t="s">
-        <v>268</v>
+        <v>266</v>
+      </c>
+      <c r="V52" t="s">
+        <v>274</v>
       </c>
       <c r="AA52">
         <v>0</v>
@@ -4942,16 +4936,16 @@
     </row>
     <row r="53" spans="1:34">
       <c r="A53">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C53" t="s">
         <v>57</v>
       </c>
       <c r="D53" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E53" t="s">
         <v>61</v>
@@ -4978,7 +4972,7 @@
         <v>221</v>
       </c>
       <c r="O53">
-        <v>16975953</v>
+        <v>17948767</v>
       </c>
       <c r="P53" t="s">
         <v>238</v>
@@ -4990,10 +4984,7 @@
         <v>-1</v>
       </c>
       <c r="T53" t="s">
-        <v>266</v>
-      </c>
-      <c r="V53" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="AA53">
         <v>0</v>
@@ -5007,16 +4998,16 @@
     </row>
     <row r="54" spans="1:34">
       <c r="A54">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C54" t="s">
         <v>57</v>
       </c>
       <c r="D54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E54" t="s">
         <v>61</v>
@@ -5043,7 +5034,7 @@
         <v>221</v>
       </c>
       <c r="O54">
-        <v>17948767</v>
+        <v>18085155</v>
       </c>
       <c r="P54" t="s">
         <v>238</v>
@@ -5055,7 +5046,10 @@
         <v>-1</v>
       </c>
       <c r="T54" t="s">
-        <v>263</v>
+        <v>264</v>
+      </c>
+      <c r="V54" t="s">
+        <v>274</v>
       </c>
       <c r="AA54">
         <v>0</v>
@@ -5069,16 +5063,16 @@
     </row>
     <row r="55" spans="1:34">
       <c r="A55">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B55" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C55" t="s">
         <v>57</v>
       </c>
       <c r="D55" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E55" t="s">
         <v>61</v>
@@ -5105,7 +5099,7 @@
         <v>221</v>
       </c>
       <c r="O55">
-        <v>18085155</v>
+        <v>17948929</v>
       </c>
       <c r="P55" t="s">
         <v>238</v>
@@ -5119,9 +5113,6 @@
       <c r="T55" t="s">
         <v>264</v>
       </c>
-      <c r="V55" t="s">
-        <v>274</v>
-      </c>
       <c r="AA55">
         <v>0</v>
       </c>
@@ -5134,10 +5125,10 @@
     </row>
     <row r="56" spans="1:34">
       <c r="A56">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B56" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
         <v>57</v>
@@ -5170,7 +5161,7 @@
         <v>221</v>
       </c>
       <c r="O56">
-        <v>17948929</v>
+        <v>18084956</v>
       </c>
       <c r="P56" t="s">
         <v>238</v>
@@ -5184,6 +5175,9 @@
       <c r="T56" t="s">
         <v>264</v>
       </c>
+      <c r="V56" t="s">
+        <v>274</v>
+      </c>
       <c r="AA56">
         <v>0</v>
       </c>
@@ -5196,16 +5190,16 @@
     </row>
     <row r="57" spans="1:34">
       <c r="A57">
-        <v>6779</v>
+        <v>6703</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C57" t="s">
         <v>57</v>
       </c>
       <c r="D57" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E57" t="s">
         <v>61</v>
@@ -5214,7 +5208,7 @@
         <v>64</v>
       </c>
       <c r="G57">
-        <v>1793</v>
+        <v>1796</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -5223,16 +5217,16 @@
         <v>68</v>
       </c>
       <c r="J57" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="L57" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="N57" t="s">
         <v>221</v>
       </c>
       <c r="O57">
-        <v>18084956</v>
+        <v>18073099</v>
       </c>
       <c r="P57" t="s">
         <v>238</v>
@@ -5241,19 +5235,16 @@
         <v>257</v>
       </c>
       <c r="S57">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T57" t="s">
-        <v>264</v>
-      </c>
-      <c r="V57" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="AA57">
         <v>0</v>
       </c>
       <c r="AG57" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AH57" t="s">
         <v>384</v>
@@ -5261,16 +5252,16 @@
     </row>
     <row r="58" spans="1:34">
       <c r="A58">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B58" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C58" t="s">
         <v>57</v>
       </c>
       <c r="D58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E58" t="s">
         <v>61</v>
@@ -5279,16 +5270,16 @@
         <v>64</v>
       </c>
       <c r="G58">
-        <v>1796</v>
+        <v>6884</v>
       </c>
       <c r="H58">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I58" t="s">
         <v>68</v>
       </c>
       <c r="J58" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="L58" s="1">
         <v>46303</v>
@@ -5297,7 +5288,7 @@
         <v>221</v>
       </c>
       <c r="O58">
-        <v>18073099</v>
+        <v>16976208</v>
       </c>
       <c r="P58" t="s">
         <v>238</v>
@@ -5309,7 +5300,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="s">
-        <v>263</v>
+        <v>266</v>
+      </c>
+      <c r="V58" t="s">
+        <v>274</v>
       </c>
       <c r="AA58">
         <v>0</v>
@@ -5323,16 +5317,16 @@
     </row>
     <row r="59" spans="1:34">
       <c r="A59">
-        <v>6486</v>
+        <v>6705</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C59" t="s">
         <v>57</v>
       </c>
       <c r="D59" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E59" t="s">
         <v>61</v>
@@ -5359,7 +5353,7 @@
         <v>221</v>
       </c>
       <c r="O59">
-        <v>16976208</v>
+        <v>17949040</v>
       </c>
       <c r="P59" t="s">
         <v>238</v>
@@ -5371,10 +5365,7 @@
         <v>0</v>
       </c>
       <c r="T59" t="s">
-        <v>266</v>
-      </c>
-      <c r="V59" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="AA59">
         <v>0</v>
@@ -5406,7 +5397,7 @@
         <v>64</v>
       </c>
       <c r="G60">
-        <v>6884</v>
+        <v>6294</v>
       </c>
       <c r="H60">
         <v>1788</v>
@@ -5415,16 +5406,16 @@
         <v>68</v>
       </c>
       <c r="J60" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="L60" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="N60" t="s">
         <v>221</v>
       </c>
       <c r="O60">
-        <v>17949040</v>
+        <v>17949000</v>
       </c>
       <c r="P60" t="s">
         <v>238</v>
@@ -5433,7 +5424,7 @@
         <v>257</v>
       </c>
       <c r="S60">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="T60" t="s">
         <v>264</v>
@@ -5450,16 +5441,16 @@
     </row>
     <row r="61" spans="1:34">
       <c r="A61">
-        <v>6705</v>
+        <v>6486</v>
       </c>
       <c r="B61" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C61" t="s">
         <v>57</v>
       </c>
       <c r="D61" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E61" t="s">
         <v>61</v>
@@ -5468,16 +5459,16 @@
         <v>64</v>
       </c>
       <c r="G61">
-        <v>6294</v>
+        <v>11303</v>
       </c>
       <c r="H61">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I61" t="s">
         <v>68</v>
       </c>
       <c r="J61" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L61" s="1">
         <v>46308</v>
@@ -5486,7 +5477,7 @@
         <v>221</v>
       </c>
       <c r="O61">
-        <v>17949000</v>
+        <v>16976352</v>
       </c>
       <c r="P61" t="s">
         <v>238</v>
@@ -5498,7 +5489,10 @@
         <v>-5</v>
       </c>
       <c r="T61" t="s">
-        <v>264</v>
+        <v>266</v>
+      </c>
+      <c r="V61" t="s">
+        <v>274</v>
       </c>
       <c r="AA61">
         <v>0</v>
@@ -5512,10 +5506,10 @@
     </row>
     <row r="62" spans="1:34">
       <c r="A62">
-        <v>6486</v>
+        <v>6949</v>
       </c>
       <c r="B62" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C62" t="s">
         <v>57</v>
@@ -5527,66 +5521,63 @@
         <v>61</v>
       </c>
       <c r="F62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G62">
-        <v>11303</v>
+        <v>950</v>
       </c>
       <c r="H62">
         <v>0</v>
       </c>
       <c r="I62" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J62" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L62" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="N62" t="s">
         <v>221</v>
       </c>
       <c r="O62">
-        <v>16976352</v>
+        <v>18178133</v>
       </c>
       <c r="P62" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q62" t="s">
         <v>257</v>
       </c>
       <c r="S62">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="T62" t="s">
-        <v>266</v>
-      </c>
-      <c r="V62" t="s">
-        <v>274</v>
+        <v>265</v>
+      </c>
+      <c r="W62" t="s">
+        <v>285</v>
       </c>
       <c r="AA62">
         <v>0</v>
       </c>
       <c r="AG62" t="s">
-        <v>378</v>
-      </c>
-      <c r="AH62" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="63" spans="1:34">
       <c r="A63">
-        <v>6949</v>
+        <v>6963</v>
       </c>
       <c r="B63" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C63" t="s">
         <v>57</v>
       </c>
       <c r="D63" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E63" t="s">
         <v>61</v>
@@ -5613,7 +5604,7 @@
         <v>221</v>
       </c>
       <c r="O63">
-        <v>18178133</v>
+        <v>18188624</v>
       </c>
       <c r="P63" t="s">
         <v>239</v>
@@ -5625,7 +5616,7 @@
         <v>-1</v>
       </c>
       <c r="T63" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="W63" t="s">
         <v>286</v>
@@ -5639,25 +5630,25 @@
     </row>
     <row r="64" spans="1:34">
       <c r="A64">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B64" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C64" t="s">
         <v>57</v>
       </c>
       <c r="D64" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E64" t="s">
         <v>61</v>
       </c>
       <c r="F64" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G64">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="H64">
         <v>0</v>
@@ -5666,7 +5657,7 @@
         <v>69</v>
       </c>
       <c r="J64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L64" s="1">
         <v>46304</v>
@@ -5675,7 +5666,7 @@
         <v>221</v>
       </c>
       <c r="O64">
-        <v>18188624</v>
+        <v>17222406</v>
       </c>
       <c r="P64" t="s">
         <v>239</v>
@@ -5687,7 +5678,10 @@
         <v>-1</v>
       </c>
       <c r="T64" t="s">
-        <v>267</v>
+        <v>261</v>
+      </c>
+      <c r="V64" t="s">
+        <v>274</v>
       </c>
       <c r="W64" t="s">
         <v>287</v>
@@ -14712,10 +14706,10 @@
     </row>
     <row r="192" spans="1:34">
       <c r="A192">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B192" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C192" t="s">
         <v>57</v>
@@ -14724,7 +14718,7 @@
         <v>59</v>
       </c>
       <c r="E192" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F192" t="s">
         <v>64</v>
@@ -14744,26 +14738,29 @@
       <c r="L192" s="1">
         <v>46304</v>
       </c>
+      <c r="M192" t="s">
+        <v>208</v>
+      </c>
       <c r="N192" t="s">
         <v>221</v>
       </c>
       <c r="O192">
-        <v>17968380</v>
+        <v>17988544</v>
       </c>
       <c r="P192" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Q192" t="s">
         <v>258</v>
       </c>
       <c r="R192" s="1">
-        <v>46301.53482881944</v>
+        <v>46303.37146987268</v>
       </c>
       <c r="S192">
         <v>-1</v>
       </c>
       <c r="T192" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="V192" t="s">
         <v>274</v>
@@ -14775,7 +14772,7 @@
         <v>0</v>
       </c>
       <c r="AB192" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AG192" t="s">
         <v>379</v>
@@ -14786,22 +14783,22 @@
     </row>
     <row r="193" spans="1:34">
       <c r="A193">
-        <v>6945</v>
+        <v>6627</v>
       </c>
       <c r="B193" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C193" t="s">
         <v>57</v>
       </c>
       <c r="D193" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E193" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F193" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G193">
         <v>1867</v>
@@ -14818,14 +14815,11 @@
       <c r="L193" s="1">
         <v>46304</v>
       </c>
-      <c r="M193" t="s">
-        <v>211</v>
-      </c>
       <c r="N193" t="s">
         <v>221</v>
       </c>
       <c r="O193">
-        <v>18220183</v>
+        <v>17968380</v>
       </c>
       <c r="P193" t="s">
         <v>235</v>
@@ -14834,13 +14828,16 @@
         <v>258</v>
       </c>
       <c r="R193" s="1">
-        <v>46301.61803621528</v>
+        <v>46301.53482881944</v>
       </c>
       <c r="S193">
         <v>-1</v>
       </c>
       <c r="T193" t="s">
-        <v>259</v>
+        <v>262</v>
+      </c>
+      <c r="V193" t="s">
+        <v>274</v>
       </c>
       <c r="W193" t="s">
         <v>331</v>
@@ -14860,16 +14857,16 @@
     </row>
     <row r="194" spans="1:34">
       <c r="A194">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B194" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C194" t="s">
         <v>57</v>
       </c>
       <c r="D194" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E194" t="s">
         <v>61</v>
@@ -14892,11 +14889,14 @@
       <c r="L194" s="1">
         <v>46304</v>
       </c>
+      <c r="M194" t="s">
+        <v>211</v>
+      </c>
       <c r="N194" t="s">
         <v>221</v>
       </c>
       <c r="O194">
-        <v>18214860</v>
+        <v>18220183</v>
       </c>
       <c r="P194" t="s">
         <v>235</v>
@@ -14905,13 +14905,13 @@
         <v>258</v>
       </c>
       <c r="R194" s="1">
-        <v>46301.68910333333</v>
+        <v>46301.61803621528</v>
       </c>
       <c r="S194">
         <v>-1</v>
       </c>
       <c r="T194" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="W194" t="s">
         <v>332</v>
@@ -14931,16 +14931,16 @@
     </row>
     <row r="195" spans="1:34">
       <c r="A195">
-        <v>6963</v>
+        <v>6949</v>
       </c>
       <c r="B195" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C195" t="s">
         <v>57</v>
       </c>
       <c r="D195" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E195" t="s">
         <v>61</v>
@@ -14967,22 +14967,22 @@
         <v>221</v>
       </c>
       <c r="O195">
-        <v>18187220</v>
+        <v>18214860</v>
       </c>
       <c r="P195" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="Q195" t="s">
         <v>258</v>
       </c>
       <c r="R195" s="1">
-        <v>46302.40335295139</v>
+        <v>46301.68910333333</v>
       </c>
       <c r="S195">
         <v>-1</v>
       </c>
       <c r="T195" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="W195" t="s">
         <v>333</v>
@@ -14991,7 +14991,7 @@
         <v>0</v>
       </c>
       <c r="AB195" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="AG195" t="s">
         <v>379</v>
@@ -15002,70 +15002,73 @@
     </row>
     <row r="196" spans="1:34">
       <c r="A196">
-        <v>5417</v>
+        <v>6963</v>
       </c>
       <c r="B196" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C196" t="s">
         <v>57</v>
       </c>
       <c r="D196" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E196" t="s">
         <v>61</v>
       </c>
       <c r="F196" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G196">
-        <v>6883</v>
+        <v>1867</v>
       </c>
       <c r="H196">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I196" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J196" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="L196" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="N196" t="s">
         <v>221</v>
       </c>
       <c r="O196">
-        <v>17399251</v>
+        <v>18187220</v>
       </c>
       <c r="P196" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Q196" t="s">
         <v>258</v>
       </c>
       <c r="R196" s="1">
-        <v>46297.37673402778</v>
+        <v>46302.40335295139</v>
       </c>
       <c r="S196">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="T196" t="s">
-        <v>260</v>
+        <v>267</v>
+      </c>
+      <c r="W196" t="s">
+        <v>334</v>
       </c>
       <c r="AA196">
         <v>0</v>
       </c>
       <c r="AB196" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AG196" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="AH196" t="s">
-        <v>384</v>
+        <v>371</v>
       </c>
     </row>
     <row r="197" spans="1:34">
@@ -15088,7 +15091,7 @@
         <v>64</v>
       </c>
       <c r="G197">
-        <v>1836</v>
+        <v>6883</v>
       </c>
       <c r="H197">
         <v>1788</v>
@@ -15097,16 +15100,16 @@
         <v>68</v>
       </c>
       <c r="J197" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="L197" s="1">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="N197" t="s">
         <v>221</v>
       </c>
       <c r="O197">
-        <v>17398976</v>
+        <v>17399251</v>
       </c>
       <c r="P197" t="s">
         <v>238</v>
@@ -15115,10 +15118,10 @@
         <v>258</v>
       </c>
       <c r="R197" s="1">
-        <v>46297.37618915509</v>
+        <v>46297.37673402778</v>
       </c>
       <c r="S197">
-        <v>3</v>
+        <v>-5</v>
       </c>
       <c r="T197" t="s">
         <v>260</v>
@@ -15138,10 +15141,10 @@
     </row>
     <row r="198" spans="1:34">
       <c r="A198">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B198" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C198" t="s">
         <v>57</v>
@@ -15174,7 +15177,7 @@
         <v>221</v>
       </c>
       <c r="O198">
-        <v>18155319</v>
+        <v>17398976</v>
       </c>
       <c r="P198" t="s">
         <v>238</v>
@@ -15183,16 +15186,13 @@
         <v>258</v>
       </c>
       <c r="R198" s="1">
-        <v>46297.66736068287</v>
+        <v>46297.37618915509</v>
       </c>
       <c r="S198">
         <v>3</v>
       </c>
       <c r="T198" t="s">
-        <v>266</v>
-      </c>
-      <c r="V198" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="AA198">
         <v>0</v>
@@ -15209,10 +15209,10 @@
     </row>
     <row r="199" spans="1:34">
       <c r="A199">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B199" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C199" t="s">
         <v>57</v>
@@ -15245,7 +15245,7 @@
         <v>221</v>
       </c>
       <c r="O199">
-        <v>18085221</v>
+        <v>18155319</v>
       </c>
       <c r="P199" t="s">
         <v>238</v>
@@ -15254,13 +15254,13 @@
         <v>258</v>
       </c>
       <c r="R199" s="1">
-        <v>46297.45935385417</v>
+        <v>46297.66736068287</v>
       </c>
       <c r="S199">
         <v>3</v>
       </c>
       <c r="T199" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="V199" t="s">
         <v>274</v>
@@ -15280,10 +15280,10 @@
     </row>
     <row r="200" spans="1:34">
       <c r="A200">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B200" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C200" t="s">
         <v>57</v>
@@ -15298,7 +15298,7 @@
         <v>64</v>
       </c>
       <c r="G200">
-        <v>6802</v>
+        <v>1836</v>
       </c>
       <c r="H200">
         <v>1788</v>
@@ -15307,7 +15307,7 @@
         <v>68</v>
       </c>
       <c r="J200" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L200" s="1">
         <v>46300</v>
@@ -15316,7 +15316,7 @@
         <v>221</v>
       </c>
       <c r="O200">
-        <v>17399221</v>
+        <v>18085221</v>
       </c>
       <c r="P200" t="s">
         <v>238</v>
@@ -15325,13 +15325,16 @@
         <v>258</v>
       </c>
       <c r="R200" s="1">
-        <v>46297.37681010416</v>
+        <v>46297.45935385417</v>
       </c>
       <c r="S200">
         <v>3</v>
       </c>
       <c r="T200" t="s">
-        <v>260</v>
+        <v>264</v>
+      </c>
+      <c r="V200" t="s">
+        <v>274</v>
       </c>
       <c r="AA200">
         <v>0</v>
@@ -15366,16 +15369,16 @@
         <v>64</v>
       </c>
       <c r="G201">
-        <v>6801</v>
+        <v>6802</v>
       </c>
       <c r="H201">
-        <v>1796</v>
+        <v>1788</v>
       </c>
       <c r="I201" t="s">
         <v>68</v>
       </c>
       <c r="J201" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L201" s="1">
         <v>46300</v>
@@ -15384,7 +15387,7 @@
         <v>221</v>
       </c>
       <c r="O201">
-        <v>17399211</v>
+        <v>17399221</v>
       </c>
       <c r="P201" t="s">
         <v>238</v>
@@ -15393,7 +15396,7 @@
         <v>258</v>
       </c>
       <c r="R201" s="1">
-        <v>46297.37686377315</v>
+        <v>46297.37681010416</v>
       </c>
       <c r="S201">
         <v>3</v>
@@ -15434,16 +15437,16 @@
         <v>64</v>
       </c>
       <c r="G202">
-        <v>6014</v>
+        <v>6801</v>
       </c>
       <c r="H202">
-        <v>1788</v>
+        <v>1796</v>
       </c>
       <c r="I202" t="s">
         <v>68</v>
       </c>
       <c r="J202" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L202" s="1">
         <v>46300</v>
@@ -15452,7 +15455,7 @@
         <v>221</v>
       </c>
       <c r="O202">
-        <v>17399137</v>
+        <v>17399211</v>
       </c>
       <c r="P202" t="s">
         <v>238</v>
@@ -15461,7 +15464,7 @@
         <v>258</v>
       </c>
       <c r="R202" s="1">
-        <v>46297.37606362269</v>
+        <v>46297.37686377315</v>
       </c>
       <c r="S202">
         <v>3</v>
@@ -15484,10 +15487,10 @@
     </row>
     <row r="203" spans="1:34">
       <c r="A203">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B203" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C203" t="s">
         <v>57</v>
@@ -15520,7 +15523,7 @@
         <v>221</v>
       </c>
       <c r="O203">
-        <v>18155328</v>
+        <v>17399137</v>
       </c>
       <c r="P203" t="s">
         <v>238</v>
@@ -15529,16 +15532,13 @@
         <v>258</v>
       </c>
       <c r="R203" s="1">
-        <v>46297.66734447917</v>
+        <v>46297.37606362269</v>
       </c>
       <c r="S203">
         <v>3</v>
       </c>
       <c r="T203" t="s">
-        <v>266</v>
-      </c>
-      <c r="V203" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="AA203">
         <v>0</v>
@@ -15555,10 +15555,10 @@
     </row>
     <row r="204" spans="1:34">
       <c r="A204">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B204" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C204" t="s">
         <v>57</v>
@@ -15591,7 +15591,7 @@
         <v>221</v>
       </c>
       <c r="O204">
-        <v>18085232</v>
+        <v>18155328</v>
       </c>
       <c r="P204" t="s">
         <v>238</v>
@@ -15600,13 +15600,13 @@
         <v>258</v>
       </c>
       <c r="R204" s="1">
-        <v>46297.45929016203</v>
+        <v>46297.66734447917</v>
       </c>
       <c r="S204">
         <v>3</v>
       </c>
       <c r="T204" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="V204" t="s">
         <v>274</v>
@@ -15626,10 +15626,10 @@
     </row>
     <row r="205" spans="1:34">
       <c r="A205">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B205" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C205" t="s">
         <v>57</v>
@@ -15644,16 +15644,16 @@
         <v>64</v>
       </c>
       <c r="G205">
-        <v>6233</v>
+        <v>6014</v>
       </c>
       <c r="H205">
-        <v>6232</v>
+        <v>1788</v>
       </c>
       <c r="I205" t="s">
         <v>68</v>
       </c>
       <c r="J205" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="L205" s="1">
         <v>46300</v>
@@ -15662,7 +15662,7 @@
         <v>221</v>
       </c>
       <c r="O205">
-        <v>17399177</v>
+        <v>18085232</v>
       </c>
       <c r="P205" t="s">
         <v>238</v>
@@ -15671,19 +15671,22 @@
         <v>258</v>
       </c>
       <c r="R205" s="1">
-        <v>46297.37537966435</v>
+        <v>46297.45929016203</v>
       </c>
       <c r="S205">
         <v>3</v>
       </c>
       <c r="T205" t="s">
-        <v>260</v>
+        <v>264</v>
+      </c>
+      <c r="V205" t="s">
+        <v>274</v>
       </c>
       <c r="AA205">
         <v>0</v>
       </c>
       <c r="AB205" t="s">
-        <v>372</v>
+        <v>238</v>
       </c>
       <c r="AG205" t="s">
         <v>378</v>
@@ -15694,16 +15697,16 @@
     </row>
     <row r="206" spans="1:34">
       <c r="A206">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B206" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C206" t="s">
         <v>57</v>
       </c>
       <c r="D206" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E206" t="s">
         <v>61</v>
@@ -15730,7 +15733,7 @@
         <v>221</v>
       </c>
       <c r="O206">
-        <v>16962295</v>
+        <v>17399177</v>
       </c>
       <c r="P206" t="s">
         <v>238</v>
@@ -15739,13 +15742,13 @@
         <v>258</v>
       </c>
       <c r="R206" s="1">
-        <v>46297.45869950231</v>
+        <v>46297.37537966435</v>
       </c>
       <c r="S206">
         <v>3</v>
       </c>
       <c r="T206" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="AA206">
         <v>0</v>
@@ -15762,16 +15765,16 @@
     </row>
     <row r="207" spans="1:34">
       <c r="A207">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B207" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C207" t="s">
         <v>57</v>
       </c>
       <c r="D207" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E207" t="s">
         <v>61</v>
@@ -15798,7 +15801,7 @@
         <v>221</v>
       </c>
       <c r="O207">
-        <v>16976157</v>
+        <v>16962295</v>
       </c>
       <c r="P207" t="s">
         <v>238</v>
@@ -15807,16 +15810,13 @@
         <v>258</v>
       </c>
       <c r="R207" s="1">
-        <v>46300.66721489583</v>
+        <v>46297.45869950231</v>
       </c>
       <c r="S207">
         <v>3</v>
       </c>
       <c r="T207" t="s">
-        <v>266</v>
-      </c>
-      <c r="V207" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="AA207">
         <v>0</v>
@@ -15833,16 +15833,16 @@
     </row>
     <row r="208" spans="1:34">
       <c r="A208">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B208" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C208" t="s">
         <v>57</v>
       </c>
       <c r="D208" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E208" t="s">
         <v>61</v>
@@ -15869,7 +15869,7 @@
         <v>221</v>
       </c>
       <c r="O208">
-        <v>17948845</v>
+        <v>16976157</v>
       </c>
       <c r="P208" t="s">
         <v>238</v>
@@ -15878,13 +15878,16 @@
         <v>258</v>
       </c>
       <c r="R208" s="1">
-        <v>46297.45870309028</v>
+        <v>46300.66721489583</v>
       </c>
       <c r="S208">
         <v>3</v>
       </c>
       <c r="T208" t="s">
-        <v>263</v>
+        <v>266</v>
+      </c>
+      <c r="V208" t="s">
+        <v>274</v>
       </c>
       <c r="AA208">
         <v>0</v>
@@ -15901,16 +15904,16 @@
     </row>
     <row r="209" spans="1:34">
       <c r="A209">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B209" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C209" t="s">
         <v>57</v>
       </c>
       <c r="D209" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E209" t="s">
         <v>61</v>
@@ -15937,7 +15940,7 @@
         <v>221</v>
       </c>
       <c r="O209">
-        <v>18085265</v>
+        <v>17948845</v>
       </c>
       <c r="P209" t="s">
         <v>238</v>
@@ -15946,16 +15949,13 @@
         <v>258</v>
       </c>
       <c r="R209" s="1">
-        <v>46297.45870405093</v>
+        <v>46297.45870309028</v>
       </c>
       <c r="S209">
         <v>3</v>
       </c>
       <c r="T209" t="s">
-        <v>264</v>
-      </c>
-      <c r="V209" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="AA209">
         <v>0</v>
@@ -15972,16 +15972,16 @@
     </row>
     <row r="210" spans="1:34">
       <c r="A210">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B210" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C210" t="s">
         <v>57</v>
       </c>
       <c r="D210" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E210" t="s">
         <v>61</v>
@@ -16008,7 +16008,7 @@
         <v>221</v>
       </c>
       <c r="O210">
-        <v>17948990</v>
+        <v>18085265</v>
       </c>
       <c r="P210" t="s">
         <v>238</v>
@@ -16017,7 +16017,7 @@
         <v>258</v>
       </c>
       <c r="R210" s="1">
-        <v>46297.45870177083</v>
+        <v>46297.45870405093</v>
       </c>
       <c r="S210">
         <v>3</v>
@@ -16025,6 +16025,9 @@
       <c r="T210" t="s">
         <v>264</v>
       </c>
+      <c r="V210" t="s">
+        <v>274</v>
+      </c>
       <c r="AA210">
         <v>0</v>
       </c>
@@ -16040,16 +16043,16 @@
     </row>
     <row r="211" spans="1:34">
       <c r="A211">
-        <v>5417</v>
+        <v>6705</v>
       </c>
       <c r="B211" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C211" t="s">
         <v>57</v>
       </c>
       <c r="D211" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E211" t="s">
         <v>61</v>
@@ -16058,16 +16061,16 @@
         <v>64</v>
       </c>
       <c r="G211">
-        <v>6230</v>
+        <v>6233</v>
       </c>
       <c r="H211">
-        <v>9114</v>
+        <v>6232</v>
       </c>
       <c r="I211" t="s">
         <v>68</v>
       </c>
       <c r="J211" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L211" s="1">
         <v>46300</v>
@@ -16076,7 +16079,7 @@
         <v>221</v>
       </c>
       <c r="O211">
-        <v>17399157</v>
+        <v>17948990</v>
       </c>
       <c r="P211" t="s">
         <v>238</v>
@@ -16085,13 +16088,13 @@
         <v>258</v>
       </c>
       <c r="R211" s="1">
-        <v>46300.65013206018</v>
+        <v>46297.45870177083</v>
       </c>
       <c r="S211">
         <v>3</v>
       </c>
       <c r="T211" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="AA211">
         <v>0</v>
@@ -16108,16 +16111,16 @@
     </row>
     <row r="212" spans="1:34">
       <c r="A212">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B212" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C212" t="s">
         <v>57</v>
       </c>
       <c r="D212" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E212" t="s">
         <v>61</v>
@@ -16144,7 +16147,7 @@
         <v>221</v>
       </c>
       <c r="O212">
-        <v>16962275</v>
+        <v>17399157</v>
       </c>
       <c r="P212" t="s">
         <v>238</v>
@@ -16153,13 +16156,13 @@
         <v>258</v>
       </c>
       <c r="R212" s="1">
-        <v>46300.65011049769</v>
+        <v>46300.65013206018</v>
       </c>
       <c r="S212">
         <v>3</v>
       </c>
       <c r="T212" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="AA212">
         <v>0</v>
@@ -16176,16 +16179,16 @@
     </row>
     <row r="213" spans="1:34">
       <c r="A213">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B213" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C213" t="s">
         <v>57</v>
       </c>
       <c r="D213" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E213" t="s">
         <v>61</v>
@@ -16212,7 +16215,7 @@
         <v>221</v>
       </c>
       <c r="O213">
-        <v>16976137</v>
+        <v>16962275</v>
       </c>
       <c r="P213" t="s">
         <v>238</v>
@@ -16221,16 +16224,13 @@
         <v>258</v>
       </c>
       <c r="R213" s="1">
-        <v>46300.66713765046</v>
+        <v>46300.65011049769</v>
       </c>
       <c r="S213">
         <v>3</v>
       </c>
       <c r="T213" t="s">
-        <v>266</v>
-      </c>
-      <c r="V213" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="AA213">
         <v>0</v>
@@ -16247,16 +16247,16 @@
     </row>
     <row r="214" spans="1:34">
       <c r="A214">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B214" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C214" t="s">
         <v>57</v>
       </c>
       <c r="D214" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E214" t="s">
         <v>61</v>
@@ -16283,7 +16283,7 @@
         <v>221</v>
       </c>
       <c r="O214">
-        <v>17948825</v>
+        <v>16976137</v>
       </c>
       <c r="P214" t="s">
         <v>238</v>
@@ -16292,13 +16292,16 @@
         <v>258</v>
       </c>
       <c r="R214" s="1">
-        <v>46300.66713784722</v>
+        <v>46300.66713765046</v>
       </c>
       <c r="S214">
         <v>3</v>
       </c>
       <c r="T214" t="s">
-        <v>263</v>
+        <v>266</v>
+      </c>
+      <c r="V214" t="s">
+        <v>274</v>
       </c>
       <c r="AA214">
         <v>0</v>
@@ -16315,16 +16318,16 @@
     </row>
     <row r="215" spans="1:34">
       <c r="A215">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B215" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C215" t="s">
         <v>57</v>
       </c>
       <c r="D215" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E215" t="s">
         <v>61</v>
@@ -16351,7 +16354,7 @@
         <v>221</v>
       </c>
       <c r="O215">
-        <v>18085243</v>
+        <v>17948825</v>
       </c>
       <c r="P215" t="s">
         <v>238</v>
@@ -16360,16 +16363,13 @@
         <v>258</v>
       </c>
       <c r="R215" s="1">
-        <v>46300.66713822917</v>
+        <v>46300.66713784722</v>
       </c>
       <c r="S215">
         <v>3</v>
       </c>
       <c r="T215" t="s">
-        <v>264</v>
-      </c>
-      <c r="V215" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="AA215">
         <v>0</v>
@@ -16386,16 +16386,16 @@
     </row>
     <row r="216" spans="1:34">
       <c r="A216">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B216" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C216" t="s">
         <v>57</v>
       </c>
       <c r="D216" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E216" t="s">
         <v>61</v>
@@ -16422,7 +16422,7 @@
         <v>221</v>
       </c>
       <c r="O216">
-        <v>17948970</v>
+        <v>18085243</v>
       </c>
       <c r="P216" t="s">
         <v>238</v>
@@ -16431,7 +16431,7 @@
         <v>258</v>
       </c>
       <c r="R216" s="1">
-        <v>46300.75530894676</v>
+        <v>46300.66713822917</v>
       </c>
       <c r="S216">
         <v>3</v>
@@ -16439,6 +16439,9 @@
       <c r="T216" t="s">
         <v>264</v>
       </c>
+      <c r="V216" t="s">
+        <v>274</v>
+      </c>
       <c r="AA216">
         <v>0</v>
       </c>
@@ -16454,16 +16457,16 @@
     </row>
     <row r="217" spans="1:34">
       <c r="A217">
-        <v>6486</v>
+        <v>6705</v>
       </c>
       <c r="B217" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C217" t="s">
         <v>57</v>
       </c>
       <c r="D217" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E217" t="s">
         <v>61</v>
@@ -16472,25 +16475,25 @@
         <v>64</v>
       </c>
       <c r="G217">
-        <v>11359</v>
+        <v>6230</v>
       </c>
       <c r="H217">
-        <v>0</v>
+        <v>9114</v>
       </c>
       <c r="I217" t="s">
         <v>68</v>
       </c>
       <c r="J217" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="L217" s="1">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="N217" t="s">
         <v>221</v>
       </c>
       <c r="O217">
-        <v>18155346</v>
+        <v>17948970</v>
       </c>
       <c r="P217" t="s">
         <v>238</v>
@@ -16499,22 +16502,19 @@
         <v>258</v>
       </c>
       <c r="R217" s="1">
-        <v>46297.66734765047</v>
+        <v>46300.75530894676</v>
       </c>
       <c r="S217">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T217" t="s">
-        <v>266</v>
-      </c>
-      <c r="V217" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="AA217">
         <v>0</v>
       </c>
       <c r="AB217" t="s">
-        <v>238</v>
+        <v>372</v>
       </c>
       <c r="AG217" t="s">
         <v>378</v>
@@ -16525,10 +16525,10 @@
     </row>
     <row r="218" spans="1:34">
       <c r="A218">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B218" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C218" t="s">
         <v>57</v>
@@ -16543,7 +16543,7 @@
         <v>64</v>
       </c>
       <c r="G218">
-        <v>11303</v>
+        <v>11359</v>
       </c>
       <c r="H218">
         <v>0</v>
@@ -16552,16 +16552,16 @@
         <v>68</v>
       </c>
       <c r="J218" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="L218" s="1">
-        <v>46308</v>
+        <v>46297</v>
       </c>
       <c r="N218" t="s">
         <v>221</v>
       </c>
       <c r="O218">
-        <v>17399455</v>
+        <v>18155346</v>
       </c>
       <c r="P218" t="s">
         <v>238</v>
@@ -16570,19 +16570,22 @@
         <v>258</v>
       </c>
       <c r="R218" s="1">
-        <v>46301.70844945602</v>
+        <v>46297.66734765047</v>
       </c>
       <c r="S218">
-        <v>-5</v>
+        <v>6</v>
       </c>
       <c r="T218" t="s">
-        <v>260</v>
+        <v>266</v>
+      </c>
+      <c r="V218" t="s">
+        <v>274</v>
       </c>
       <c r="AA218">
         <v>0</v>
       </c>
       <c r="AB218" t="s">
-        <v>370</v>
+        <v>238</v>
       </c>
       <c r="AG218" t="s">
         <v>378</v>
@@ -16593,16 +16596,16 @@
     </row>
     <row r="219" spans="1:34">
       <c r="A219">
-        <v>6705</v>
+        <v>5417</v>
       </c>
       <c r="B219" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C219" t="s">
         <v>57</v>
       </c>
       <c r="D219" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E219" t="s">
         <v>61</v>
@@ -16629,7 +16632,7 @@
         <v>221</v>
       </c>
       <c r="O219">
-        <v>17949080</v>
+        <v>17399455</v>
       </c>
       <c r="P219" t="s">
         <v>238</v>
@@ -16638,13 +16641,13 @@
         <v>258</v>
       </c>
       <c r="R219" s="1">
-        <v>46301.70847283565</v>
+        <v>46301.70844945602</v>
       </c>
       <c r="S219">
         <v>-5</v>
       </c>
       <c r="T219" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="AA219">
         <v>0</v>
@@ -16661,16 +16664,16 @@
     </row>
     <row r="220" spans="1:34">
       <c r="A220">
-        <v>6703</v>
+        <v>6705</v>
       </c>
       <c r="B220" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C220" t="s">
         <v>57</v>
       </c>
       <c r="D220" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E220" t="s">
         <v>61</v>
@@ -16679,66 +16682,66 @@
         <v>64</v>
       </c>
       <c r="G220">
-        <v>950</v>
+        <v>11303</v>
       </c>
       <c r="H220">
         <v>0</v>
       </c>
       <c r="I220" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J220" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L220" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="N220" t="s">
         <v>221</v>
       </c>
       <c r="O220">
-        <v>17941147</v>
+        <v>17949080</v>
       </c>
       <c r="P220" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="Q220" t="s">
         <v>258</v>
       </c>
       <c r="R220" s="1">
-        <v>46296.37684039352</v>
+        <v>46301.70847283565</v>
       </c>
       <c r="S220">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="T220" t="s">
-        <v>263</v>
-      </c>
-      <c r="W220" t="s">
-        <v>334</v>
+        <v>264</v>
       </c>
       <c r="AA220">
         <v>0</v>
       </c>
       <c r="AB220" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="AG220" t="s">
-        <v>379</v>
+        <v>378</v>
+      </c>
+      <c r="AH220" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="221" spans="1:34">
       <c r="A221">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B221" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C221" t="s">
         <v>57</v>
       </c>
       <c r="D221" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E221" t="s">
         <v>61</v>
@@ -16765,25 +16768,25 @@
         <v>221</v>
       </c>
       <c r="O221">
-        <v>17952341</v>
+        <v>17941147</v>
       </c>
       <c r="P221" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="Q221" t="s">
         <v>258</v>
       </c>
       <c r="R221" s="1">
-        <v>46057.390791875</v>
+        <v>46296.37684039352</v>
       </c>
       <c r="S221">
         <v>-1</v>
       </c>
       <c r="T221" t="s">
-        <v>264</v>
-      </c>
-      <c r="V221" t="s">
-        <v>274</v>
+        <v>263</v>
+      </c>
+      <c r="W221" t="s">
+        <v>335</v>
       </c>
       <c r="AA221">
         <v>0</v>
@@ -16797,22 +16800,22 @@
     </row>
     <row r="222" spans="1:34">
       <c r="A222">
-        <v>6962</v>
+        <v>6704</v>
       </c>
       <c r="B222" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C222" t="s">
         <v>57</v>
       </c>
       <c r="D222" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E222" t="s">
         <v>61</v>
       </c>
       <c r="F222" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G222">
         <v>950</v>
@@ -16833,7 +16836,7 @@
         <v>221</v>
       </c>
       <c r="O222">
-        <v>18188718</v>
+        <v>17952341</v>
       </c>
       <c r="P222" t="s">
         <v>239</v>
@@ -16842,13 +16845,16 @@
         <v>258</v>
       </c>
       <c r="R222" s="1">
-        <v>46192.56685424769</v>
+        <v>46057.390791875</v>
       </c>
       <c r="S222">
         <v>-1</v>
       </c>
       <c r="T222" t="s">
-        <v>267</v>
+        <v>264</v>
+      </c>
+      <c r="V222" t="s">
+        <v>274</v>
       </c>
       <c r="AA222">
         <v>0</v>
@@ -16862,25 +16868,25 @@
     </row>
     <row r="223" spans="1:34">
       <c r="A223">
-        <v>6548</v>
+        <v>6962</v>
       </c>
       <c r="B223" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C223" t="s">
         <v>57</v>
       </c>
       <c r="D223" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E223" t="s">
         <v>61</v>
       </c>
       <c r="F223" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G223">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H223">
         <v>0</v>
@@ -16889,7 +16895,7 @@
         <v>69</v>
       </c>
       <c r="J223" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L223" s="1">
         <v>46304</v>
@@ -16898,7 +16904,7 @@
         <v>221</v>
       </c>
       <c r="O223">
-        <v>17222406</v>
+        <v>18188718</v>
       </c>
       <c r="P223" t="s">
         <v>239</v>
@@ -16907,19 +16913,13 @@
         <v>258</v>
       </c>
       <c r="R223" s="1">
-        <v>46296.37726273148</v>
+        <v>46192.56685424769</v>
       </c>
       <c r="S223">
         <v>-1</v>
       </c>
       <c r="T223" t="s">
-        <v>261</v>
-      </c>
-      <c r="V223" t="s">
-        <v>274</v>
-      </c>
-      <c r="W223" t="s">
-        <v>335</v>
+        <v>267</v>
       </c>
       <c r="AA223">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-14 12:04
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9100" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9102" uniqueCount="426">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1160,6 +1160,9 @@
 PROCESSANDO - Data Comentário: 14/10/2026 10:16</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 15/10/2026 - Data Comentário: 14/10/2026 11:37</t>
+  </si>
+  <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 16/10/2026 - Data Comentário: 14/10/2026 10:41</t>
   </si>
   <si>
@@ -1286,13 +1289,10 @@
     <t>Karina Fonseca</t>
   </si>
   <si>
-    <t>Tarefa reaberta. A previsão de conclusão está prevista para 03/10/2026. - Data Comentário: 02/10/2026 16:45</t>
+    <t>Tarefa reaberta. A previsão de conclusão está prevista para 14/10/2026. - Data Comentário: 14/10/2026 11:59</t>
   </si>
   <si>
-    <t>Tarefa reaberta. A previsão de conclusão está prevista para 25/09/2026. - Data Comentário: 24/09/2026 13:40</t>
-  </si>
-  <si>
-    <t>03/10/2026</t>
+    <t>Tarefa reaberta. A previsão de conclusão está prevista para 14/10/2026. - Data Comentário: 14/10/2026 12:00</t>
   </si>
   <si>
     <t>Tarefa</t>
@@ -3196,7 +3196,7 @@
         <v>415</v>
       </c>
       <c r="AH22" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="23" spans="1:34">
@@ -3261,7 +3261,7 @@
         <v>414</v>
       </c>
       <c r="AH23" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="24" spans="1:34">
@@ -3323,7 +3323,7 @@
         <v>414</v>
       </c>
       <c r="AH24" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="25" spans="1:34">
@@ -3385,7 +3385,7 @@
         <v>414</v>
       </c>
       <c r="AH25" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="26" spans="1:34">
@@ -3707,7 +3707,7 @@
         <v>0</v>
       </c>
       <c r="AB30" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG30" t="s">
         <v>414</v>
@@ -3778,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="AB31" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG31" t="s">
         <v>414</v>
@@ -3849,7 +3849,7 @@
         <v>0</v>
       </c>
       <c r="AB32" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG32" t="s">
         <v>414</v>
@@ -3917,7 +3917,7 @@
         <v>0</v>
       </c>
       <c r="AB33" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG33" t="s">
         <v>414</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="AB34" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG34" t="s">
         <v>414</v>
@@ -4053,7 +4053,7 @@
         <v>0</v>
       </c>
       <c r="AB35" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG35" t="s">
         <v>414</v>
@@ -4121,7 +4121,7 @@
         <v>0</v>
       </c>
       <c r="AB36" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG36" t="s">
         <v>414</v>
@@ -4189,13 +4189,13 @@
         <v>0</v>
       </c>
       <c r="AB37" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG37" t="s">
         <v>414</v>
       </c>
       <c r="AH37" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="38" spans="1:34">
@@ -4260,7 +4260,7 @@
         <v>0</v>
       </c>
       <c r="AB38" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG38" t="s">
         <v>414</v>
@@ -4328,7 +4328,7 @@
         <v>0</v>
       </c>
       <c r="AB39" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG39" t="s">
         <v>414</v>
@@ -4399,7 +4399,7 @@
         <v>0</v>
       </c>
       <c r="AB40" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG40" t="s">
         <v>414</v>
@@ -7012,7 +7012,7 @@
         <v>0</v>
       </c>
       <c r="AB76" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG76" t="s">
         <v>416</v>
@@ -10131,7 +10131,7 @@
         <v>414</v>
       </c>
       <c r="AH119" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="120" spans="1:34">
@@ -10202,7 +10202,7 @@
         <v>414</v>
       </c>
       <c r="AH120" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="121" spans="1:34">
@@ -10273,7 +10273,7 @@
         <v>414</v>
       </c>
       <c r="AH121" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="122" spans="1:34">
@@ -10344,7 +10344,7 @@
         <v>414</v>
       </c>
       <c r="AH122" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="123" spans="1:34">
@@ -10415,7 +10415,7 @@
         <v>414</v>
       </c>
       <c r="AH123" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="124" spans="1:34">
@@ -10486,7 +10486,7 @@
         <v>414</v>
       </c>
       <c r="AH124" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="125" spans="1:34">
@@ -10557,7 +10557,7 @@
         <v>414</v>
       </c>
       <c r="AH125" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="126" spans="1:34">
@@ -10628,7 +10628,7 @@
         <v>414</v>
       </c>
       <c r="AH126" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="127" spans="1:34">
@@ -10699,7 +10699,7 @@
         <v>414</v>
       </c>
       <c r="AH127" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="128" spans="1:34">
@@ -10770,7 +10770,7 @@
         <v>414</v>
       </c>
       <c r="AH128" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="129" spans="1:34">
@@ -10838,7 +10838,7 @@
         <v>414</v>
       </c>
       <c r="AH129" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="130" spans="1:34">
@@ -10900,13 +10900,13 @@
         <v>0</v>
       </c>
       <c r="AB130" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AG130" t="s">
         <v>414</v>
       </c>
       <c r="AH130" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="131" spans="1:34">
@@ -10974,7 +10974,7 @@
         <v>414</v>
       </c>
       <c r="AH131" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="132" spans="1:34">
@@ -11045,7 +11045,7 @@
         <v>414</v>
       </c>
       <c r="AH132" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="133" spans="1:34">
@@ -11116,7 +11116,7 @@
         <v>414</v>
       </c>
       <c r="AH133" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="134" spans="1:34">
@@ -11187,7 +11187,7 @@
         <v>414</v>
       </c>
       <c r="AH134" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="135" spans="1:34">
@@ -11249,13 +11249,13 @@
         <v>0</v>
       </c>
       <c r="AB135" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AG135" t="s">
         <v>414</v>
       </c>
       <c r="AH135" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="136" spans="1:34">
@@ -11326,7 +11326,7 @@
         <v>414</v>
       </c>
       <c r="AH136" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="137" spans="1:34">
@@ -11394,7 +11394,7 @@
         <v>414</v>
       </c>
       <c r="AH137" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="138" spans="1:34">
@@ -11462,7 +11462,7 @@
         <v>414</v>
       </c>
       <c r="AH138" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="139" spans="1:34">
@@ -11524,13 +11524,13 @@
         <v>0</v>
       </c>
       <c r="AB139" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG139" t="s">
         <v>414</v>
       </c>
       <c r="AH139" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="140" spans="1:34">
@@ -11592,13 +11592,13 @@
         <v>0</v>
       </c>
       <c r="AB140" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG140" t="s">
         <v>414</v>
       </c>
       <c r="AH140" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="141" spans="1:34">
@@ -11663,13 +11663,13 @@
         <v>0</v>
       </c>
       <c r="AB141" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG141" t="s">
         <v>414</v>
       </c>
       <c r="AH141" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="142" spans="1:34">
@@ -11731,13 +11731,13 @@
         <v>0</v>
       </c>
       <c r="AB142" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG142" t="s">
         <v>414</v>
       </c>
       <c r="AH142" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="143" spans="1:34">
@@ -11799,13 +11799,13 @@
         <v>0</v>
       </c>
       <c r="AB143" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG143" t="s">
         <v>414</v>
       </c>
       <c r="AH143" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="144" spans="1:34">
@@ -11876,7 +11876,7 @@
         <v>414</v>
       </c>
       <c r="AH144" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="145" spans="1:34">
@@ -11947,7 +11947,7 @@
         <v>414</v>
       </c>
       <c r="AH145" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="146" spans="1:34">
@@ -12018,7 +12018,7 @@
         <v>414</v>
       </c>
       <c r="AH146" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="147" spans="1:34">
@@ -12089,7 +12089,7 @@
         <v>414</v>
       </c>
       <c r="AH147" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="148" spans="1:34">
@@ -12160,7 +12160,7 @@
         <v>414</v>
       </c>
       <c r="AH148" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="149" spans="1:34">
@@ -12231,7 +12231,7 @@
         <v>414</v>
       </c>
       <c r="AH149" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="150" spans="1:34">
@@ -12302,7 +12302,7 @@
         <v>415</v>
       </c>
       <c r="AH150" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="151" spans="1:34">
@@ -12373,7 +12373,7 @@
         <v>415</v>
       </c>
       <c r="AH151" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="152" spans="1:34">
@@ -12444,7 +12444,7 @@
         <v>415</v>
       </c>
       <c r="AH152" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="153" spans="1:34">
@@ -12512,7 +12512,7 @@
         <v>415</v>
       </c>
       <c r="AH153" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="154" spans="1:34">
@@ -12580,7 +12580,7 @@
         <v>415</v>
       </c>
       <c r="AH154" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="155" spans="1:34">
@@ -12654,7 +12654,7 @@
         <v>415</v>
       </c>
       <c r="AH155" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="156" spans="1:34">
@@ -12728,7 +12728,7 @@
         <v>415</v>
       </c>
       <c r="AH156" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="157" spans="1:34">
@@ -12805,7 +12805,7 @@
         <v>416</v>
       </c>
       <c r="AH157" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="158" spans="1:34">
@@ -12876,7 +12876,7 @@
         <v>416</v>
       </c>
       <c r="AH158" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="159" spans="1:34">
@@ -12941,13 +12941,13 @@
         <v>0</v>
       </c>
       <c r="AB159" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG159" t="s">
         <v>416</v>
       </c>
       <c r="AH159" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="160" spans="1:34">
@@ -13012,13 +13012,13 @@
         <v>0</v>
       </c>
       <c r="AB160" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG160" t="s">
         <v>416</v>
       </c>
       <c r="AH160" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="161" spans="1:34">
@@ -13095,7 +13095,7 @@
         <v>416</v>
       </c>
       <c r="AH161" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="162" spans="1:34">
@@ -13169,7 +13169,7 @@
         <v>416</v>
       </c>
       <c r="AH162" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="163" spans="1:34">
@@ -13243,7 +13243,7 @@
         <v>416</v>
       </c>
       <c r="AH163" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="164" spans="1:34">
@@ -13314,7 +13314,7 @@
         <v>416</v>
       </c>
       <c r="AH164" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="165" spans="1:34">
@@ -13382,13 +13382,13 @@
         <v>0</v>
       </c>
       <c r="AB165" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AG165" t="s">
         <v>416</v>
       </c>
       <c r="AH165" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="166" spans="1:34">
@@ -13459,7 +13459,7 @@
         <v>416</v>
       </c>
       <c r="AH166" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="167" spans="1:34">
@@ -13533,7 +13533,7 @@
         <v>414</v>
       </c>
       <c r="AH167" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="168" spans="1:34">
@@ -14219,7 +14219,7 @@
         <v>0</v>
       </c>
       <c r="AB177" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG177" t="s">
         <v>414</v>
@@ -14287,7 +14287,7 @@
         <v>0</v>
       </c>
       <c r="AB178" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG178" t="s">
         <v>414</v>
@@ -14358,7 +14358,7 @@
         <v>0</v>
       </c>
       <c r="AB179" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG179" t="s">
         <v>414</v>
@@ -14426,7 +14426,7 @@
         <v>0</v>
       </c>
       <c r="AB180" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG180" t="s">
         <v>414</v>
@@ -14497,7 +14497,7 @@
         <v>0</v>
       </c>
       <c r="AB181" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG181" t="s">
         <v>414</v>
@@ -14565,7 +14565,7 @@
         <v>0</v>
       </c>
       <c r="AB182" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG182" t="s">
         <v>414</v>
@@ -14633,7 +14633,7 @@
         <v>0</v>
       </c>
       <c r="AB183" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG183" t="s">
         <v>414</v>
@@ -14701,7 +14701,7 @@
         <v>0</v>
       </c>
       <c r="AB184" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG184" t="s">
         <v>414</v>
@@ -14772,7 +14772,7 @@
         <v>0</v>
       </c>
       <c r="AB185" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG185" t="s">
         <v>414</v>
@@ -14840,7 +14840,7 @@
         <v>0</v>
       </c>
       <c r="AB186" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG186" t="s">
         <v>414</v>
@@ -14911,7 +14911,7 @@
         <v>0</v>
       </c>
       <c r="AB187" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG187" t="s">
         <v>414</v>
@@ -14979,7 +14979,7 @@
         <v>0</v>
       </c>
       <c r="AB188" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG188" t="s">
         <v>414</v>
@@ -15899,7 +15899,7 @@
         <v>0</v>
       </c>
       <c r="AB201" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG201" t="s">
         <v>414</v>
@@ -15967,7 +15967,7 @@
         <v>0</v>
       </c>
       <c r="AB202" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG202" t="s">
         <v>414</v>
@@ -16106,7 +16106,7 @@
         <v>0</v>
       </c>
       <c r="AB204" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG204" t="s">
         <v>416</v>
@@ -16585,7 +16585,7 @@
         <v>0</v>
       </c>
       <c r="AB211" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG211" t="s">
         <v>416</v>
@@ -17061,7 +17061,7 @@
         <v>0</v>
       </c>
       <c r="AB218" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG218" t="s">
         <v>415</v>
@@ -17126,7 +17126,7 @@
         <v>0</v>
       </c>
       <c r="AB219" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG219" t="s">
         <v>415</v>
@@ -17194,7 +17194,7 @@
         <v>0</v>
       </c>
       <c r="AB220" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG220" t="s">
         <v>415</v>
@@ -17262,7 +17262,7 @@
         <v>0</v>
       </c>
       <c r="AB221" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG221" t="s">
         <v>415</v>
@@ -17330,7 +17330,7 @@
         <v>0</v>
       </c>
       <c r="AB222" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG222" t="s">
         <v>415</v>
@@ -17398,7 +17398,7 @@
         <v>0</v>
       </c>
       <c r="AB223" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG223" t="s">
         <v>415</v>
@@ -17463,7 +17463,7 @@
         <v>0</v>
       </c>
       <c r="AB224" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG224" t="s">
         <v>415</v>
@@ -17531,7 +17531,7 @@
         <v>0</v>
       </c>
       <c r="AB225" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG225" t="s">
         <v>415</v>
@@ -17596,7 +17596,7 @@
         <v>0</v>
       </c>
       <c r="AB226" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG226" t="s">
         <v>415</v>
@@ -17664,7 +17664,7 @@
         <v>0</v>
       </c>
       <c r="AB227" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG227" t="s">
         <v>415</v>
@@ -17729,7 +17729,7 @@
         <v>0</v>
       </c>
       <c r="AB228" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG228" t="s">
         <v>415</v>
@@ -17794,7 +17794,7 @@
         <v>0</v>
       </c>
       <c r="AB229" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG229" t="s">
         <v>415</v>
@@ -17859,7 +17859,7 @@
         <v>0</v>
       </c>
       <c r="AB230" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG230" t="s">
         <v>415</v>
@@ -17924,7 +17924,7 @@
         <v>0</v>
       </c>
       <c r="AB231" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG231" t="s">
         <v>415</v>
@@ -17995,7 +17995,7 @@
         <v>0</v>
       </c>
       <c r="AB232" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG232" t="s">
         <v>415</v>
@@ -18066,7 +18066,7 @@
         <v>0</v>
       </c>
       <c r="AB233" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG233" t="s">
         <v>415</v>
@@ -18140,7 +18140,7 @@
         <v>0</v>
       </c>
       <c r="AB234" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG234" t="s">
         <v>415</v>
@@ -18214,7 +18214,7 @@
         <v>0</v>
       </c>
       <c r="AB235" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG235" t="s">
         <v>415</v>
@@ -18288,7 +18288,7 @@
         <v>0</v>
       </c>
       <c r="AB236" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG236" t="s">
         <v>415</v>
@@ -18362,7 +18362,7 @@
         <v>0</v>
       </c>
       <c r="AB237" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG237" t="s">
         <v>415</v>
@@ -18433,7 +18433,7 @@
         <v>0</v>
       </c>
       <c r="AB238" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG238" t="s">
         <v>415</v>
@@ -18578,7 +18578,7 @@
         <v>0</v>
       </c>
       <c r="AB240" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG240" t="s">
         <v>415</v>
@@ -18649,7 +18649,7 @@
         <v>0</v>
       </c>
       <c r="AB241" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG241" t="s">
         <v>415</v>
@@ -18720,7 +18720,7 @@
         <v>0</v>
       </c>
       <c r="AB242" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG242" t="s">
         <v>415</v>
@@ -19249,7 +19249,7 @@
         <v>0</v>
       </c>
       <c r="AB250" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG250" t="s">
         <v>415</v>
@@ -19314,7 +19314,7 @@
         <v>0</v>
       </c>
       <c r="AB251" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG251" t="s">
         <v>415</v>
@@ -19382,7 +19382,7 @@
         <v>0</v>
       </c>
       <c r="AB252" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG252" t="s">
         <v>415</v>
@@ -19450,7 +19450,7 @@
         <v>0</v>
       </c>
       <c r="AB253" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG253" t="s">
         <v>415</v>
@@ -19518,7 +19518,7 @@
         <v>0</v>
       </c>
       <c r="AB254" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG254" t="s">
         <v>415</v>
@@ -19586,7 +19586,7 @@
         <v>0</v>
       </c>
       <c r="AB255" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG255" t="s">
         <v>415</v>
@@ -19651,7 +19651,7 @@
         <v>0</v>
       </c>
       <c r="AB256" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG256" t="s">
         <v>415</v>
@@ -19719,7 +19719,7 @@
         <v>0</v>
       </c>
       <c r="AB257" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG257" t="s">
         <v>415</v>
@@ -19784,7 +19784,7 @@
         <v>0</v>
       </c>
       <c r="AB258" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG258" t="s">
         <v>415</v>
@@ -19852,7 +19852,7 @@
         <v>0</v>
       </c>
       <c r="AB259" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG259" t="s">
         <v>415</v>
@@ -19917,7 +19917,7 @@
         <v>0</v>
       </c>
       <c r="AB260" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG260" t="s">
         <v>415</v>
@@ -19982,7 +19982,7 @@
         <v>0</v>
       </c>
       <c r="AB261" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG261" t="s">
         <v>415</v>
@@ -20047,7 +20047,7 @@
         <v>0</v>
       </c>
       <c r="AB262" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG262" t="s">
         <v>415</v>
@@ -20112,7 +20112,7 @@
         <v>0</v>
       </c>
       <c r="AB263" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG263" t="s">
         <v>415</v>
@@ -20177,7 +20177,7 @@
         <v>0</v>
       </c>
       <c r="AB264" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG264" t="s">
         <v>415</v>
@@ -20242,7 +20242,7 @@
         <v>0</v>
       </c>
       <c r="AB265" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG265" t="s">
         <v>415</v>
@@ -20310,7 +20310,7 @@
         <v>0</v>
       </c>
       <c r="AB266" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG266" t="s">
         <v>415</v>
@@ -20378,7 +20378,7 @@
         <v>0</v>
       </c>
       <c r="AB267" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG267" t="s">
         <v>415</v>
@@ -20446,7 +20446,7 @@
         <v>0</v>
       </c>
       <c r="AB268" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG268" t="s">
         <v>415</v>
@@ -20514,7 +20514,7 @@
         <v>0</v>
       </c>
       <c r="AB269" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG269" t="s">
         <v>415</v>
@@ -20579,7 +20579,7 @@
         <v>0</v>
       </c>
       <c r="AB270" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG270" t="s">
         <v>415</v>
@@ -20718,7 +20718,7 @@
         <v>0</v>
       </c>
       <c r="AB272" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG272" t="s">
         <v>415</v>
@@ -20783,7 +20783,7 @@
         <v>0</v>
       </c>
       <c r="AB273" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG273" t="s">
         <v>415</v>
@@ -20848,7 +20848,7 @@
         <v>0</v>
       </c>
       <c r="AB274" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG274" t="s">
         <v>415</v>
@@ -21496,7 +21496,7 @@
         <v>0</v>
       </c>
       <c r="AB283" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="AG283" t="s">
         <v>414</v>
@@ -21564,7 +21564,7 @@
         <v>0</v>
       </c>
       <c r="AB284" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="AG284" t="s">
         <v>414</v>
@@ -23723,7 +23723,7 @@
         <v>414</v>
       </c>
       <c r="AH318" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="319" spans="1:34">
@@ -23788,7 +23788,7 @@
         <v>414</v>
       </c>
       <c r="AH319" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="320" spans="1:34">
@@ -23915,7 +23915,7 @@
         <v>415</v>
       </c>
       <c r="AH321" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="322" spans="1:34">
@@ -24042,7 +24042,7 @@
         <v>415</v>
       </c>
       <c r="AH323" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="324" spans="1:34">
@@ -24104,7 +24104,7 @@
         <v>415</v>
       </c>
       <c r="AH324" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="325" spans="1:34">
@@ -24358,7 +24358,7 @@
         <v>416</v>
       </c>
       <c r="AH328" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="329" spans="1:34">
@@ -24423,7 +24423,7 @@
         <v>416</v>
       </c>
       <c r="AH329" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="330" spans="1:34">
@@ -24550,7 +24550,7 @@
         <v>414</v>
       </c>
       <c r="AH331" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="332" spans="1:34">
@@ -24612,7 +24612,7 @@
         <v>415</v>
       </c>
       <c r="AH332" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="333" spans="1:34">
@@ -24739,7 +24739,7 @@
         <v>415</v>
       </c>
       <c r="AH334" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="335" spans="1:34">
@@ -24801,7 +24801,7 @@
         <v>415</v>
       </c>
       <c r="AH335" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="336" spans="1:34">
@@ -24990,7 +24990,7 @@
         <v>414</v>
       </c>
       <c r="AH338" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="339" spans="1:34">
@@ -25052,7 +25052,7 @@
         <v>414</v>
       </c>
       <c r="AH339" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="340" spans="1:34">
@@ -25117,7 +25117,7 @@
         <v>414</v>
       </c>
       <c r="AH340" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="341" spans="1:34">
@@ -25371,7 +25371,7 @@
         <v>414</v>
       </c>
       <c r="AH344" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="345" spans="1:34">
@@ -25433,7 +25433,7 @@
         <v>414</v>
       </c>
       <c r="AH345" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="346" spans="1:34">
@@ -25687,7 +25687,7 @@
         <v>414</v>
       </c>
       <c r="AH349" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="350" spans="1:34">
@@ -28096,6 +28096,9 @@
       <c r="L387" s="1">
         <v>46311</v>
       </c>
+      <c r="M387" t="s">
+        <v>204</v>
+      </c>
       <c r="N387" t="s">
         <v>220</v>
       </c>
@@ -28113,6 +28116,9 @@
       </c>
       <c r="T387" t="s">
         <v>267</v>
+      </c>
+      <c r="W387" t="s">
+        <v>371</v>
       </c>
       <c r="AA387">
         <v>0</v>
@@ -28493,7 +28499,7 @@
         <v>265</v>
       </c>
       <c r="W393" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AA393">
         <v>0</v>
@@ -30318,7 +30324,7 @@
         <v>260</v>
       </c>
       <c r="W422" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="AA422">
         <v>0</v>
@@ -30708,7 +30714,7 @@
         <v>267</v>
       </c>
       <c r="W428" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="AA428">
         <v>0</v>
@@ -30776,7 +30782,7 @@
         <v>267</v>
       </c>
       <c r="W429" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AA429">
         <v>0</v>
@@ -30844,7 +30850,7 @@
         <v>260</v>
       </c>
       <c r="W430" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="AA430">
         <v>0</v>
@@ -30918,7 +30924,7 @@
         <v>414</v>
       </c>
       <c r="AH431" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="432" spans="1:34">
@@ -30983,7 +30989,7 @@
         <v>414</v>
       </c>
       <c r="AH432" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="433" spans="1:34">
@@ -31045,7 +31051,7 @@
         <v>414</v>
       </c>
       <c r="AH433" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="434" spans="1:34">
@@ -31104,7 +31110,7 @@
         <v>268</v>
       </c>
       <c r="W434" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="AA434">
         <v>0</v>
@@ -31169,7 +31175,7 @@
         <v>268</v>
       </c>
       <c r="W435" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="AA435">
         <v>0</v>
@@ -31237,7 +31243,7 @@
         <v>416</v>
       </c>
       <c r="AH436" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="437" spans="1:34">
@@ -31299,7 +31305,7 @@
         <v>416</v>
       </c>
       <c r="AH437" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="438" spans="1:34">
@@ -31364,7 +31370,7 @@
         <v>416</v>
       </c>
       <c r="AH438" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="439" spans="1:34">
@@ -31429,7 +31435,7 @@
         <v>416</v>
       </c>
       <c r="AH439" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="440" spans="1:34">
@@ -31491,7 +31497,7 @@
         <v>416</v>
       </c>
       <c r="AH440" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="441" spans="1:34">
@@ -31553,7 +31559,7 @@
         <v>274</v>
       </c>
       <c r="W441" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="AA441">
         <v>0</v>
@@ -31562,7 +31568,7 @@
         <v>416</v>
       </c>
       <c r="AH441" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="442" spans="1:34">
@@ -31624,7 +31630,7 @@
         <v>416</v>
       </c>
       <c r="AH442" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="443" spans="1:34">
@@ -31686,7 +31692,7 @@
         <v>416</v>
       </c>
       <c r="AH443" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="444" spans="1:34">
@@ -31748,7 +31754,7 @@
         <v>416</v>
       </c>
       <c r="AH444" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="445" spans="1:34">
@@ -31810,7 +31816,7 @@
         <v>416</v>
       </c>
       <c r="AH445" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="446" spans="1:34">
@@ -31872,7 +31878,7 @@
         <v>416</v>
       </c>
       <c r="AH446" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="447" spans="1:34">
@@ -31937,7 +31943,7 @@
         <v>416</v>
       </c>
       <c r="AH447" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="448" spans="1:34">
@@ -32002,7 +32008,7 @@
         <v>416</v>
       </c>
       <c r="AH448" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="449" spans="1:34">
@@ -32064,7 +32070,7 @@
         <v>416</v>
       </c>
       <c r="AH449" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="450" spans="1:34">
@@ -32129,7 +32135,7 @@
         <v>414</v>
       </c>
       <c r="AH450" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="451" spans="1:34">
@@ -32194,7 +32200,7 @@
         <v>414</v>
       </c>
       <c r="AH451" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="452" spans="1:34">
@@ -32259,7 +32265,7 @@
         <v>414</v>
       </c>
       <c r="AH452" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="453" spans="1:34">
@@ -32324,7 +32330,7 @@
         <v>414</v>
       </c>
       <c r="AH453" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="454" spans="1:34">
@@ -32386,7 +32392,7 @@
         <v>414</v>
       </c>
       <c r="AH454" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="455" spans="1:34">
@@ -32448,7 +32454,7 @@
         <v>414</v>
       </c>
       <c r="AH455" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="456" spans="1:34">
@@ -32510,7 +32516,7 @@
         <v>414</v>
       </c>
       <c r="AH456" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="457" spans="1:34">
@@ -37572,7 +37578,7 @@
         <v>262</v>
       </c>
       <c r="W539" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="AA539">
         <v>0</v>
@@ -37643,7 +37649,7 @@
         <v>0</v>
       </c>
       <c r="AB540" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG540" t="s">
         <v>414</v>
@@ -37711,7 +37717,7 @@
         <v>0</v>
       </c>
       <c r="AB541" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG541" t="s">
         <v>414</v>
@@ -37785,7 +37791,7 @@
         <v>414</v>
       </c>
       <c r="AH542" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="543" spans="1:34">
@@ -37850,13 +37856,13 @@
         <v>0</v>
       </c>
       <c r="AB543" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="AG543" t="s">
         <v>414</v>
       </c>
       <c r="AH543" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="544" spans="1:34">
@@ -38190,7 +38196,7 @@
         <v>0</v>
       </c>
       <c r="AB548" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG548" t="s">
         <v>416</v>
@@ -38261,7 +38267,7 @@
         <v>0</v>
       </c>
       <c r="AB549" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG549" t="s">
         <v>416</v>
@@ -38338,7 +38344,7 @@
         <v>414</v>
       </c>
       <c r="AH550" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="551" spans="1:34">
@@ -38409,7 +38415,7 @@
         <v>414</v>
       </c>
       <c r="AH551" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="552" spans="1:34">
@@ -38477,7 +38483,7 @@
         <v>414</v>
       </c>
       <c r="AH552" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="553" spans="1:34">
@@ -38542,13 +38548,13 @@
         <v>0</v>
       </c>
       <c r="AB553" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG553" t="s">
         <v>414</v>
       </c>
       <c r="AH553" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="554" spans="1:34">
@@ -38610,13 +38616,13 @@
         <v>0</v>
       </c>
       <c r="AB554" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG554" t="s">
         <v>414</v>
       </c>
       <c r="AH554" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="555" spans="1:34">
@@ -38746,13 +38752,13 @@
         <v>262</v>
       </c>
       <c r="W556" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AA556">
         <v>0</v>
       </c>
       <c r="AB556" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG556" t="s">
         <v>414</v>
@@ -38888,13 +38894,13 @@
         <v>274</v>
       </c>
       <c r="W558" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="AA558">
         <v>0</v>
       </c>
       <c r="AB558" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG558" t="s">
         <v>416</v>
@@ -38959,7 +38965,7 @@
         <v>0</v>
       </c>
       <c r="AB559" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG559" t="s">
         <v>416</v>
@@ -39024,13 +39030,13 @@
         <v>274</v>
       </c>
       <c r="W560" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AA560">
         <v>0</v>
       </c>
       <c r="AB560" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG560" t="s">
         <v>416</v>
@@ -39092,13 +39098,13 @@
         <v>260</v>
       </c>
       <c r="W561" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="AA561">
         <v>0</v>
       </c>
       <c r="AB561" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG561" t="s">
         <v>416</v>
@@ -39160,13 +39166,13 @@
         <v>262</v>
       </c>
       <c r="W562" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AA562">
         <v>0</v>
       </c>
       <c r="AB562" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG562" t="s">
         <v>416</v>
@@ -39231,7 +39237,7 @@
         <v>0</v>
       </c>
       <c r="AB563" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG563" t="s">
         <v>416</v>
@@ -39293,13 +39299,13 @@
         <v>263</v>
       </c>
       <c r="W564" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AA564">
         <v>0</v>
       </c>
       <c r="AB564" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG564" t="s">
         <v>416</v>
@@ -39361,13 +39367,13 @@
         <v>265</v>
       </c>
       <c r="W565" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AA565">
         <v>0</v>
       </c>
       <c r="AB565" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG565" t="s">
         <v>416</v>
@@ -39435,7 +39441,7 @@
         <v>0</v>
       </c>
       <c r="AB566" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG566" t="s">
         <v>416</v>
@@ -39497,13 +39503,13 @@
         <v>262</v>
       </c>
       <c r="W567" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AA567">
         <v>0</v>
       </c>
       <c r="AB567" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG567" t="s">
         <v>416</v>
@@ -39568,13 +39574,13 @@
         <v>274</v>
       </c>
       <c r="W568" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="AA568">
         <v>0</v>
       </c>
       <c r="AB568" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG568" t="s">
         <v>416</v>
@@ -39639,13 +39645,13 @@
         <v>274</v>
       </c>
       <c r="W569" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AA569">
         <v>0</v>
       </c>
       <c r="AB569" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG569" t="s">
         <v>416</v>
@@ -39707,13 +39713,13 @@
         <v>263</v>
       </c>
       <c r="W570" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="AA570">
         <v>0</v>
       </c>
       <c r="AB570" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG570" t="s">
         <v>416</v>
@@ -39775,13 +39781,13 @@
         <v>265</v>
       </c>
       <c r="W571" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="AA571">
         <v>0</v>
       </c>
       <c r="AB571" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG571" t="s">
         <v>416</v>
@@ -39843,13 +39849,13 @@
         <v>262</v>
       </c>
       <c r="W572" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="AA572">
         <v>0</v>
       </c>
       <c r="AB572" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG572" t="s">
         <v>416</v>
@@ -39914,7 +39920,7 @@
         <v>0</v>
       </c>
       <c r="AB573" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG573" t="s">
         <v>416</v>
@@ -39976,13 +39982,13 @@
         <v>263</v>
       </c>
       <c r="W574" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="AA574">
         <v>0</v>
       </c>
       <c r="AB574" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG574" t="s">
         <v>416</v>
@@ -40047,13 +40053,13 @@
         <v>274</v>
       </c>
       <c r="W575" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="AA575">
         <v>0</v>
       </c>
       <c r="AB575" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG575" t="s">
         <v>416</v>
@@ -40115,13 +40121,13 @@
         <v>265</v>
       </c>
       <c r="W576" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="AA576">
         <v>0</v>
       </c>
       <c r="AB576" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG576" t="s">
         <v>416</v>
@@ -40189,7 +40195,7 @@
         <v>0</v>
       </c>
       <c r="AB577" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG577" t="s">
         <v>416</v>
@@ -40251,13 +40257,13 @@
         <v>267</v>
       </c>
       <c r="W578" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="AA578">
         <v>0</v>
       </c>
       <c r="AB578" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG578" t="s">
         <v>416</v>
@@ -40322,7 +40328,7 @@
         <v>0</v>
       </c>
       <c r="AB579" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG579" t="s">
         <v>416</v>
@@ -40387,7 +40393,7 @@
         <v>0</v>
       </c>
       <c r="AB580" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG580" t="s">
         <v>416</v>
@@ -40452,7 +40458,7 @@
         <v>0</v>
       </c>
       <c r="AB581" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG581" t="s">
         <v>416</v>
@@ -40517,7 +40523,7 @@
         <v>0</v>
       </c>
       <c r="AB582" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG582" t="s">
         <v>416</v>
@@ -40582,7 +40588,7 @@
         <v>0</v>
       </c>
       <c r="AB583" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG583" t="s">
         <v>416</v>
@@ -41170,13 +41176,13 @@
         <v>263</v>
       </c>
       <c r="W592" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AA592">
         <v>0</v>
       </c>
       <c r="AB592" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG592" t="s">
         <v>414</v>
@@ -41238,13 +41244,13 @@
         <v>262</v>
       </c>
       <c r="W593" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="AA593">
         <v>0</v>
       </c>
       <c r="AB593" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG593" t="s">
         <v>414</v>
@@ -41309,13 +41315,13 @@
         <v>274</v>
       </c>
       <c r="W594" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AA594">
         <v>0</v>
       </c>
       <c r="AB594" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG594" t="s">
         <v>414</v>
@@ -41377,13 +41383,13 @@
         <v>262</v>
       </c>
       <c r="W595" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="AA595">
         <v>0</v>
       </c>
       <c r="AB595" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG595" t="s">
         <v>414</v>
@@ -41448,7 +41454,7 @@
         <v>0</v>
       </c>
       <c r="AB596" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG596" t="s">
         <v>414</v>
@@ -41513,7 +41519,7 @@
         <v>0</v>
       </c>
       <c r="AB597" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG597" t="s">
         <v>414</v>
@@ -41575,7 +41581,7 @@
         <v>260</v>
       </c>
       <c r="W598" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AG598" t="s">
         <v>415</v>
@@ -41640,13 +41646,13 @@
         <v>260</v>
       </c>
       <c r="W599" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG599" t="s">
         <v>415</v>
       </c>
       <c r="AH599" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="600" spans="1:34">
@@ -41705,7 +41711,7 @@
         <v>270</v>
       </c>
       <c r="W600" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="AG600" t="s">
         <v>414</v>
@@ -42225,7 +42231,7 @@
         <v>260</v>
       </c>
       <c r="W608" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG608" t="s">
         <v>414</v>
@@ -42287,7 +42293,7 @@
         <v>273</v>
       </c>
       <c r="W609" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG609" t="s">
         <v>414</v>
@@ -42349,7 +42355,7 @@
         <v>273</v>
       </c>
       <c r="W610" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG610" t="s">
         <v>414</v>
@@ -42411,7 +42417,7 @@
         <v>260</v>
       </c>
       <c r="W611" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG611" t="s">
         <v>414</v>
@@ -42473,7 +42479,7 @@
         <v>273</v>
       </c>
       <c r="W612" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG612" t="s">
         <v>414</v>
@@ -42535,7 +42541,7 @@
         <v>273</v>
       </c>
       <c r="W613" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG613" t="s">
         <v>414</v>
@@ -42597,7 +42603,7 @@
         <v>260</v>
       </c>
       <c r="W614" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG614" t="s">
         <v>414</v>
@@ -42659,7 +42665,7 @@
         <v>273</v>
       </c>
       <c r="W615" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG615" t="s">
         <v>414</v>
@@ -42721,7 +42727,7 @@
         <v>273</v>
       </c>
       <c r="W616" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG616" t="s">
         <v>414</v>
@@ -42783,7 +42789,7 @@
         <v>260</v>
       </c>
       <c r="W617" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG617" t="s">
         <v>414</v>
@@ -42845,7 +42851,7 @@
         <v>273</v>
       </c>
       <c r="W618" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG618" t="s">
         <v>414</v>
@@ -42907,7 +42913,7 @@
         <v>273</v>
       </c>
       <c r="W619" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG619" t="s">
         <v>414</v>
@@ -42969,7 +42975,7 @@
         <v>260</v>
       </c>
       <c r="W620" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG620" t="s">
         <v>414</v>
@@ -43031,7 +43037,7 @@
         <v>273</v>
       </c>
       <c r="W621" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG621" t="s">
         <v>414</v>
@@ -43093,7 +43099,7 @@
         <v>273</v>
       </c>
       <c r="W622" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG622" t="s">
         <v>414</v>
@@ -43155,7 +43161,7 @@
         <v>260</v>
       </c>
       <c r="W623" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG623" t="s">
         <v>414</v>
@@ -43217,7 +43223,7 @@
         <v>273</v>
       </c>
       <c r="W624" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG624" t="s">
         <v>414</v>
@@ -43279,7 +43285,7 @@
         <v>273</v>
       </c>
       <c r="W625" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG625" t="s">
         <v>414</v>
@@ -43341,7 +43347,7 @@
         <v>260</v>
       </c>
       <c r="W626" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG626" t="s">
         <v>414</v>
@@ -43403,7 +43409,7 @@
         <v>273</v>
       </c>
       <c r="W627" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG627" t="s">
         <v>414</v>
@@ -43465,7 +43471,7 @@
         <v>273</v>
       </c>
       <c r="W628" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG628" t="s">
         <v>414</v>
@@ -43527,7 +43533,7 @@
         <v>260</v>
       </c>
       <c r="W629" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG629" t="s">
         <v>414</v>
@@ -43589,7 +43595,7 @@
         <v>273</v>
       </c>
       <c r="W630" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG630" t="s">
         <v>414</v>
@@ -43651,7 +43657,7 @@
         <v>273</v>
       </c>
       <c r="W631" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG631" t="s">
         <v>414</v>
@@ -43713,7 +43719,7 @@
         <v>260</v>
       </c>
       <c r="W632" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG632" t="s">
         <v>414</v>
@@ -43775,7 +43781,7 @@
         <v>273</v>
       </c>
       <c r="W633" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG633" t="s">
         <v>414</v>
@@ -43837,7 +43843,7 @@
         <v>273</v>
       </c>
       <c r="W634" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG634" t="s">
         <v>414</v>
@@ -43899,7 +43905,7 @@
         <v>260</v>
       </c>
       <c r="W635" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG635" t="s">
         <v>414</v>
@@ -43961,7 +43967,7 @@
         <v>273</v>
       </c>
       <c r="W636" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG636" t="s">
         <v>414</v>
@@ -44023,7 +44029,7 @@
         <v>273</v>
       </c>
       <c r="W637" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG637" t="s">
         <v>414</v>
@@ -44085,7 +44091,7 @@
         <v>260</v>
       </c>
       <c r="W638" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG638" t="s">
         <v>414</v>
@@ -44147,7 +44153,7 @@
         <v>273</v>
       </c>
       <c r="W639" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG639" t="s">
         <v>414</v>
@@ -44209,7 +44215,7 @@
         <v>273</v>
       </c>
       <c r="W640" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG640" t="s">
         <v>414</v>
@@ -44271,7 +44277,7 @@
         <v>260</v>
       </c>
       <c r="W641" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG641" t="s">
         <v>414</v>
@@ -44333,7 +44339,7 @@
         <v>273</v>
       </c>
       <c r="W642" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG642" t="s">
         <v>414</v>
@@ -44395,7 +44401,7 @@
         <v>273</v>
       </c>
       <c r="W643" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG643" t="s">
         <v>414</v>
@@ -44457,13 +44463,13 @@
         <v>263</v>
       </c>
       <c r="W644" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="AE644" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="AF644" t="s">
-        <v>413</v>
+        <v>202</v>
       </c>
       <c r="AG644" t="s">
         <v>414</v>
@@ -44525,13 +44531,13 @@
         <v>262</v>
       </c>
       <c r="W645" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="AE645" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AF645" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="AG645" t="s">
         <v>414</v>
@@ -44593,7 +44599,7 @@
         <v>260</v>
       </c>
       <c r="W646" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="AG646" t="s">
         <v>414</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-22 09:17
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1494,8 +1494,8 @@
 Sem procuração, aguardando emissão do cliente para prosseguirmos com escituraçã - Data Comentário: 16/10/2026 15:33</t>
   </si>
   <si>
-    <t>Aguardando login e senha com Paralegal   Previsão para conclusão dia 22/10/2026 
-Cliente sem procuração federal para envio da REINF, aberto chamado para o paralegal n° 85064 - Data Comentário: 21/10/2026 18:27</t>
+    <t>Aguardando a Liberação da Gerência de Contas   Previsão para conclusão dia 30/10/2026 
+Cliente sem procuração federal para envio da REINF, aberto chamado para o paralegal n° 85064 - Data Comentário: 22/10/2026 08:40</t>
   </si>
   <si>
     <t>Aguardando login e senha com Paralegal   Previsão para conclusão dia 22/10/2026 
@@ -44365,7 +44365,7 @@
         <v>46308</v>
       </c>
       <c r="M612" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="N612" t="s">
         <v>221</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-27 15:05
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -835,8 +835,8 @@
     <t>F</t>
   </si>
   <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/10/2026 
-Sem procuração, aguardando emissão do cliente para darmos inicio aos processos - Data Comentário: 23/10/2026 16:33</t>
+    <t>Aguardando a Liberação da Gerência de Contas   Previsão para conclusão dia 30/10/2026 
+consulta em 27/10/26 ainda não tem procuração, a empresa precisa fazer certificado da empresa 7095- Brasil Administradora de Serviços, David já falou com gerente Lopes, o mesmo está ciente - Data Comentário: 27/10/2026 14:24</t>
   </si>
   <si>
     <t>Para 2.300,00 a partir de 01/09/2026 alteração de função para pleno. - Data Comentário: 02/10/2026 14:39</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-28 11:17
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9900" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9886" uniqueCount="526">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1982,7 +1982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH627"/>
+  <dimension ref="A1:AH626"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:34">
@@ -47664,68 +47664,6 @@
         <v>519</v>
       </c>
     </row>
-    <row r="627" spans="1:34">
-      <c r="A627">
-        <v>7095</v>
-      </c>
-      <c r="B627" t="s">
-        <v>50</v>
-      </c>
-      <c r="C627" t="s">
-        <v>56</v>
-      </c>
-      <c r="D627" t="s">
-        <v>58</v>
-      </c>
-      <c r="E627" t="s">
-        <v>60</v>
-      </c>
-      <c r="F627" t="s">
-        <v>62</v>
-      </c>
-      <c r="G627">
-        <v>1877</v>
-      </c>
-      <c r="H627">
-        <v>0</v>
-      </c>
-      <c r="I627" t="s">
-        <v>68</v>
-      </c>
-      <c r="J627" t="s">
-        <v>139</v>
-      </c>
-      <c r="L627" s="1">
-        <v>46323</v>
-      </c>
-      <c r="N627" t="s">
-        <v>216</v>
-      </c>
-      <c r="O627">
-        <v>18292290</v>
-      </c>
-      <c r="P627" t="s">
-        <v>237</v>
-      </c>
-      <c r="Q627" t="s">
-        <v>250</v>
-      </c>
-      <c r="S627">
-        <v>0</v>
-      </c>
-      <c r="T627" t="s">
-        <v>251</v>
-      </c>
-      <c r="U627" t="s">
-        <v>265</v>
-      </c>
-      <c r="AG627" t="s">
-        <v>520</v>
-      </c>
-      <c r="AH627" t="s">
-        <v>507</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-28 17:01
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1174,7 +1174,7 @@
 Prazo de conclusão 28/10/2026 - Data Comentário: 27/10/2026 17:50</t>
   </si>
   <si>
-    <t>3. Folha, Aguardando Resumo p/ Processamento  Previsão para conclusão dia 28/10/2026 - Data Comentário: 26/10/2026 14:06</t>
+    <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 29/10/2026 - Data Comentário: 28/10/2026 16:39</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/10/2026 
@@ -25061,7 +25061,7 @@
         <v>46323</v>
       </c>
       <c r="M315" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="N315" t="s">
         <v>215</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-29 15:34
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9833" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9834" uniqueCount="525">
   <si>
     <t>CodCliente</t>
   </si>
@@ -23650,10 +23650,10 @@
     </row>
     <row r="295" spans="1:34">
       <c r="A295">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B295" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C295" t="s">
         <v>53</v>
@@ -23686,10 +23686,10 @@
         <v>209</v>
       </c>
       <c r="O295">
-        <v>17967986</v>
+        <v>17042386</v>
       </c>
       <c r="P295" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q295" t="s">
         <v>243</v>
@@ -23698,7 +23698,7 @@
         <v>0</v>
       </c>
       <c r="T295" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="U295" t="s">
         <v>257</v>
@@ -23713,15 +23713,15 @@
         <v>517</v>
       </c>
       <c r="AH295" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
     </row>
     <row r="296" spans="1:34">
       <c r="A296">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B296" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C296" t="s">
         <v>53</v>
@@ -23754,10 +23754,10 @@
         <v>209</v>
       </c>
       <c r="O296">
-        <v>17042386</v>
+        <v>18178273</v>
       </c>
       <c r="P296" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q296" t="s">
         <v>243</v>
@@ -23766,13 +23766,10 @@
         <v>0</v>
       </c>
       <c r="T296" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="U296" t="s">
-        <v>257</v>
-      </c>
-      <c r="V296" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="AA296">
         <v>0</v>
@@ -23781,21 +23778,21 @@
         <v>517</v>
       </c>
       <c r="AH296" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
     </row>
     <row r="297" spans="1:34">
       <c r="A297">
-        <v>6949</v>
+        <v>6963</v>
       </c>
       <c r="B297" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C297" t="s">
         <v>53</v>
       </c>
       <c r="D297" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E297" t="s">
         <v>57</v>
@@ -23804,7 +23801,7 @@
         <v>59</v>
       </c>
       <c r="G297">
-        <v>1651</v>
+        <v>10992</v>
       </c>
       <c r="H297">
         <v>0</v>
@@ -23813,40 +23810,40 @@
         <v>61</v>
       </c>
       <c r="J297" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L297" s="1">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="N297" t="s">
         <v>209</v>
       </c>
       <c r="O297">
-        <v>18178273</v>
+        <v>18249093</v>
       </c>
       <c r="P297" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="Q297" t="s">
         <v>243</v>
       </c>
       <c r="S297">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T297" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U297" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AA297">
         <v>0</v>
       </c>
       <c r="AG297" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="AH297" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
     </row>
     <row r="298" spans="1:34">
@@ -23869,7 +23866,7 @@
         <v>59</v>
       </c>
       <c r="G298">
-        <v>10992</v>
+        <v>7875</v>
       </c>
       <c r="H298">
         <v>0</v>
@@ -23878,7 +23875,7 @@
         <v>61</v>
       </c>
       <c r="J298" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L298" s="1">
         <v>46325</v>
@@ -23887,7 +23884,7 @@
         <v>209</v>
       </c>
       <c r="O298">
-        <v>18249093</v>
+        <v>18200057</v>
       </c>
       <c r="P298" t="s">
         <v>218</v>
@@ -23916,16 +23913,16 @@
     </row>
     <row r="299" spans="1:34">
       <c r="A299">
-        <v>6963</v>
+        <v>5417</v>
       </c>
       <c r="B299" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C299" t="s">
         <v>53</v>
       </c>
       <c r="D299" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E299" t="s">
         <v>57</v>
@@ -23934,63 +23931,63 @@
         <v>59</v>
       </c>
       <c r="G299">
-        <v>7875</v>
+        <v>1582</v>
       </c>
       <c r="H299">
         <v>0</v>
       </c>
       <c r="I299" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J299" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L299" s="1">
-        <v>46325</v>
+        <v>46324</v>
       </c>
       <c r="N299" t="s">
         <v>209</v>
       </c>
       <c r="O299">
-        <v>18200057</v>
+        <v>17398914</v>
       </c>
       <c r="P299" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="Q299" t="s">
         <v>243</v>
       </c>
       <c r="S299">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T299" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="U299" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AA299">
         <v>0</v>
       </c>
       <c r="AG299" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="AH299" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
     </row>
     <row r="300" spans="1:34">
       <c r="A300">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B300" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C300" t="s">
         <v>53</v>
       </c>
       <c r="D300" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E300" t="s">
         <v>57</v>
@@ -23999,7 +23996,7 @@
         <v>59</v>
       </c>
       <c r="G300">
-        <v>1582</v>
+        <v>10988</v>
       </c>
       <c r="H300">
         <v>0</v>
@@ -24008,54 +24005,54 @@
         <v>62</v>
       </c>
       <c r="J300" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L300" s="1">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="N300" t="s">
         <v>209</v>
       </c>
       <c r="O300">
-        <v>17398914</v>
+        <v>16962445</v>
       </c>
       <c r="P300" t="s">
-        <v>219</v>
+        <v>236</v>
       </c>
       <c r="Q300" t="s">
         <v>243</v>
       </c>
       <c r="S300">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T300" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="U300" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AA300">
         <v>0</v>
       </c>
       <c r="AG300" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="AH300" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="301" spans="1:34">
       <c r="A301">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B301" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C301" t="s">
         <v>53</v>
       </c>
       <c r="D301" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E301" t="s">
         <v>57</v>
@@ -24064,7 +24061,7 @@
         <v>59</v>
       </c>
       <c r="G301">
-        <v>10988</v>
+        <v>7874</v>
       </c>
       <c r="H301">
         <v>0</v>
@@ -24073,7 +24070,7 @@
         <v>62</v>
       </c>
       <c r="J301" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L301" s="1">
         <v>46325</v>
@@ -24082,10 +24079,10 @@
         <v>209</v>
       </c>
       <c r="O301">
-        <v>16962445</v>
+        <v>18096768</v>
       </c>
       <c r="P301" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="Q301" t="s">
         <v>243</v>
@@ -24094,10 +24091,13 @@
         <v>-1</v>
       </c>
       <c r="T301" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="U301" t="s">
-        <v>257</v>
+        <v>258</v>
+      </c>
+      <c r="V301" t="s">
+        <v>261</v>
       </c>
       <c r="AA301">
         <v>0</v>
@@ -24111,10 +24111,10 @@
     </row>
     <row r="302" spans="1:34">
       <c r="A302">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B302" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C302" t="s">
         <v>53</v>
@@ -24129,28 +24129,31 @@
         <v>59</v>
       </c>
       <c r="G302">
-        <v>7874</v>
+        <v>11542</v>
       </c>
       <c r="H302">
         <v>0</v>
       </c>
       <c r="I302" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J302" t="s">
-        <v>130</v>
+        <v>73</v>
       </c>
       <c r="L302" s="1">
         <v>46325</v>
       </c>
+      <c r="M302" t="s">
+        <v>183</v>
+      </c>
       <c r="N302" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="O302">
-        <v>18096768</v>
+        <v>18248557</v>
       </c>
       <c r="P302" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="Q302" t="s">
         <v>243</v>
@@ -24159,30 +24162,30 @@
         <v>-1</v>
       </c>
       <c r="T302" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="U302" t="s">
         <v>258</v>
       </c>
-      <c r="V302" t="s">
-        <v>261</v>
+      <c r="W302" t="s">
+        <v>366</v>
       </c>
       <c r="AA302">
         <v>0</v>
       </c>
       <c r="AG302" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="AH302" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
     </row>
     <row r="303" spans="1:34">
       <c r="A303">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B303" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C303" t="s">
         <v>53</v>
@@ -24218,10 +24221,10 @@
         <v>211</v>
       </c>
       <c r="O303">
-        <v>18248557</v>
+        <v>18190473</v>
       </c>
       <c r="P303" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Q303" t="s">
         <v>243</v>
@@ -24230,13 +24233,13 @@
         <v>-1</v>
       </c>
       <c r="T303" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="U303" t="s">
         <v>258</v>
       </c>
       <c r="W303" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="AA303">
         <v>0</v>
@@ -24245,7 +24248,7 @@
         <v>518</v>
       </c>
       <c r="AH303" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
     </row>
     <row r="304" spans="1:34">
@@ -24268,7 +24271,7 @@
         <v>59</v>
       </c>
       <c r="G304">
-        <v>11542</v>
+        <v>11541</v>
       </c>
       <c r="H304">
         <v>0</v>
@@ -24277,7 +24280,7 @@
         <v>60</v>
       </c>
       <c r="J304" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L304" s="1">
         <v>46325</v>
@@ -24289,7 +24292,7 @@
         <v>211</v>
       </c>
       <c r="O304">
-        <v>18190473</v>
+        <v>18190467</v>
       </c>
       <c r="P304" t="s">
         <v>222</v>
@@ -24307,7 +24310,7 @@
         <v>258</v>
       </c>
       <c r="W304" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AA304">
         <v>0</v>
@@ -24339,7 +24342,7 @@
         <v>59</v>
       </c>
       <c r="G305">
-        <v>11541</v>
+        <v>6348</v>
       </c>
       <c r="H305">
         <v>0</v>
@@ -24348,7 +24351,7 @@
         <v>60</v>
       </c>
       <c r="J305" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="L305" s="1">
         <v>46325</v>
@@ -24357,13 +24360,13 @@
         <v>183</v>
       </c>
       <c r="N305" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="O305">
-        <v>18190467</v>
+        <v>18272235</v>
       </c>
       <c r="P305" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="Q305" t="s">
         <v>243</v>
@@ -24378,24 +24381,24 @@
         <v>258</v>
       </c>
       <c r="W305" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AA305">
         <v>0</v>
       </c>
       <c r="AG305" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="AH305" t="s">
-        <v>514</v>
+        <v>523</v>
       </c>
     </row>
     <row r="306" spans="1:34">
       <c r="A306">
-        <v>6949</v>
+        <v>6704</v>
       </c>
       <c r="B306" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C306" t="s">
         <v>53</v>
@@ -24410,16 +24413,16 @@
         <v>59</v>
       </c>
       <c r="G306">
-        <v>6348</v>
+        <v>949</v>
       </c>
       <c r="H306">
         <v>0</v>
       </c>
       <c r="I306" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="J306" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="L306" s="1">
         <v>46325</v>
@@ -24428,13 +24431,13 @@
         <v>183</v>
       </c>
       <c r="N306" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O306">
-        <v>18272235</v>
+        <v>17952332</v>
       </c>
       <c r="P306" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="Q306" t="s">
         <v>243</v>
@@ -24443,13 +24446,16 @@
         <v>-1</v>
       </c>
       <c r="T306" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="U306" t="s">
         <v>258</v>
       </c>
+      <c r="V306" t="s">
+        <v>261</v>
+      </c>
       <c r="W306" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="AA306">
         <v>0</v>
@@ -24457,22 +24463,19 @@
       <c r="AG306" t="s">
         <v>517</v>
       </c>
-      <c r="AH306" t="s">
-        <v>523</v>
-      </c>
     </row>
     <row r="307" spans="1:34">
       <c r="A307">
-        <v>6704</v>
+        <v>6404</v>
       </c>
       <c r="B307" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C307" t="s">
         <v>53</v>
       </c>
       <c r="D307" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E307" t="s">
         <v>57</v>
@@ -24481,7 +24484,7 @@
         <v>59</v>
       </c>
       <c r="G307">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="H307">
         <v>0</v>
@@ -24490,7 +24493,7 @@
         <v>65</v>
       </c>
       <c r="J307" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L307" s="1">
         <v>46325</v>
@@ -24502,7 +24505,7 @@
         <v>209</v>
       </c>
       <c r="O307">
-        <v>17952332</v>
+        <v>16962100</v>
       </c>
       <c r="P307" t="s">
         <v>234</v>
@@ -24514,16 +24517,13 @@
         <v>-1</v>
       </c>
       <c r="T307" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="U307" t="s">
-        <v>258</v>
-      </c>
-      <c r="V307" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="W307" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="AA307">
         <v>0</v>
@@ -24534,10 +24534,10 @@
     </row>
     <row r="308" spans="1:34">
       <c r="A308">
-        <v>6404</v>
+        <v>6703</v>
       </c>
       <c r="B308" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C308" t="s">
         <v>53</v>
@@ -24573,7 +24573,7 @@
         <v>209</v>
       </c>
       <c r="O308">
-        <v>16962100</v>
+        <v>17941139</v>
       </c>
       <c r="P308" t="s">
         <v>234</v>
@@ -24585,13 +24585,13 @@
         <v>-1</v>
       </c>
       <c r="T308" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="U308" t="s">
         <v>257</v>
       </c>
       <c r="W308" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AA308">
         <v>0</v>
@@ -24602,16 +24602,16 @@
     </row>
     <row r="309" spans="1:34">
       <c r="A309">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B309" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C309" t="s">
         <v>53</v>
       </c>
       <c r="D309" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E309" t="s">
         <v>57</v>
@@ -24620,31 +24620,28 @@
         <v>59</v>
       </c>
       <c r="G309">
-        <v>948</v>
+        <v>957</v>
       </c>
       <c r="H309">
         <v>0</v>
       </c>
       <c r="I309" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J309" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L309" s="1">
         <v>46325</v>
       </c>
-      <c r="M309" t="s">
-        <v>183</v>
-      </c>
       <c r="N309" t="s">
         <v>209</v>
       </c>
       <c r="O309">
-        <v>17941139</v>
+        <v>17398900</v>
       </c>
       <c r="P309" t="s">
-        <v>234</v>
+        <v>57</v>
       </c>
       <c r="Q309" t="s">
         <v>243</v>
@@ -24653,27 +24650,24 @@
         <v>-1</v>
       </c>
       <c r="T309" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="U309" t="s">
-        <v>257</v>
-      </c>
-      <c r="W309" t="s">
-        <v>372</v>
+        <v>258</v>
       </c>
       <c r="AA309">
         <v>0</v>
       </c>
       <c r="AG309" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="310" spans="1:34">
       <c r="A310">
-        <v>5417</v>
+        <v>6627</v>
       </c>
       <c r="B310" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C310" t="s">
         <v>53</v>
@@ -24706,7 +24700,7 @@
         <v>209</v>
       </c>
       <c r="O310">
-        <v>17398900</v>
+        <v>17042326</v>
       </c>
       <c r="P310" t="s">
         <v>57</v>
@@ -24718,10 +24712,13 @@
         <v>-1</v>
       </c>
       <c r="T310" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="U310" t="s">
-        <v>258</v>
+        <v>257</v>
+      </c>
+      <c r="V310" t="s">
+        <v>260</v>
       </c>
       <c r="AA310">
         <v>0</v>
@@ -24750,34 +24747,37 @@
         <v>59</v>
       </c>
       <c r="G311">
-        <v>957</v>
+        <v>7869</v>
       </c>
       <c r="H311">
         <v>0</v>
       </c>
       <c r="I311" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="J311" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L311" s="1">
-        <v>46325</v>
+        <v>46321</v>
       </c>
       <c r="N311" t="s">
         <v>209</v>
       </c>
       <c r="O311">
-        <v>17042326</v>
+        <v>17042548</v>
       </c>
       <c r="P311" t="s">
-        <v>57</v>
+        <v>216</v>
       </c>
       <c r="Q311" t="s">
-        <v>243</v>
+        <v>242</v>
+      </c>
+      <c r="R311" s="1">
+        <v>46317.63681168982</v>
       </c>
       <c r="S311">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="T311" t="s">
         <v>246</v>
@@ -24791,22 +24791,28 @@
       <c r="AA311">
         <v>0</v>
       </c>
+      <c r="AB311" t="s">
+        <v>509</v>
+      </c>
       <c r="AG311" t="s">
         <v>516</v>
       </c>
+      <c r="AH311" t="s">
+        <v>520</v>
+      </c>
     </row>
     <row r="312" spans="1:34">
       <c r="A312">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B312" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C312" t="s">
         <v>53</v>
       </c>
       <c r="D312" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E312" t="s">
         <v>57</v>
@@ -24833,7 +24839,7 @@
         <v>209</v>
       </c>
       <c r="O312">
-        <v>17042548</v>
+        <v>16960049</v>
       </c>
       <c r="P312" t="s">
         <v>216</v>
@@ -24842,7 +24848,7 @@
         <v>242</v>
       </c>
       <c r="R312" s="1">
-        <v>46317.63681168982</v>
+        <v>46317.63681204861</v>
       </c>
       <c r="S312">
         <v>3</v>
@@ -24871,16 +24877,16 @@
     </row>
     <row r="313" spans="1:34">
       <c r="A313">
-        <v>6628</v>
+        <v>6949</v>
       </c>
       <c r="B313" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C313" t="s">
         <v>53</v>
       </c>
       <c r="D313" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E313" t="s">
         <v>57</v>
@@ -24907,28 +24913,25 @@
         <v>209</v>
       </c>
       <c r="O313">
-        <v>16960049</v>
+        <v>18178301</v>
       </c>
       <c r="P313" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q313" t="s">
         <v>242</v>
       </c>
       <c r="R313" s="1">
-        <v>46317.63681204861</v>
+        <v>46317.63682094908</v>
       </c>
       <c r="S313">
         <v>3</v>
       </c>
       <c r="T313" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="U313" t="s">
-        <v>257</v>
-      </c>
-      <c r="V313" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="AA313">
         <v>0</v>
@@ -24940,21 +24943,21 @@
         <v>516</v>
       </c>
       <c r="AH313" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
     </row>
     <row r="314" spans="1:34">
       <c r="A314">
-        <v>6949</v>
+        <v>6628</v>
       </c>
       <c r="B314" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C314" t="s">
         <v>53</v>
       </c>
       <c r="D314" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E314" t="s">
         <v>57</v>
@@ -24963,7 +24966,7 @@
         <v>59</v>
       </c>
       <c r="G314">
-        <v>7869</v>
+        <v>1650</v>
       </c>
       <c r="H314">
         <v>0</v>
@@ -24972,66 +24975,69 @@
         <v>61</v>
       </c>
       <c r="J314" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L314" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="N314" t="s">
         <v>209</v>
       </c>
       <c r="O314">
-        <v>18178301</v>
+        <v>16959975</v>
       </c>
       <c r="P314" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q314" t="s">
         <v>242</v>
       </c>
       <c r="R314" s="1">
-        <v>46317.63682094908</v>
+        <v>46295.04093612268</v>
       </c>
       <c r="S314">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T314" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="U314" t="s">
-        <v>258</v>
+        <v>257</v>
+      </c>
+      <c r="V314" t="s">
+        <v>260</v>
       </c>
       <c r="AA314">
         <v>0</v>
       </c>
       <c r="AB314" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="AG314" t="s">
         <v>516</v>
       </c>
       <c r="AH314" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
     </row>
     <row r="315" spans="1:34">
       <c r="A315">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B315" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C315" t="s">
         <v>53</v>
       </c>
       <c r="D315" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E315" t="s">
         <v>57</v>
       </c>
       <c r="F315" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G315">
         <v>1650</v>
@@ -25052,29 +25058,26 @@
         <v>209</v>
       </c>
       <c r="O315">
-        <v>16959975</v>
+        <v>18163668</v>
       </c>
       <c r="P315" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Q315" t="s">
         <v>242</v>
       </c>
       <c r="R315" s="1">
-        <v>46295.04093612268</v>
+        <v>46295.04098302083</v>
       </c>
       <c r="S315">
         <v>1</v>
       </c>
       <c r="T315" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="U315" t="s">
         <v>257</v>
       </c>
-      <c r="V315" t="s">
-        <v>260</v>
-      </c>
       <c r="AA315">
         <v>0</v>
       </c>
@@ -25090,10 +25093,10 @@
     </row>
     <row r="316" spans="1:34">
       <c r="A316">
-        <v>6945</v>
+        <v>6627</v>
       </c>
       <c r="B316" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C316" t="s">
         <v>53</v>
@@ -25105,10 +25108,10 @@
         <v>57</v>
       </c>
       <c r="F316" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G316">
-        <v>1650</v>
+        <v>6892</v>
       </c>
       <c r="H316">
         <v>0</v>
@@ -25117,43 +25120,52 @@
         <v>61</v>
       </c>
       <c r="J316" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="L316" s="1">
-        <v>46323</v>
+        <v>46321</v>
+      </c>
+      <c r="M316" t="s">
+        <v>200</v>
       </c>
       <c r="N316" t="s">
         <v>209</v>
       </c>
       <c r="O316">
-        <v>18163668</v>
+        <v>17042488</v>
       </c>
       <c r="P316" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="Q316" t="s">
         <v>242</v>
       </c>
       <c r="R316" s="1">
-        <v>46295.04098302083</v>
+        <v>46324.49322108796</v>
       </c>
       <c r="S316">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T316" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="U316" t="s">
         <v>257</v>
       </c>
+      <c r="V316" t="s">
+        <v>260</v>
+      </c>
+      <c r="W316" t="s">
+        <v>360</v>
+      </c>
       <c r="AA316">
         <v>0</v>
       </c>
       <c r="AB316" t="s">
-        <v>505</v>
+        <v>216</v>
       </c>
       <c r="AG316" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="AH316" t="s">
         <v>520</v>
@@ -25161,16 +25173,16 @@
     </row>
     <row r="317" spans="1:34">
       <c r="A317">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B317" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C317" t="s">
         <v>53</v>
       </c>
       <c r="D317" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E317" t="s">
         <v>57</v>
@@ -25193,14 +25205,11 @@
       <c r="L317" s="1">
         <v>46321</v>
       </c>
-      <c r="M317" t="s">
-        <v>200</v>
-      </c>
       <c r="N317" t="s">
         <v>209</v>
       </c>
       <c r="O317">
-        <v>17042488</v>
+        <v>16960025</v>
       </c>
       <c r="P317" t="s">
         <v>216</v>
@@ -25209,7 +25218,7 @@
         <v>242</v>
       </c>
       <c r="R317" s="1">
-        <v>46324.49322108796</v>
+        <v>46318.63617619213</v>
       </c>
       <c r="S317">
         <v>3</v>
@@ -25223,14 +25232,11 @@
       <c r="V317" t="s">
         <v>260</v>
       </c>
-      <c r="W317" t="s">
-        <v>360</v>
-      </c>
       <c r="AA317">
         <v>0</v>
       </c>
       <c r="AB317" t="s">
-        <v>216</v>
+        <v>509</v>
       </c>
       <c r="AG317" t="s">
         <v>518</v>
@@ -25241,16 +25247,16 @@
     </row>
     <row r="318" spans="1:34">
       <c r="A318">
-        <v>6628</v>
+        <v>6962</v>
       </c>
       <c r="B318" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C318" t="s">
         <v>53</v>
       </c>
       <c r="D318" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E318" t="s">
         <v>57</v>
@@ -25273,38 +25279,41 @@
       <c r="L318" s="1">
         <v>46321</v>
       </c>
+      <c r="M318" t="s">
+        <v>200</v>
+      </c>
       <c r="N318" t="s">
         <v>209</v>
       </c>
       <c r="O318">
-        <v>16960025</v>
+        <v>18187956</v>
       </c>
       <c r="P318" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="Q318" t="s">
         <v>242</v>
       </c>
       <c r="R318" s="1">
-        <v>46318.63617619213</v>
+        <v>46322.698238125</v>
       </c>
       <c r="S318">
         <v>3</v>
       </c>
       <c r="T318" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="U318" t="s">
-        <v>257</v>
-      </c>
-      <c r="V318" t="s">
-        <v>260</v>
+        <v>259</v>
+      </c>
+      <c r="W318" t="s">
+        <v>360</v>
       </c>
       <c r="AA318">
         <v>0</v>
       </c>
       <c r="AB318" t="s">
-        <v>509</v>
+        <v>218</v>
       </c>
       <c r="AG318" t="s">
         <v>518</v>
@@ -25315,10 +25324,10 @@
     </row>
     <row r="319" spans="1:34">
       <c r="A319">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B319" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C319" t="s">
         <v>53</v>
@@ -25354,7 +25363,7 @@
         <v>209</v>
       </c>
       <c r="O319">
-        <v>18187956</v>
+        <v>18187894</v>
       </c>
       <c r="P319" t="s">
         <v>218</v>
@@ -25363,7 +25372,7 @@
         <v>242</v>
       </c>
       <c r="R319" s="1">
-        <v>46322.698238125</v>
+        <v>46323.49171587963</v>
       </c>
       <c r="S319">
         <v>3</v>
@@ -25392,16 +25401,16 @@
     </row>
     <row r="320" spans="1:34">
       <c r="A320">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B320" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C320" t="s">
         <v>53</v>
       </c>
       <c r="D320" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E320" t="s">
         <v>57</v>
@@ -25410,7 +25419,7 @@
         <v>59</v>
       </c>
       <c r="G320">
-        <v>6892</v>
+        <v>1651</v>
       </c>
       <c r="H320">
         <v>0</v>
@@ -25419,52 +25428,49 @@
         <v>61</v>
       </c>
       <c r="J320" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="L320" s="1">
-        <v>46321</v>
-      </c>
-      <c r="M320" t="s">
-        <v>200</v>
+        <v>46324</v>
       </c>
       <c r="N320" t="s">
         <v>209</v>
       </c>
       <c r="O320">
-        <v>18187894</v>
+        <v>17967986</v>
       </c>
       <c r="P320" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="Q320" t="s">
         <v>242</v>
       </c>
       <c r="R320" s="1">
-        <v>46323.49171587963</v>
+        <v>46324.63946440972</v>
       </c>
       <c r="S320">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T320" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="U320" t="s">
-        <v>259</v>
-      </c>
-      <c r="W320" t="s">
-        <v>360</v>
+        <v>257</v>
+      </c>
+      <c r="V320" t="s">
+        <v>260</v>
       </c>
       <c r="AA320">
         <v>0</v>
       </c>
       <c r="AB320" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AG320" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="AH320" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
     </row>
     <row r="321" spans="1:34">

</xml_diff>

<commit_message>
Atualização automática: 2026-10-30 11:31
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9907" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9912" uniqueCount="540">
   <si>
     <t>CodCliente</t>
   </si>
@@ -403,37 +403,37 @@
     <t>Agenda de Reunião</t>
   </si>
   <si>
+    <t>Fed - IRPJ/CSLL</t>
+  </si>
+  <si>
+    <t>Rebto planilha/Resumo de Folha (28)</t>
+  </si>
+  <si>
+    <t>Movimento - Analise de Balanço Lucro Real</t>
+  </si>
+  <si>
+    <t>Movimento - Analise de Balanço Simples Nacional</t>
+  </si>
+  <si>
+    <t>Movimento - Analise de Balanço Lucro Presumido</t>
+  </si>
+  <si>
+    <t>Confirm Rec - IRPJ/CSLL (CTB)</t>
+  </si>
+  <si>
+    <t>Definição do Lucro Trimestral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envio do Razão Conta - Valores à Classificar </t>
+  </si>
+  <si>
+    <t>Fechamento Mensal</t>
+  </si>
+  <si>
     <t>Fed - DCTFWEB</t>
   </si>
   <si>
-    <t>Fed - IRPJ/CSLL</t>
-  </si>
-  <si>
     <t>Módulo de Inclusão Tributária (MIT)</t>
-  </si>
-  <si>
-    <t>Rebto planilha/Resumo de Folha (28)</t>
-  </si>
-  <si>
-    <t>Movimento - Analise de Balanço Lucro Real</t>
-  </si>
-  <si>
-    <t>Movimento - Analise de Balanço Simples Nacional</t>
-  </si>
-  <si>
-    <t>Movimento - Analise de Balanço Lucro Presumido</t>
-  </si>
-  <si>
-    <t>Confirm Rec - IRPJ/CSLL (CTB)</t>
-  </si>
-  <si>
-    <t>Definição do Lucro Trimestral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envio do Razão Conta - Valores à Classificar </t>
-  </si>
-  <si>
-    <t>Fechamento Mensal</t>
   </si>
   <si>
     <t>Outras Receitas</t>
@@ -1142,45 +1142,45 @@
 A reunião está confirmada com o cliente para hoje - Data Comentário: 09/10/2026 10:00</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsto para conclusão dia 30/10/2026 - Data Comentário: 29/10/2026 18:12</t>
+  </si>
+  <si>
+    <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 30/10/2026 - Data Comentário: 29/10/2026 17:46</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/10/2026 
+Aguardando envio do cliente. - Data Comentário: 29/10/2026 16:53</t>
+  </si>
+  <si>
+    <t>Reaberto via API integração MGC x Analise Balanço em 16/10/2026 13:52:48. - Data Comentário: 29/10/2026 18:15</t>
+  </si>
+  <si>
+    <t>Reaberto via API integração MGC x Analise Balanço em 27/10/2026 16:34:07. - Data Comentário: 29/10/2026 18:15</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/10/2026 
+em liberação - Data Comentário: 26/10/2026 14:11</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/10/2026 
+EM PROCESSAMENTO! - Data Comentário: 28/10/2026 17:49</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/10/2026 
+EM PROCESSAMENTO! - Data Comentário: 28/10/2026 17:50</t>
+  </si>
+  <si>
+    <t>Término de Experiência no prazo em 24/10/2026 - Pgto 03/11/2026 - Data Comentário: 11/09/2026 09:53</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1582] sendo a ultima baixa feita [1582]-29/10/2026 16:16:25.. - Data Comentário: 29/10/2026 16:11</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1582] sendo a ultima baixa feita [1582]-28/10/2026 20:37:32.. - Data Comentário: 28/10/2026 20:32</t>
+  </si>
+  <si>
     <t>Sem informações para a realização da tarefa  Previsão para conclusão dia 30/10/2026 
 Aguardando liberação do IRPJ/CSLL - Data Comentário: 29/10/2026 18:14</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsto para conclusão dia 30/10/2026 - Data Comentário: 29/10/2026 18:12</t>
-  </si>
-  <si>
-    <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 30/10/2026 - Data Comentário: 29/10/2026 17:46</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/10/2026 
-Aguardando envio do cliente. - Data Comentário: 29/10/2026 16:53</t>
-  </si>
-  <si>
-    <t>Reaberto via API integração MGC x Analise Balanço em 16/10/2026 13:52:48. - Data Comentário: 29/10/2026 18:15</t>
-  </si>
-  <si>
-    <t>Reaberto via API integração MGC x Analise Balanço em 27/10/2026 16:34:07. - Data Comentário: 29/10/2026 18:15</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/10/2026 
-em liberação - Data Comentário: 26/10/2026 14:11</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/10/2026 
-EM PROCESSAMENTO! - Data Comentário: 28/10/2026 17:49</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/10/2026 
-EM PROCESSAMENTO! - Data Comentário: 28/10/2026 17:50</t>
-  </si>
-  <si>
-    <t>Término de Experiência no prazo em 24/10/2026 - Pgto 03/11/2026 - Data Comentário: 11/09/2026 09:53</t>
-  </si>
-  <si>
-    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1582] sendo a ultima baixa feita [1582]-29/10/2026 16:16:25.. - Data Comentário: 29/10/2026 16:11</t>
-  </si>
-  <si>
-    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1582] sendo a ultima baixa feita [1582]-28/10/2026 20:37:32.. - Data Comentário: 28/10/2026 20:32</t>
   </si>
   <si>
     <t>Sem informações para a realização da tarefa  Previsão para conclusão dia 29/10/2026 
@@ -23054,10 +23054,10 @@
     </row>
     <row r="286" spans="1:34">
       <c r="A286">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B286" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C286" t="s">
         <v>55</v>
@@ -23072,7 +23072,7 @@
         <v>61</v>
       </c>
       <c r="G286">
-        <v>6892</v>
+        <v>1651</v>
       </c>
       <c r="H286">
         <v>0</v>
@@ -23084,7 +23084,7 @@
         <v>129</v>
       </c>
       <c r="L286" s="1">
-        <v>46321</v>
+        <v>46324</v>
       </c>
       <c r="M286" t="s">
         <v>186</v>
@@ -23093,19 +23093,19 @@
         <v>213</v>
       </c>
       <c r="O286">
-        <v>17968018</v>
+        <v>17042386</v>
       </c>
       <c r="P286" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q286" t="s">
         <v>247</v>
       </c>
       <c r="S286">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T286" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="U286" t="s">
         <v>264</v>
@@ -23120,18 +23120,18 @@
         <v>0</v>
       </c>
       <c r="AG286" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AH286" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
     </row>
     <row r="287" spans="1:34">
       <c r="A287">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B287" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C287" t="s">
         <v>55</v>
@@ -23146,69 +23146,69 @@
         <v>61</v>
       </c>
       <c r="G287">
-        <v>6892</v>
+        <v>5847</v>
       </c>
       <c r="H287">
-        <v>0</v>
+        <v>5784</v>
       </c>
       <c r="I287" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J287" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L287" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="M287" t="s">
         <v>186</v>
       </c>
       <c r="N287" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="O287">
-        <v>18178289</v>
+        <v>18158418</v>
       </c>
       <c r="P287" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="Q287" t="s">
         <v>247</v>
       </c>
       <c r="S287">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T287" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="U287" t="s">
         <v>265</v>
       </c>
       <c r="W287" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AA287">
         <v>0</v>
       </c>
       <c r="AG287" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="AH287" t="s">
-        <v>524</v>
+        <v>536</v>
       </c>
     </row>
     <row r="288" spans="1:34">
       <c r="A288">
-        <v>6627</v>
+        <v>6779</v>
       </c>
       <c r="B288" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C288" t="s">
         <v>55</v>
       </c>
       <c r="D288" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E288" t="s">
         <v>59</v>
@@ -23217,66 +23217,66 @@
         <v>61</v>
       </c>
       <c r="G288">
-        <v>1651</v>
+        <v>5847</v>
       </c>
       <c r="H288">
-        <v>0</v>
+        <v>5784</v>
       </c>
       <c r="I288" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J288" t="s">
         <v>130</v>
       </c>
       <c r="L288" s="1">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="M288" t="s">
         <v>186</v>
       </c>
       <c r="N288" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="O288">
-        <v>17042386</v>
+        <v>18158765</v>
       </c>
       <c r="P288" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="Q288" t="s">
         <v>247</v>
       </c>
       <c r="S288">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T288" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="U288" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="V288" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="W288" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AA288">
         <v>0</v>
       </c>
       <c r="AG288" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="AH288" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="289" spans="1:34">
       <c r="A289">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B289" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C289" t="s">
         <v>55</v>
@@ -23291,19 +23291,19 @@
         <v>61</v>
       </c>
       <c r="G289">
-        <v>1651</v>
+        <v>7877</v>
       </c>
       <c r="H289">
         <v>0</v>
       </c>
       <c r="I289" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J289" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L289" s="1">
-        <v>46324</v>
+        <v>46321</v>
       </c>
       <c r="M289" t="s">
         <v>186</v>
@@ -23312,42 +23312,39 @@
         <v>213</v>
       </c>
       <c r="O289">
-        <v>18178273</v>
+        <v>17399331</v>
       </c>
       <c r="P289" t="s">
-        <v>219</v>
+        <v>59</v>
       </c>
       <c r="Q289" t="s">
         <v>247</v>
       </c>
       <c r="S289">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T289" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="U289" t="s">
         <v>265</v>
       </c>
       <c r="W289" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="AA289">
         <v>0</v>
       </c>
       <c r="AG289" t="s">
-        <v>532</v>
-      </c>
-      <c r="AH289" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
     </row>
     <row r="290" spans="1:34">
       <c r="A290">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B290" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C290" t="s">
         <v>55</v>
@@ -23362,16 +23359,16 @@
         <v>61</v>
       </c>
       <c r="G290">
-        <v>11516</v>
+        <v>9774</v>
       </c>
       <c r="H290">
         <v>0</v>
       </c>
       <c r="I290" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J290" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L290" s="1">
         <v>46321</v>
@@ -23383,10 +23380,10 @@
         <v>213</v>
       </c>
       <c r="O290">
-        <v>17968054</v>
+        <v>16976322</v>
       </c>
       <c r="P290" t="s">
-        <v>219</v>
+        <v>59</v>
       </c>
       <c r="Q290" t="s">
         <v>247</v>
@@ -23395,39 +23392,33 @@
         <v>4</v>
       </c>
       <c r="T290" t="s">
-        <v>251</v>
-      </c>
-      <c r="U290" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="V290" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="W290" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="AA290">
         <v>0</v>
       </c>
       <c r="AG290" t="s">
-        <v>533</v>
-      </c>
-      <c r="AH290" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
     </row>
     <row r="291" spans="1:34">
       <c r="A291">
-        <v>6949</v>
+        <v>6404</v>
       </c>
       <c r="B291" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C291" t="s">
         <v>55</v>
       </c>
       <c r="D291" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E291" t="s">
         <v>59</v>
@@ -23436,63 +23427,57 @@
         <v>61</v>
       </c>
       <c r="G291">
-        <v>11516</v>
+        <v>10988</v>
       </c>
       <c r="H291">
         <v>0</v>
       </c>
       <c r="I291" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J291" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="L291" s="1">
-        <v>46321</v>
-      </c>
-      <c r="M291" t="s">
-        <v>186</v>
+        <v>46325</v>
       </c>
       <c r="N291" t="s">
         <v>213</v>
       </c>
       <c r="O291">
-        <v>18178315</v>
+        <v>16962445</v>
       </c>
       <c r="P291" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="Q291" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="S291">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T291" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="U291" t="s">
-        <v>265</v>
-      </c>
-      <c r="W291" t="s">
-        <v>367</v>
+        <v>264</v>
       </c>
       <c r="AA291">
         <v>0</v>
       </c>
       <c r="AG291" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="AH291" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="292" spans="1:34">
       <c r="A292">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B292" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C292" t="s">
         <v>55</v>
@@ -23507,46 +23492,43 @@
         <v>61</v>
       </c>
       <c r="G292">
-        <v>5847</v>
+        <v>7874</v>
       </c>
       <c r="H292">
-        <v>5784</v>
+        <v>0</v>
       </c>
       <c r="I292" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J292" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L292" s="1">
-        <v>46323</v>
-      </c>
-      <c r="M292" t="s">
-        <v>186</v>
+        <v>46325</v>
       </c>
       <c r="N292" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O292">
-        <v>18158418</v>
+        <v>18096768</v>
       </c>
       <c r="P292" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="Q292" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="S292">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T292" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="U292" t="s">
         <v>265</v>
       </c>
-      <c r="W292" t="s">
-        <v>369</v>
+      <c r="V292" t="s">
+        <v>268</v>
       </c>
       <c r="AA292">
         <v>0</v>
@@ -23555,21 +23537,21 @@
         <v>531</v>
       </c>
       <c r="AH292" t="s">
-        <v>536</v>
+        <v>525</v>
       </c>
     </row>
     <row r="293" spans="1:34">
       <c r="A293">
-        <v>6779</v>
+        <v>5417</v>
       </c>
       <c r="B293" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C293" t="s">
         <v>55</v>
       </c>
       <c r="D293" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E293" t="s">
         <v>59</v>
@@ -23578,55 +23560,52 @@
         <v>61</v>
       </c>
       <c r="G293">
-        <v>5847</v>
+        <v>11542</v>
       </c>
       <c r="H293">
-        <v>5784</v>
+        <v>0</v>
       </c>
       <c r="I293" t="s">
         <v>62</v>
       </c>
       <c r="J293" t="s">
-        <v>132</v>
+        <v>75</v>
       </c>
       <c r="L293" s="1">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="M293" t="s">
         <v>186</v>
       </c>
       <c r="N293" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="O293">
-        <v>18158765</v>
+        <v>18248557</v>
       </c>
       <c r="P293" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="Q293" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="S293">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T293" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="U293" t="s">
         <v>265</v>
       </c>
-      <c r="V293" t="s">
-        <v>268</v>
-      </c>
       <c r="W293" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="AA293">
         <v>0</v>
       </c>
       <c r="AG293" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="AH293" t="s">
         <v>536</v>
@@ -23634,10 +23613,10 @@
     </row>
     <row r="294" spans="1:34">
       <c r="A294">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B294" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C294" t="s">
         <v>55</v>
@@ -23652,60 +23631,63 @@
         <v>61</v>
       </c>
       <c r="G294">
-        <v>7877</v>
+        <v>11542</v>
       </c>
       <c r="H294">
         <v>0</v>
       </c>
       <c r="I294" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="J294" t="s">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="L294" s="1">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="M294" t="s">
         <v>186</v>
       </c>
       <c r="N294" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="O294">
-        <v>17399331</v>
+        <v>18190473</v>
       </c>
       <c r="P294" t="s">
-        <v>59</v>
+        <v>226</v>
       </c>
       <c r="Q294" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="S294">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T294" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="U294" t="s">
         <v>265</v>
       </c>
       <c r="W294" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="AA294">
         <v>0</v>
       </c>
       <c r="AG294" t="s">
-        <v>531</v>
+        <v>533</v>
+      </c>
+      <c r="AH294" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="295" spans="1:34">
       <c r="A295">
-        <v>6486</v>
+        <v>6949</v>
       </c>
       <c r="B295" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C295" t="s">
         <v>55</v>
@@ -23720,66 +23702,69 @@
         <v>61</v>
       </c>
       <c r="G295">
-        <v>9774</v>
+        <v>11541</v>
       </c>
       <c r="H295">
         <v>0</v>
       </c>
       <c r="I295" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="J295" t="s">
-        <v>134</v>
+        <v>80</v>
       </c>
       <c r="L295" s="1">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="M295" t="s">
         <v>186</v>
       </c>
       <c r="N295" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="O295">
-        <v>16976322</v>
+        <v>18190467</v>
       </c>
       <c r="P295" t="s">
-        <v>59</v>
+        <v>226</v>
       </c>
       <c r="Q295" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="S295">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T295" t="s">
-        <v>257</v>
-      </c>
-      <c r="V295" t="s">
-        <v>269</v>
+        <v>253</v>
+      </c>
+      <c r="U295" t="s">
+        <v>265</v>
       </c>
       <c r="W295" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="AA295">
         <v>0</v>
       </c>
       <c r="AG295" t="s">
-        <v>531</v>
+        <v>533</v>
+      </c>
+      <c r="AH295" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="296" spans="1:34">
       <c r="A296">
-        <v>6404</v>
+        <v>6949</v>
       </c>
       <c r="B296" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C296" t="s">
         <v>55</v>
       </c>
       <c r="D296" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E296" t="s">
         <v>59</v>
@@ -23788,28 +23773,31 @@
         <v>61</v>
       </c>
       <c r="G296">
-        <v>10988</v>
+        <v>6348</v>
       </c>
       <c r="H296">
         <v>0</v>
       </c>
       <c r="I296" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J296" t="s">
-        <v>135</v>
+        <v>89</v>
       </c>
       <c r="L296" s="1">
         <v>46325</v>
       </c>
+      <c r="M296" t="s">
+        <v>186</v>
+      </c>
       <c r="N296" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="O296">
-        <v>16962445</v>
+        <v>18272235</v>
       </c>
       <c r="P296" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="Q296" t="s">
         <v>249</v>
@@ -23818,27 +23806,30 @@
         <v>0</v>
       </c>
       <c r="T296" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="U296" t="s">
-        <v>264</v>
+        <v>265</v>
+      </c>
+      <c r="W296" t="s">
+        <v>375</v>
       </c>
       <c r="AA296">
         <v>0</v>
       </c>
       <c r="AG296" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="AH296" t="s">
-        <v>525</v>
+        <v>538</v>
       </c>
     </row>
     <row r="297" spans="1:34">
       <c r="A297">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B297" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C297" t="s">
         <v>55</v>
@@ -23853,28 +23844,31 @@
         <v>61</v>
       </c>
       <c r="G297">
-        <v>7874</v>
+        <v>949</v>
       </c>
       <c r="H297">
         <v>0</v>
       </c>
       <c r="I297" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J297" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L297" s="1">
         <v>46325</v>
       </c>
+      <c r="M297" t="s">
+        <v>186</v>
+      </c>
       <c r="N297" t="s">
         <v>213</v>
       </c>
       <c r="O297">
-        <v>18096768</v>
+        <v>17398876</v>
       </c>
       <c r="P297" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="Q297" t="s">
         <v>249</v>
@@ -23883,30 +23877,27 @@
         <v>0</v>
       </c>
       <c r="T297" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="U297" t="s">
         <v>265</v>
       </c>
-      <c r="V297" t="s">
-        <v>268</v>
+      <c r="W297" t="s">
+        <v>376</v>
       </c>
       <c r="AA297">
         <v>0</v>
       </c>
       <c r="AG297" t="s">
-        <v>531</v>
-      </c>
-      <c r="AH297" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
     </row>
     <row r="298" spans="1:34">
       <c r="A298">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B298" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C298" t="s">
         <v>55</v>
@@ -23921,16 +23912,16 @@
         <v>61</v>
       </c>
       <c r="G298">
-        <v>11542</v>
+        <v>949</v>
       </c>
       <c r="H298">
         <v>0</v>
       </c>
       <c r="I298" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="J298" t="s">
-        <v>75</v>
+        <v>134</v>
       </c>
       <c r="L298" s="1">
         <v>46325</v>
@@ -23939,13 +23930,13 @@
         <v>186</v>
       </c>
       <c r="N298" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="O298">
-        <v>18248557</v>
+        <v>17952332</v>
       </c>
       <c r="P298" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="Q298" t="s">
         <v>249</v>
@@ -23954,30 +23945,30 @@
         <v>0</v>
       </c>
       <c r="T298" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="U298" t="s">
         <v>265</v>
       </c>
+      <c r="V298" t="s">
+        <v>268</v>
+      </c>
       <c r="W298" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="AA298">
         <v>0</v>
       </c>
       <c r="AG298" t="s">
-        <v>533</v>
-      </c>
-      <c r="AH298" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
     </row>
     <row r="299" spans="1:34">
       <c r="A299">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B299" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C299" t="s">
         <v>55</v>
@@ -23992,31 +23983,28 @@
         <v>61</v>
       </c>
       <c r="G299">
-        <v>11542</v>
+        <v>957</v>
       </c>
       <c r="H299">
         <v>0</v>
       </c>
       <c r="I299" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="J299" t="s">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="L299" s="1">
         <v>46325</v>
       </c>
-      <c r="M299" t="s">
-        <v>186</v>
-      </c>
       <c r="N299" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="O299">
-        <v>18190473</v>
+        <v>17398900</v>
       </c>
       <c r="P299" t="s">
-        <v>226</v>
+        <v>59</v>
       </c>
       <c r="Q299" t="s">
         <v>249</v>
@@ -24025,30 +24013,24 @@
         <v>0</v>
       </c>
       <c r="T299" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="U299" t="s">
         <v>265</v>
       </c>
-      <c r="W299" t="s">
-        <v>374</v>
-      </c>
       <c r="AA299">
         <v>0</v>
       </c>
       <c r="AG299" t="s">
-        <v>533</v>
-      </c>
-      <c r="AH299" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="300" spans="1:34">
       <c r="A300">
-        <v>6949</v>
+        <v>6627</v>
       </c>
       <c r="B300" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C300" t="s">
         <v>55</v>
@@ -24063,31 +24045,28 @@
         <v>61</v>
       </c>
       <c r="G300">
-        <v>11541</v>
+        <v>957</v>
       </c>
       <c r="H300">
         <v>0</v>
       </c>
       <c r="I300" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="J300" t="s">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="L300" s="1">
         <v>46325</v>
       </c>
-      <c r="M300" t="s">
-        <v>186</v>
-      </c>
       <c r="N300" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="O300">
-        <v>18190467</v>
+        <v>17042326</v>
       </c>
       <c r="P300" t="s">
-        <v>226</v>
+        <v>59</v>
       </c>
       <c r="Q300" t="s">
         <v>249</v>
@@ -24096,30 +24075,27 @@
         <v>0</v>
       </c>
       <c r="T300" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="U300" t="s">
-        <v>265</v>
-      </c>
-      <c r="W300" t="s">
-        <v>375</v>
+        <v>264</v>
+      </c>
+      <c r="V300" t="s">
+        <v>267</v>
       </c>
       <c r="AA300">
         <v>0</v>
       </c>
       <c r="AG300" t="s">
-        <v>533</v>
-      </c>
-      <c r="AH300" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="301" spans="1:34">
       <c r="A301">
-        <v>6949</v>
+        <v>6627</v>
       </c>
       <c r="B301" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C301" t="s">
         <v>55</v>
@@ -24134,69 +24110,72 @@
         <v>61</v>
       </c>
       <c r="G301">
-        <v>6348</v>
+        <v>7869</v>
       </c>
       <c r="H301">
         <v>0</v>
       </c>
       <c r="I301" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J301" t="s">
-        <v>89</v>
+        <v>136</v>
       </c>
       <c r="L301" s="1">
-        <v>46325</v>
-      </c>
-      <c r="M301" t="s">
-        <v>186</v>
+        <v>46321</v>
       </c>
       <c r="N301" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O301">
-        <v>18272235</v>
+        <v>17042548</v>
       </c>
       <c r="P301" t="s">
-        <v>241</v>
+        <v>220</v>
       </c>
       <c r="Q301" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+      <c r="R301" s="1">
+        <v>46317.63681168982</v>
       </c>
       <c r="S301">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T301" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="U301" t="s">
-        <v>265</v>
-      </c>
-      <c r="W301" t="s">
-        <v>376</v>
+        <v>264</v>
+      </c>
+      <c r="V301" t="s">
+        <v>267</v>
       </c>
       <c r="AA301">
         <v>0</v>
       </c>
+      <c r="AB301" t="s">
+        <v>524</v>
+      </c>
       <c r="AG301" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="AH301" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="302" spans="1:34">
       <c r="A302">
-        <v>5417</v>
+        <v>6628</v>
       </c>
       <c r="B302" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C302" t="s">
         <v>55</v>
       </c>
       <c r="D302" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E302" t="s">
         <v>59</v>
@@ -24205,60 +24184,66 @@
         <v>61</v>
       </c>
       <c r="G302">
-        <v>949</v>
+        <v>7869</v>
       </c>
       <c r="H302">
         <v>0</v>
       </c>
       <c r="I302" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J302" t="s">
         <v>136</v>
       </c>
       <c r="L302" s="1">
-        <v>46325</v>
-      </c>
-      <c r="M302" t="s">
-        <v>186</v>
+        <v>46321</v>
       </c>
       <c r="N302" t="s">
         <v>213</v>
       </c>
       <c r="O302">
-        <v>17398876</v>
+        <v>16960049</v>
       </c>
       <c r="P302" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="Q302" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+      <c r="R302" s="1">
+        <v>46317.63681204861</v>
       </c>
       <c r="S302">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T302" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="U302" t="s">
-        <v>265</v>
-      </c>
-      <c r="W302" t="s">
-        <v>377</v>
+        <v>264</v>
+      </c>
+      <c r="V302" t="s">
+        <v>267</v>
       </c>
       <c r="AA302">
         <v>0</v>
       </c>
+      <c r="AB302" t="s">
+        <v>524</v>
+      </c>
       <c r="AG302" t="s">
-        <v>532</v>
+        <v>531</v>
+      </c>
+      <c r="AH302" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="303" spans="1:34">
       <c r="A303">
-        <v>6704</v>
+        <v>6949</v>
       </c>
       <c r="B303" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C303" t="s">
         <v>55</v>
@@ -24273,69 +24258,69 @@
         <v>61</v>
       </c>
       <c r="G303">
-        <v>949</v>
+        <v>7869</v>
       </c>
       <c r="H303">
         <v>0</v>
       </c>
       <c r="I303" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J303" t="s">
         <v>136</v>
       </c>
       <c r="L303" s="1">
-        <v>46325</v>
-      </c>
-      <c r="M303" t="s">
-        <v>186</v>
+        <v>46321</v>
       </c>
       <c r="N303" t="s">
         <v>213</v>
       </c>
       <c r="O303">
-        <v>17952332</v>
+        <v>18178301</v>
       </c>
       <c r="P303" t="s">
-        <v>238</v>
+        <v>219</v>
       </c>
       <c r="Q303" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+      <c r="R303" s="1">
+        <v>46317.63682094908</v>
       </c>
       <c r="S303">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T303" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="U303" t="s">
         <v>265</v>
       </c>
-      <c r="V303" t="s">
-        <v>268</v>
-      </c>
-      <c r="W303" t="s">
-        <v>378</v>
-      </c>
       <c r="AA303">
         <v>0</v>
       </c>
+      <c r="AB303" t="s">
+        <v>524</v>
+      </c>
       <c r="AG303" t="s">
-        <v>532</v>
+        <v>531</v>
+      </c>
+      <c r="AH303" t="s">
+        <v>524</v>
       </c>
     </row>
     <row r="304" spans="1:34">
       <c r="A304">
-        <v>5417</v>
+        <v>6628</v>
       </c>
       <c r="B304" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C304" t="s">
         <v>55</v>
       </c>
       <c r="D304" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E304" t="s">
         <v>59</v>
@@ -24344,54 +24329,66 @@
         <v>61</v>
       </c>
       <c r="G304">
-        <v>957</v>
+        <v>1650</v>
       </c>
       <c r="H304">
         <v>0</v>
       </c>
       <c r="I304" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J304" t="s">
         <v>137</v>
       </c>
       <c r="L304" s="1">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="N304" t="s">
         <v>213</v>
       </c>
       <c r="O304">
-        <v>17398900</v>
+        <v>16959975</v>
       </c>
       <c r="P304" t="s">
-        <v>59</v>
+        <v>220</v>
       </c>
       <c r="Q304" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+      <c r="R304" s="1">
+        <v>46295.04093612268</v>
       </c>
       <c r="S304">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T304" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="U304" t="s">
-        <v>265</v>
+        <v>264</v>
+      </c>
+      <c r="V304" t="s">
+        <v>267</v>
       </c>
       <c r="AA304">
         <v>0</v>
+      </c>
+      <c r="AB304" t="s">
+        <v>521</v>
       </c>
       <c r="AG304" t="s">
         <v>531</v>
       </c>
+      <c r="AH304" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="305" spans="1:34">
       <c r="A305">
-        <v>6627</v>
+        <v>6945</v>
       </c>
       <c r="B305" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C305" t="s">
         <v>55</v>
@@ -24403,60 +24400,66 @@
         <v>59</v>
       </c>
       <c r="F305" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G305">
-        <v>957</v>
+        <v>1650</v>
       </c>
       <c r="H305">
         <v>0</v>
       </c>
       <c r="I305" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J305" t="s">
         <v>137</v>
       </c>
       <c r="L305" s="1">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="N305" t="s">
         <v>213</v>
       </c>
       <c r="O305">
-        <v>17042326</v>
+        <v>18163668</v>
       </c>
       <c r="P305" t="s">
-        <v>59</v>
+        <v>221</v>
       </c>
       <c r="Q305" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+      <c r="R305" s="1">
+        <v>46295.04098302083</v>
       </c>
       <c r="S305">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T305" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="U305" t="s">
         <v>264</v>
       </c>
-      <c r="V305" t="s">
-        <v>267</v>
-      </c>
       <c r="AA305">
         <v>0</v>
+      </c>
+      <c r="AB305" t="s">
+        <v>521</v>
       </c>
       <c r="AG305" t="s">
         <v>531</v>
       </c>
+      <c r="AH305" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="306" spans="1:34">
       <c r="A306">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B306" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C306" t="s">
         <v>55</v>
@@ -24471,7 +24474,7 @@
         <v>61</v>
       </c>
       <c r="G306">
-        <v>7869</v>
+        <v>6892</v>
       </c>
       <c r="H306">
         <v>0</v>
@@ -24485,26 +24488,29 @@
       <c r="L306" s="1">
         <v>46321</v>
       </c>
+      <c r="M306" t="s">
+        <v>186</v>
+      </c>
       <c r="N306" t="s">
         <v>213</v>
       </c>
       <c r="O306">
-        <v>17042548</v>
+        <v>17968018</v>
       </c>
       <c r="P306" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Q306" t="s">
         <v>248</v>
       </c>
       <c r="R306" s="1">
-        <v>46317.63681168982</v>
+        <v>46325.45772567129</v>
       </c>
       <c r="S306">
         <v>4</v>
       </c>
       <c r="T306" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="U306" t="s">
         <v>264</v>
@@ -24512,31 +24518,34 @@
       <c r="V306" t="s">
         <v>267</v>
       </c>
+      <c r="W306" t="s">
+        <v>378</v>
+      </c>
       <c r="AA306">
         <v>0</v>
       </c>
       <c r="AB306" t="s">
+        <v>219</v>
+      </c>
+      <c r="AG306" t="s">
+        <v>533</v>
+      </c>
+      <c r="AH306" t="s">
         <v>524</v>
-      </c>
-      <c r="AG306" t="s">
-        <v>531</v>
-      </c>
-      <c r="AH306" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="307" spans="1:34">
       <c r="A307">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B307" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C307" t="s">
         <v>55</v>
       </c>
       <c r="D307" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E307" t="s">
         <v>59</v>
@@ -24545,7 +24554,7 @@
         <v>61</v>
       </c>
       <c r="G307">
-        <v>7869</v>
+        <v>6892</v>
       </c>
       <c r="H307">
         <v>0</v>
@@ -24559,11 +24568,14 @@
       <c r="L307" s="1">
         <v>46321</v>
       </c>
+      <c r="M307" t="s">
+        <v>203</v>
+      </c>
       <c r="N307" t="s">
         <v>213</v>
       </c>
       <c r="O307">
-        <v>16960049</v>
+        <v>17042488</v>
       </c>
       <c r="P307" t="s">
         <v>220</v>
@@ -24572,7 +24584,7 @@
         <v>248</v>
       </c>
       <c r="R307" s="1">
-        <v>46317.63681204861</v>
+        <v>46324.49322108796</v>
       </c>
       <c r="S307">
         <v>4</v>
@@ -24586,14 +24598,17 @@
       <c r="V307" t="s">
         <v>267</v>
       </c>
+      <c r="W307" t="s">
+        <v>379</v>
+      </c>
       <c r="AA307">
         <v>0</v>
       </c>
       <c r="AB307" t="s">
-        <v>524</v>
+        <v>220</v>
       </c>
       <c r="AG307" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="AH307" t="s">
         <v>535</v>
@@ -24601,16 +24616,16 @@
     </row>
     <row r="308" spans="1:34">
       <c r="A308">
-        <v>6949</v>
+        <v>6628</v>
       </c>
       <c r="B308" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C308" t="s">
         <v>55</v>
       </c>
       <c r="D308" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E308" t="s">
         <v>59</v>
@@ -24619,7 +24634,7 @@
         <v>61</v>
       </c>
       <c r="G308">
-        <v>7869</v>
+        <v>6892</v>
       </c>
       <c r="H308">
         <v>0</v>
@@ -24637,25 +24652,28 @@
         <v>213</v>
       </c>
       <c r="O308">
-        <v>18178301</v>
+        <v>16960025</v>
       </c>
       <c r="P308" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q308" t="s">
         <v>248</v>
       </c>
       <c r="R308" s="1">
-        <v>46317.63682094908</v>
+        <v>46318.63617619213</v>
       </c>
       <c r="S308">
         <v>4</v>
       </c>
       <c r="T308" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="U308" t="s">
-        <v>265</v>
+        <v>264</v>
+      </c>
+      <c r="V308" t="s">
+        <v>267</v>
       </c>
       <c r="AA308">
         <v>0</v>
@@ -24664,33 +24682,33 @@
         <v>524</v>
       </c>
       <c r="AG308" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="AH308" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
     </row>
     <row r="309" spans="1:34">
       <c r="A309">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B309" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C309" t="s">
         <v>55</v>
       </c>
       <c r="D309" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E309" t="s">
         <v>59</v>
       </c>
       <c r="F309" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G309">
-        <v>1650</v>
+        <v>6892</v>
       </c>
       <c r="H309">
         <v>0</v>
@@ -24699,46 +24717,49 @@
         <v>63</v>
       </c>
       <c r="J309" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L309" s="1">
-        <v>46323</v>
+        <v>46321</v>
+      </c>
+      <c r="M309" t="s">
+        <v>186</v>
       </c>
       <c r="N309" t="s">
         <v>213</v>
       </c>
       <c r="O309">
-        <v>16959975</v>
+        <v>18163677</v>
       </c>
       <c r="P309" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Q309" t="s">
         <v>248</v>
       </c>
       <c r="R309" s="1">
-        <v>46295.04093612268</v>
+        <v>46324.81241204861</v>
       </c>
       <c r="S309">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T309" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="U309" t="s">
         <v>264</v>
       </c>
-      <c r="V309" t="s">
-        <v>267</v>
+      <c r="W309" t="s">
+        <v>378</v>
       </c>
       <c r="AA309">
         <v>0</v>
       </c>
       <c r="AB309" t="s">
-        <v>521</v>
+        <v>221</v>
       </c>
       <c r="AG309" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="AH309" t="s">
         <v>535</v>
@@ -24746,10 +24767,10 @@
     </row>
     <row r="310" spans="1:34">
       <c r="A310">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B310" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C310" t="s">
         <v>55</v>
@@ -24761,10 +24782,10 @@
         <v>59</v>
       </c>
       <c r="F310" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G310">
-        <v>1650</v>
+        <v>6892</v>
       </c>
       <c r="H310">
         <v>0</v>
@@ -24773,60 +24794,66 @@
         <v>63</v>
       </c>
       <c r="J310" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L310" s="1">
-        <v>46323</v>
+        <v>46321</v>
+      </c>
+      <c r="M310" t="s">
+        <v>186</v>
       </c>
       <c r="N310" t="s">
         <v>213</v>
       </c>
       <c r="O310">
-        <v>18163668</v>
+        <v>18178289</v>
       </c>
       <c r="P310" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="Q310" t="s">
         <v>248</v>
       </c>
       <c r="R310" s="1">
-        <v>46295.04098302083</v>
+        <v>46325.45772603009</v>
       </c>
       <c r="S310">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T310" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="U310" t="s">
-        <v>264</v>
+        <v>265</v>
+      </c>
+      <c r="W310" t="s">
+        <v>378</v>
       </c>
       <c r="AA310">
         <v>0</v>
       </c>
       <c r="AB310" t="s">
-        <v>521</v>
+        <v>219</v>
       </c>
       <c r="AG310" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="AH310" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="311" spans="1:34">
       <c r="A311">
-        <v>6627</v>
+        <v>6962</v>
       </c>
       <c r="B311" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C311" t="s">
         <v>55</v>
       </c>
       <c r="D311" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E311" t="s">
         <v>59</v>
@@ -24844,7 +24871,7 @@
         <v>63</v>
       </c>
       <c r="J311" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L311" s="1">
         <v>46321</v>
@@ -24856,28 +24883,25 @@
         <v>213</v>
       </c>
       <c r="O311">
-        <v>17042488</v>
+        <v>18187956</v>
       </c>
       <c r="P311" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q311" t="s">
         <v>248</v>
       </c>
       <c r="R311" s="1">
-        <v>46324.49322108796</v>
+        <v>46322.698238125</v>
       </c>
       <c r="S311">
         <v>4</v>
       </c>
       <c r="T311" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="U311" t="s">
-        <v>264</v>
-      </c>
-      <c r="V311" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="W311" t="s">
         <v>379</v>
@@ -24886,7 +24910,7 @@
         <v>0</v>
       </c>
       <c r="AB311" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="AG311" t="s">
         <v>533</v>
@@ -24897,16 +24921,16 @@
     </row>
     <row r="312" spans="1:34">
       <c r="A312">
-        <v>6628</v>
+        <v>6963</v>
       </c>
       <c r="B312" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C312" t="s">
         <v>55</v>
       </c>
       <c r="D312" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E312" t="s">
         <v>59</v>
@@ -24924,43 +24948,46 @@
         <v>63</v>
       </c>
       <c r="J312" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L312" s="1">
         <v>46321</v>
       </c>
+      <c r="M312" t="s">
+        <v>203</v>
+      </c>
       <c r="N312" t="s">
         <v>213</v>
       </c>
       <c r="O312">
-        <v>16960025</v>
+        <v>18187894</v>
       </c>
       <c r="P312" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q312" t="s">
         <v>248</v>
       </c>
       <c r="R312" s="1">
-        <v>46318.63617619213</v>
+        <v>46323.49171587963</v>
       </c>
       <c r="S312">
         <v>4</v>
       </c>
       <c r="T312" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="U312" t="s">
-        <v>264</v>
-      </c>
-      <c r="V312" t="s">
-        <v>267</v>
+        <v>266</v>
+      </c>
+      <c r="W312" t="s">
+        <v>379</v>
       </c>
       <c r="AA312">
         <v>0</v>
       </c>
       <c r="AB312" t="s">
-        <v>524</v>
+        <v>222</v>
       </c>
       <c r="AG312" t="s">
         <v>533</v>
@@ -24971,10 +24998,10 @@
     </row>
     <row r="313" spans="1:34">
       <c r="A313">
-        <v>6945</v>
+        <v>6548</v>
       </c>
       <c r="B313" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C313" t="s">
         <v>55</v>
@@ -24986,10 +25013,10 @@
         <v>59</v>
       </c>
       <c r="F313" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G313">
-        <v>6892</v>
+        <v>1651</v>
       </c>
       <c r="H313">
         <v>0</v>
@@ -25001,63 +25028,60 @@
         <v>129</v>
       </c>
       <c r="L313" s="1">
-        <v>46321</v>
-      </c>
-      <c r="M313" t="s">
-        <v>186</v>
+        <v>46324</v>
       </c>
       <c r="N313" t="s">
         <v>213</v>
       </c>
       <c r="O313">
-        <v>18163677</v>
+        <v>17967986</v>
       </c>
       <c r="P313" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="Q313" t="s">
         <v>248</v>
       </c>
       <c r="R313" s="1">
-        <v>46324.81241204861</v>
+        <v>46324.63946440972</v>
       </c>
       <c r="S313">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T313" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="U313" t="s">
         <v>264</v>
       </c>
-      <c r="W313" t="s">
-        <v>367</v>
+      <c r="V313" t="s">
+        <v>267</v>
       </c>
       <c r="AA313">
         <v>0</v>
       </c>
       <c r="AB313" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="AG313" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AH313" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="314" spans="1:34">
       <c r="A314">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B314" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C314" t="s">
         <v>55</v>
       </c>
       <c r="D314" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E314" t="s">
         <v>59</v>
@@ -25066,7 +25090,7 @@
         <v>61</v>
       </c>
       <c r="G314">
-        <v>6892</v>
+        <v>1651</v>
       </c>
       <c r="H314">
         <v>0</v>
@@ -25078,63 +25102,63 @@
         <v>129</v>
       </c>
       <c r="L314" s="1">
-        <v>46321</v>
+        <v>46324</v>
       </c>
       <c r="M314" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="N314" t="s">
         <v>213</v>
       </c>
       <c r="O314">
-        <v>18187956</v>
+        <v>18178273</v>
       </c>
       <c r="P314" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="Q314" t="s">
         <v>248</v>
       </c>
       <c r="R314" s="1">
-        <v>46322.698238125</v>
+        <v>46325.45814797454</v>
       </c>
       <c r="S314">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T314" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="U314" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="W314" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="AA314">
         <v>0</v>
       </c>
       <c r="AB314" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="AG314" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AH314" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="315" spans="1:34">
       <c r="A315">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B315" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C315" t="s">
         <v>55</v>
       </c>
       <c r="D315" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E315" t="s">
         <v>59</v>
@@ -25143,7 +25167,7 @@
         <v>61</v>
       </c>
       <c r="G315">
-        <v>6892</v>
+        <v>11516</v>
       </c>
       <c r="H315">
         <v>0</v>
@@ -25152,60 +25176,63 @@
         <v>63</v>
       </c>
       <c r="J315" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="L315" s="1">
         <v>46321</v>
       </c>
       <c r="M315" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="N315" t="s">
         <v>213</v>
       </c>
       <c r="O315">
-        <v>18187894</v>
+        <v>17968054</v>
       </c>
       <c r="P315" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="Q315" t="s">
         <v>248</v>
       </c>
       <c r="R315" s="1">
-        <v>46323.49171587963</v>
+        <v>46325.45940729167</v>
       </c>
       <c r="S315">
         <v>4</v>
       </c>
       <c r="T315" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="U315" t="s">
-        <v>266</v>
+        <v>264</v>
+      </c>
+      <c r="V315" t="s">
+        <v>267</v>
       </c>
       <c r="W315" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AA315">
         <v>0</v>
       </c>
       <c r="AB315" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="AG315" t="s">
         <v>533</v>
       </c>
       <c r="AH315" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="316" spans="1:34">
       <c r="A316">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B316" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C316" t="s">
         <v>55</v>
@@ -25220,7 +25247,7 @@
         <v>61</v>
       </c>
       <c r="G316">
-        <v>1651</v>
+        <v>11516</v>
       </c>
       <c r="H316">
         <v>0</v>
@@ -25229,31 +25256,34 @@
         <v>63</v>
       </c>
       <c r="J316" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="L316" s="1">
-        <v>46324</v>
+        <v>46321</v>
+      </c>
+      <c r="M316" t="s">
+        <v>186</v>
       </c>
       <c r="N316" t="s">
         <v>213</v>
       </c>
       <c r="O316">
-        <v>17967986</v>
+        <v>17042663</v>
       </c>
       <c r="P316" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q316" t="s">
         <v>248</v>
       </c>
       <c r="R316" s="1">
-        <v>46324.63946440972</v>
+        <v>46324.49347768519</v>
       </c>
       <c r="S316">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T316" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="U316" t="s">
         <v>264</v>
@@ -25261,25 +25291,28 @@
       <c r="V316" t="s">
         <v>267</v>
       </c>
+      <c r="W316" t="s">
+        <v>380</v>
+      </c>
       <c r="AA316">
         <v>0</v>
       </c>
       <c r="AB316" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AG316" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="AH316" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
     </row>
     <row r="317" spans="1:34">
       <c r="A317">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B317" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C317" t="s">
         <v>55</v>
@@ -25303,7 +25336,7 @@
         <v>63</v>
       </c>
       <c r="J317" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L317" s="1">
         <v>46321</v>
@@ -25315,43 +25348,40 @@
         <v>213</v>
       </c>
       <c r="O317">
-        <v>17042663</v>
+        <v>18178315</v>
       </c>
       <c r="P317" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Q317" t="s">
         <v>248</v>
       </c>
       <c r="R317" s="1">
-        <v>46324.49347768519</v>
+        <v>46325.45940759259</v>
       </c>
       <c r="S317">
         <v>4</v>
       </c>
       <c r="T317" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="U317" t="s">
-        <v>264</v>
-      </c>
-      <c r="V317" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="W317" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="AA317">
         <v>0</v>
       </c>
       <c r="AB317" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG317" t="s">
         <v>533</v>
       </c>
       <c r="AH317" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="318" spans="1:34">
@@ -25383,7 +25413,7 @@
         <v>63</v>
       </c>
       <c r="J318" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L318" s="1">
         <v>46321</v>
@@ -25460,7 +25490,7 @@
         <v>63</v>
       </c>
       <c r="J319" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L319" s="1">
         <v>46321</v>
@@ -25537,7 +25567,7 @@
         <v>63</v>
       </c>
       <c r="J320" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L320" s="1">
         <v>46325</v>
@@ -25614,7 +25644,7 @@
         <v>63</v>
       </c>
       <c r="J321" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L321" s="1">
         <v>46325</v>
@@ -25691,7 +25721,7 @@
         <v>63</v>
       </c>
       <c r="J322" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L322" s="1">
         <v>46325</v>
@@ -25771,7 +25801,7 @@
         <v>63</v>
       </c>
       <c r="J323" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L323" s="1">
         <v>46325</v>
@@ -25851,7 +25881,7 @@
         <v>63</v>
       </c>
       <c r="J324" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L324" s="1">
         <v>46325</v>
@@ -25928,7 +25958,7 @@
         <v>63</v>
       </c>
       <c r="J325" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L325" s="1">
         <v>46325</v>
@@ -26005,7 +26035,7 @@
         <v>63</v>
       </c>
       <c r="J326" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L326" s="1">
         <v>46325</v>
@@ -26082,7 +26112,7 @@
         <v>63</v>
       </c>
       <c r="J327" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L327" s="1">
         <v>46325</v>
@@ -26162,7 +26192,7 @@
         <v>63</v>
       </c>
       <c r="J328" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L328" s="1">
         <v>46325</v>
@@ -26609,7 +26639,7 @@
         <v>64</v>
       </c>
       <c r="J334" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L334" s="1">
         <v>46321</v>
@@ -26680,7 +26710,7 @@
         <v>64</v>
       </c>
       <c r="J335" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L335" s="1">
         <v>46321</v>
@@ -26751,7 +26781,7 @@
         <v>64</v>
       </c>
       <c r="J336" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L336" s="1">
         <v>46321</v>
@@ -26825,7 +26855,7 @@
         <v>64</v>
       </c>
       <c r="J337" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L337" s="1">
         <v>46321</v>
@@ -26896,7 +26926,7 @@
         <v>64</v>
       </c>
       <c r="J338" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L338" s="1">
         <v>46321</v>
@@ -26973,7 +27003,7 @@
         <v>64</v>
       </c>
       <c r="J339" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L339" s="1">
         <v>46321</v>
@@ -27044,7 +27074,7 @@
         <v>64</v>
       </c>
       <c r="J340" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L340" s="1">
         <v>46321</v>
@@ -27115,7 +27145,7 @@
         <v>64</v>
       </c>
       <c r="J341" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L341" s="1">
         <v>46321</v>
@@ -27195,7 +27225,7 @@
         <v>64</v>
       </c>
       <c r="J342" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L342" s="1">
         <v>46321</v>
@@ -27266,7 +27296,7 @@
         <v>64</v>
       </c>
       <c r="J343" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="L343" s="1">
         <v>46321</v>
@@ -27482,7 +27512,7 @@
         <v>64</v>
       </c>
       <c r="J346" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L346" s="1">
         <v>46324</v>
@@ -27553,7 +27583,7 @@
         <v>64</v>
       </c>
       <c r="J347" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L347" s="1">
         <v>46324</v>
@@ -27624,7 +27654,7 @@
         <v>64</v>
       </c>
       <c r="J348" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L348" s="1">
         <v>46324</v>
@@ -27840,7 +27870,7 @@
         <v>64</v>
       </c>
       <c r="J351" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L351" s="1">
         <v>46321</v>
@@ -27911,7 +27941,7 @@
         <v>64</v>
       </c>
       <c r="J352" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L352" s="1">
         <v>46321</v>
@@ -27988,7 +28018,7 @@
         <v>64</v>
       </c>
       <c r="J353" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L353" s="1">
         <v>46321</v>
@@ -28059,7 +28089,7 @@
         <v>64</v>
       </c>
       <c r="J354" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L354" s="1">
         <v>46321</v>
@@ -28130,7 +28160,7 @@
         <v>64</v>
       </c>
       <c r="J355" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="L355" s="1">
         <v>46321</v>
@@ -28210,7 +28240,7 @@
         <v>64</v>
       </c>
       <c r="J356" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L356" s="1">
         <v>46325</v>
@@ -28287,7 +28317,7 @@
         <v>64</v>
       </c>
       <c r="J357" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L357" s="1">
         <v>46325</v>
@@ -28361,7 +28391,7 @@
         <v>64</v>
       </c>
       <c r="J358" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L358" s="1">
         <v>46325</v>
@@ -28438,7 +28468,7 @@
         <v>64</v>
       </c>
       <c r="J359" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L359" s="1">
         <v>46325</v>
@@ -28515,7 +28545,7 @@
         <v>64</v>
       </c>
       <c r="J360" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L360" s="1">
         <v>46325</v>
@@ -36443,7 +36473,7 @@
         <v>65</v>
       </c>
       <c r="J466" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L466" s="1">
         <v>46311</v>
@@ -36517,7 +36547,7 @@
         <v>65</v>
       </c>
       <c r="J467" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L467" s="1">
         <v>46311</v>
@@ -36745,7 +36775,7 @@
         <v>65</v>
       </c>
       <c r="J470" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L470" s="1">
         <v>46322</v>
@@ -36822,7 +36852,7 @@
         <v>65</v>
       </c>
       <c r="J471" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L471" s="1">
         <v>46322</v>
@@ -39096,7 +39126,7 @@
         <v>66</v>
       </c>
       <c r="J501" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L501" s="1">
         <v>46322</v>
@@ -39173,7 +39203,7 @@
         <v>66</v>
       </c>
       <c r="J502" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L502" s="1">
         <v>46322</v>
@@ -40561,7 +40591,7 @@
         <v>67</v>
       </c>
       <c r="J521" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L521" s="1">
         <v>46325</v>
@@ -46015,7 +46045,7 @@
         <v>68</v>
       </c>
       <c r="J599" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L599" s="1">
         <v>46321</v>
@@ -47151,7 +47181,7 @@
         <v>63</v>
       </c>
       <c r="J615" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L615" s="1">
         <v>46321</v>
@@ -47219,7 +47249,7 @@
         <v>64</v>
       </c>
       <c r="J616" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L616" s="1">
         <v>46324</v>
@@ -47355,7 +47385,7 @@
         <v>68</v>
       </c>
       <c r="J618" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L618" s="1">
         <v>46321</v>
@@ -47420,7 +47450,7 @@
         <v>64</v>
       </c>
       <c r="J619" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L619" s="1">
         <v>46325</v>
@@ -47692,7 +47722,7 @@
         <v>68</v>
       </c>
       <c r="J623" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L623" s="1">
         <v>46325</v>
@@ -47751,7 +47781,7 @@
         <v>68</v>
       </c>
       <c r="J624" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L624" s="1">
         <v>46325</v>

</xml_diff>